<commit_message>
Re-add N/A for Seton only where absence is confirmed (Corflute items)
The 13 Corflute multi-message RSEA line items get N/A back, since the
research confirmed Seton sells that roadwork-sign range only as a
configurable build-your-own system, not as fixed priced products -
a structural confirmation, not just an unsuccessful cache search.
Every other blank Seton cell stays blank, since those are genuinely
unconfirmed (cache-search limitations, ambiguous pricing, or a size
mismatch on a product that does exist) rather than confirmed absences.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="310">
   <si>
     <t xml:space="preserve">RSEA Code</t>
   </si>
@@ -1546,9 +1546,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>406800</xdr:colOff>
+      <xdr:colOff>406440</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>263160</xdr:rowOff>
+      <xdr:rowOff>262800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1562,7 +1562,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2194560" cy="2340720"/>
+          <a:ext cx="2194200" cy="2340360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9976,8 +9976,12 @@
       <c r="Y30" s="42" t="s">
         <v>257</v>
       </c>
-      <c r="Z30" s="42"/>
-      <c r="AA30" s="42"/>
+      <c r="Z30" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA30" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB30" s="11" t="n">
         <f aca="false">IF(COUNT(I30,K30,M30,O30,Q30,S30,U30,W30,Y30,AA30)=0,"N/A",MIN(I30,K30,M30,O30,Q30,S30,U30,W30,Y30,AA30))</f>
         <v>28</v>
@@ -10079,8 +10083,12 @@
         <f aca="false">X31/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z31" s="42"/>
-      <c r="AA31" s="42"/>
+      <c r="Z31" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA31" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB31" s="11" t="n">
         <f aca="false">IF(COUNT(I31,K31,M31,O31,Q31,S31,U31,W31,Y31,AA31)=0,"N/A",MIN(I31,K31,M31,O31,Q31,S31,U31,W31,Y31,AA31))</f>
         <v>31</v>
@@ -10183,8 +10191,12 @@
       <c r="Y32" s="42" t="s">
         <v>257</v>
       </c>
-      <c r="Z32" s="42"/>
-      <c r="AA32" s="42"/>
+      <c r="Z32" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA32" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB32" s="11" t="n">
         <f aca="false">IF(COUNT(I32,K32,M32,O32,Q32,S32,U32,W32,Y32,AA32)=0,"N/A",MIN(I32,K32,M32,O32,Q32,S32,U32,W32,Y32,AA32))</f>
         <v>31</v>
@@ -10287,8 +10299,12 @@
         <f aca="false">X33/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z33" s="42"/>
-      <c r="AA33" s="42"/>
+      <c r="Z33" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA33" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB33" s="11" t="n">
         <f aca="false">IF(COUNT(I33,K33,M33,O33,Q33,S33,U33,W33,Y33,AA33)=0,"N/A",MIN(I33,K33,M33,O33,Q33,S33,U33,W33,Y33,AA33))</f>
         <v>31</v>
@@ -10392,8 +10408,12 @@
         <f aca="false">X34/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z34" s="42"/>
-      <c r="AA34" s="42"/>
+      <c r="Z34" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA34" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB34" s="11" t="n">
         <f aca="false">IF(COUNT(I34,K34,M34,O34,Q34,S34,U34,W34,Y34,AA34)=0,"N/A",MIN(I34,K34,M34,O34,Q34,S34,U34,W34,Y34,AA34))</f>
         <v>31</v>
@@ -10497,8 +10517,12 @@
         <f aca="false">X35/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z35" s="42"/>
-      <c r="AA35" s="42"/>
+      <c r="Z35" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA35" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB35" s="11" t="n">
         <f aca="false">IF(COUNT(I35,K35,M35,O35,Q35,S35,U35,W35,Y35,AA35)=0,"N/A",MIN(I35,K35,M35,O35,Q35,S35,U35,W35,Y35,AA35))</f>
         <v>31</v>
@@ -10603,8 +10627,12 @@
         <f aca="false">X36/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z36" s="42"/>
-      <c r="AA36" s="42"/>
+      <c r="Z36" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA36" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB36" s="11" t="n">
         <f aca="false">IF(COUNT(I36,K36,M36,O36,Q36,S36,U36,W36,Y36,AA36)=0,"N/A",MIN(I36,K36,M36,O36,Q36,S36,U36,W36,Y36,AA36))</f>
         <v>31</v>
@@ -10706,8 +10734,12 @@
       <c r="Y37" s="42" t="s">
         <v>257</v>
       </c>
-      <c r="Z37" s="42"/>
-      <c r="AA37" s="42"/>
+      <c r="Z37" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA37" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB37" s="11" t="n">
         <f aca="false">IF(COUNT(I37,K37,M37,O37,Q37,S37,U37,W37,Y37,AA37)=0,"N/A",MIN(I37,K37,M37,O37,Q37,S37,U37,W37,Y37,AA37))</f>
         <v>31</v>
@@ -10810,8 +10842,12 @@
         <f aca="false">X38/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z38" s="42"/>
-      <c r="AA38" s="42"/>
+      <c r="Z38" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA38" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB38" s="11" t="n">
         <f aca="false">IF(COUNT(I38,K38,M38,O38,Q38,S38,U38,W38,Y38,AA38)=0,"N/A",MIN(I38,K38,M38,O38,Q38,S38,U38,W38,Y38,AA38))</f>
         <v>31</v>
@@ -10915,8 +10951,12 @@
         <f aca="false">X39/1.1</f>
         <v>112.918181818182</v>
       </c>
-      <c r="Z39" s="42"/>
-      <c r="AA39" s="42"/>
+      <c r="Z39" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA39" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB39" s="11" t="n">
         <f aca="false">IF(COUNT(I39,K39,M39,O39,Q39,S39,U39,W39,Y39,AA39)=0,"N/A",MIN(I39,K39,M39,O39,Q39,S39,U39,W39,Y39,AA39))</f>
         <v>31</v>
@@ -11020,8 +11060,12 @@
         <f aca="false">X40/1.1</f>
         <v>112.918181818182</v>
       </c>
-      <c r="Z40" s="42"/>
-      <c r="AA40" s="42"/>
+      <c r="Z40" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA40" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB40" s="11" t="n">
         <f aca="false">IF(COUNT(I40,K40,M40,O40,Q40,S40,U40,W40,Y40,AA40)=0,"N/A",MIN(I40,K40,M40,O40,Q40,S40,U40,W40,Y40,AA40))</f>
         <v>31</v>
@@ -11125,8 +11169,12 @@
         <f aca="false">X41/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z41" s="42"/>
-      <c r="AA41" s="42"/>
+      <c r="Z41" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA41" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB41" s="11" t="n">
         <f aca="false">IF(COUNT(I41,K41,M41,O41,Q41,S41,U41,W41,Y41,AA41)=0,"N/A",MIN(I41,K41,M41,O41,Q41,S41,U41,W41,Y41,AA41))</f>
         <v>31</v>
@@ -11230,8 +11278,12 @@
         <f aca="false">X42/1.1</f>
         <v>48.3818181818182</v>
       </c>
-      <c r="Z42" s="42"/>
-      <c r="AA42" s="42"/>
+      <c r="Z42" s="42" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA42" s="42" t="s">
+        <v>257</v>
+      </c>
       <c r="AB42" s="11" t="n">
         <f aca="false">IF(COUNT(I42,K42,M42,O42,Q42,S42,U42,W42,Y42,AA42)=0,"N/A",MIN(I42,K42,M42,O42,Q42,S42,U42,W42,Y42,AA42))</f>
         <v>31</v>

</xml_diff>

<commit_message>
Add Summary tab: closest-priced competitor and where we're more expensive
Carries forward Jonathan's latest manual edits (simplified Seton column
headers). New "Summary" tab has two parts:

1. All 60 items, each showing which competitor (or RSEA) is CLOSEST to
   our 1200-stock quoted price (ex GST, can be above or below), with the
   $ and % gap and a flag for whether that competitor is cheaper than us.
2. A call-out list of the 7 items where we're more expensive than the
   single cheapest alternative in the market, with who undercuts us and
   by how much, sorted worst-overpriced first.

"Closest" and "cheapest" are deliberately different questions - closest
tells you who's most directly comparable, cheapest tells you who to
worry about. Recalculates clean with zero formula errors.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -15,6 +15,7 @@
     <sheet name="POLY ON WEBSITE" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="RSEA vs Quoted Comparison" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Market Comparison" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Summary" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1715" uniqueCount="337">
   <si>
     <t xml:space="preserve">RSEA Code</t>
   </si>
@@ -806,11 +807,11 @@
   </si>
   <si>
     <t xml:space="preserve">Seton
-(inc GST, as shown)</t>
+(inc GST)</t>
   </si>
   <si>
     <t xml:space="preserve">Seton
-(ex GST, calc.)</t>
+(ex GST)</t>
   </si>
   <si>
     <t xml:space="preserve">Cheapest of RSEA +
@@ -956,6 +957,9 @@
     <t xml:space="preserve">Jaybro: 150x150, size differs from 225x225 | All Trades Group: 150x225, size differs | eSafety Supplies: 300x450, closest, '600x450 also stocked' | Safety Signs Australia: 225x225 poly EXACT, double-sided | SafetyXpress: range 21.11-23.12, 225x300 size differs slightly | Traffic Control Products: Only physical extinguisher unit stocked, not a wall sign | National Safety Signs: From, F1411, 225x225 not confirmed | Seton: MEDIUM conf, 225x225 poly EXACT, inc GST (55.75 ex)</t>
   </si>
   <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
     <t xml:space="preserve">All Trades Group: 900x600 corflute, size differs (larger) | Safety Signs Australia: 450x600 poly EXACT | SafetyXpress: 450x600 metal EXACT size, material differs | Traffic Control Products: 600x450, 'Danger Crane Working Overhead' - different wording, poly | National Safety Signs: From, D10279 | Seton: LOW conf, bulk tier range 33.21-36.91, 600x450 Flute</t>
   </si>
   <si>
@@ -987,13 +991,97 @@
   </si>
   <si>
     <t xml:space="preserve">Median of (our 1220-Stock quote ÷ cheapest − 1), ex GST — negative means our quote is cheaper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary — Closest-Priced Competitor &amp; Where We're More Expensive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each of our 60 line items: the competitor (or RSEA) whose ex-GST price is CLOSEST to our current quoted price (1200-stock, ex GST) — this can be either above or below ours — and the $ / % gap to that closest price. This is a different question from "cheapest": closest tells you who's most directly comparable to us in the market; cheapest (separately reported, see 'Items we're MORE EXPENSIVE on' below) tells you who undercuts us the most. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Our Quoted Price
+(ex GST, 1200 Stock)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest-Priced
+Competitor (or RSEA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Their Price
+(ex GST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ Difference
+(Them − Us)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Difference
+(vs Our Price)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are We More
+Expensive?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eSafety Supplies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic Control Products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HiVis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Trades Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SafetyXpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaybro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Safety Signs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety Signs Australia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Items We're MORE EXPENSIVE On (our 1200-Stock quote vs the single cheapest alternative — 7 of 60 items)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheapest Alternative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Their Price (ex GST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Our Price (ex GST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ We're More Expensive By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% We're More Expensive By</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00_);[RED]&quot;($&quot;#,##0.00\)"/>
@@ -1001,8 +1089,9 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="\$#,##0.00_);[RED]&quot;($&quot;#,##0.00\)"/>
+    <numFmt numFmtId="171" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1111,6 +1200,52 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF17365D"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1B7A4D"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF17365D"/>
+      <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1225,7 +1360,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1414,6 +1549,50 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1452,7 +1631,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1463,7 +1642,7 @@
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF1B7A4D"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
@@ -12690,7 +12869,7 @@
         <v>257</v>
       </c>
       <c r="AA55" s="41" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="AB55" s="10" t="n">
         <f aca="false">IF(COUNT(I55,K55,M55,O55,Q55,S55,U55,W55,Y55,AA55)=0,"N/A",MIN(I55,K55,M55,O55,Q55,S55,U55,W55,Y55,AA55))</f>
@@ -13759,7 +13938,7 @@
         <v>N/A</v>
       </c>
       <c r="AE65" s="40" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13769,7 +13948,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="34" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B68" s="34"/>
       <c r="C68" s="34"/>
@@ -13780,7 +13959,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="34" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B69" s="34"/>
       <c r="C69" s="34"/>
@@ -13791,7 +13970,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="34" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B70" s="34"/>
       <c r="C70" s="34"/>
@@ -13802,7 +13981,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="34" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B71" s="34"/>
       <c r="C71" s="34"/>
@@ -13813,7 +13992,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="34" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B72" s="34"/>
       <c r="C72" s="34"/>
@@ -13824,7 +14003,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="34" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B73" s="34"/>
       <c r="C73" s="34"/>
@@ -13835,7 +14014,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="34" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B74" s="34"/>
       <c r="C74" s="34"/>
@@ -13846,7 +14025,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="34" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B75" s="34"/>
       <c r="C75" s="34"/>
@@ -13857,7 +14036,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="34" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B76" s="34"/>
       <c r="C76" s="34"/>
@@ -13868,7 +14047,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="34" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B77" s="34"/>
       <c r="C77" s="34"/>
@@ -13901,4 +14080,2157 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J74"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="47" t="s">
+        <v>311</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+    </row>
+    <row r="2" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="48" t="s">
+        <v>312</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+    </row>
+    <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="49" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>314</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>315</v>
+      </c>
+      <c r="G4" s="49" t="s">
+        <v>316</v>
+      </c>
+      <c r="H4" s="49" t="s">
+        <v>317</v>
+      </c>
+      <c r="I4" s="49" t="s">
+        <v>318</v>
+      </c>
+      <c r="J4" s="49" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="51" t="n">
+        <f aca="false">'Market Comparison'!D6</f>
+        <v>16.71</v>
+      </c>
+      <c r="E5" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="F5" s="51" t="n">
+        <v>20.05</v>
+      </c>
+      <c r="G5" s="52" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="H5" s="53" t="n">
+        <v>0.199880311190904</v>
+      </c>
+      <c r="I5" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J5" s="40"/>
+    </row>
+    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B6" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <f aca="false">'Market Comparison'!D7</f>
+        <v>66.83</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F6" s="51" t="n">
+        <v>122.718181818182</v>
+      </c>
+      <c r="G6" s="52" t="n">
+        <v>55.8881818181818</v>
+      </c>
+      <c r="H6" s="53" t="n">
+        <v>0.836273856324732</v>
+      </c>
+      <c r="I6" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J6" s="40"/>
+    </row>
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B7" s="50" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <f aca="false">'Market Comparison'!D8</f>
+        <v>44.55</v>
+      </c>
+      <c r="E7" s="50" t="s">
+        <v>322</v>
+      </c>
+      <c r="F7" s="51" t="n">
+        <v>128.75</v>
+      </c>
+      <c r="G7" s="52" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="H7" s="53" t="n">
+        <v>1.89001122334456</v>
+      </c>
+      <c r="I7" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J7" s="40"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <f aca="false">'Market Comparison'!D9</f>
+        <v>44.55</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>323</v>
+      </c>
+      <c r="F8" s="51" t="n">
+        <v>69.245</v>
+      </c>
+      <c r="G8" s="52" t="n">
+        <v>24.695</v>
+      </c>
+      <c r="H8" s="53" t="n">
+        <v>0.554320987654321</v>
+      </c>
+      <c r="I8" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J8" s="40"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <f aca="false">'Market Comparison'!D10</f>
+        <v>69.61</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>323</v>
+      </c>
+      <c r="F9" s="51" t="n">
+        <v>81.4</v>
+      </c>
+      <c r="G9" s="52" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="H9" s="53" t="n">
+        <v>0.169372216635541</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J9" s="40"/>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <f aca="false">'Market Comparison'!D11</f>
+        <v>33.41</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>324</v>
+      </c>
+      <c r="F10" s="51" t="n">
+        <v>44.209</v>
+      </c>
+      <c r="G10" s="52" t="n">
+        <v>10.799</v>
+      </c>
+      <c r="H10" s="53" t="n">
+        <v>0.323226578868603</v>
+      </c>
+      <c r="I10" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J10" s="40"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B11" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <f aca="false">'Market Comparison'!D12</f>
+        <v>44.55</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="F11" s="51" t="n">
+        <v>70.36</v>
+      </c>
+      <c r="G11" s="52" t="n">
+        <v>25.81</v>
+      </c>
+      <c r="H11" s="53" t="n">
+        <v>0.579349046015713</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J11" s="40"/>
+    </row>
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <f aca="false">'Market Comparison'!D13</f>
+        <v>33.41</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="F12" s="51" t="n">
+        <v>33.1818181818182</v>
+      </c>
+      <c r="G12" s="54" t="n">
+        <v>-0.228181818181817</v>
+      </c>
+      <c r="H12" s="55" t="n">
+        <v>-0.00682974612935698</v>
+      </c>
+      <c r="I12" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J12" s="40"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B13" s="50" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="40" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <f aca="false">'Market Comparison'!D14</f>
+        <v>25.06</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="F13" s="51" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="G13" s="52" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="H13" s="53" t="n">
+        <v>0.719473264166002</v>
+      </c>
+      <c r="I13" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J13" s="40"/>
+    </row>
+    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <f aca="false">'Market Comparison'!D15</f>
+        <v>8.35</v>
+      </c>
+      <c r="E14" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F14" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G14" s="52" t="n">
+        <v>21.6409090909091</v>
+      </c>
+      <c r="H14" s="53" t="n">
+        <v>2.59172563962983</v>
+      </c>
+      <c r="I14" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J14" s="40"/>
+    </row>
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B15" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <f aca="false">'Market Comparison'!D16</f>
+        <v>15.59</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F15" s="51" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G15" s="52" t="n">
+        <v>25.31</v>
+      </c>
+      <c r="H15" s="53" t="n">
+        <v>1.62347658755613</v>
+      </c>
+      <c r="I15" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J15" s="40"/>
+    </row>
+    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B16" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <f aca="false">'Market Comparison'!D17</f>
+        <v>8.35</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F16" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G16" s="52" t="n">
+        <v>21.6409090909091</v>
+      </c>
+      <c r="H16" s="53" t="n">
+        <v>2.59172563962983</v>
+      </c>
+      <c r="I16" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J16" s="40"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B17" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <f aca="false">'Market Comparison'!D18</f>
+        <v>29.7</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="F17" s="51" t="n">
+        <v>37.3909090909091</v>
+      </c>
+      <c r="G17" s="52" t="n">
+        <v>7.69090909090909</v>
+      </c>
+      <c r="H17" s="53" t="n">
+        <v>0.258953168044077</v>
+      </c>
+      <c r="I17" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J17" s="40"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B18" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <f aca="false">'Market Comparison'!D19</f>
+        <v>29.7</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="F18" s="51" t="n">
+        <v>28.3545454545455</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <v>-1.34545454545455</v>
+      </c>
+      <c r="H18" s="55" t="n">
+        <v>-0.0453014998469545</v>
+      </c>
+      <c r="I18" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J18" s="40"/>
+    </row>
+    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B19" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <f aca="false">'Market Comparison'!D20</f>
+        <v>16.71</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="F19" s="51" t="n">
+        <v>23.3090909090909</v>
+      </c>
+      <c r="G19" s="52" t="n">
+        <v>6.59909090909091</v>
+      </c>
+      <c r="H19" s="53" t="n">
+        <v>0.394918666013819</v>
+      </c>
+      <c r="I19" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J19" s="40"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B20" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <f aca="false">'Market Comparison'!D21</f>
+        <v>33.41</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>328</v>
+      </c>
+      <c r="F20" s="51" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="G20" s="54" t="n">
+        <v>-4.42</v>
+      </c>
+      <c r="H20" s="55" t="n">
+        <v>-0.132295719844358</v>
+      </c>
+      <c r="I20" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J20" s="40"/>
+    </row>
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B21" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <f aca="false">'Market Comparison'!D22</f>
+        <v>11.81</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F21" s="51" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G21" s="52" t="n">
+        <v>9.39</v>
+      </c>
+      <c r="H21" s="53" t="n">
+        <v>0.795088907705334</v>
+      </c>
+      <c r="I21" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J21" s="40"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B22" s="50" t="s">
+        <v>151</v>
+      </c>
+      <c r="C22" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <f aca="false">'Market Comparison'!D23</f>
+        <v>11.81</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F22" s="51" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G22" s="52" t="n">
+        <v>9.39</v>
+      </c>
+      <c r="H22" s="53" t="n">
+        <v>0.795088907705334</v>
+      </c>
+      <c r="I22" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J22" s="40"/>
+    </row>
+    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B23" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" s="51" t="n">
+        <f aca="false">'Market Comparison'!D24</f>
+        <v>5.9</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F23" s="51" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="G23" s="52" t="n">
+        <v>28.6363636363636</v>
+      </c>
+      <c r="H23" s="53" t="n">
+        <v>4.85362095531587</v>
+      </c>
+      <c r="I23" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J23" s="40"/>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B24" s="50" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <f aca="false">'Market Comparison'!D25</f>
+        <v>11.81</v>
+      </c>
+      <c r="E24" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F24" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="G24" s="54" t="n">
+        <v>-2.45545454545455</v>
+      </c>
+      <c r="H24" s="55" t="n">
+        <v>-0.207913170656609</v>
+      </c>
+      <c r="I24" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J24" s="40"/>
+    </row>
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B25" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <f aca="false">'Market Comparison'!D26</f>
+        <v>11.81</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="G25" s="54" t="n">
+        <v>-2.45545454545455</v>
+      </c>
+      <c r="H25" s="55" t="n">
+        <v>-0.207913170656609</v>
+      </c>
+      <c r="I25" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J25" s="40"/>
+    </row>
+    <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B26" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="C26" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="D26" s="51" t="n">
+        <f aca="false">'Market Comparison'!D27</f>
+        <v>11.81</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F26" s="51" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G26" s="52" t="n">
+        <v>9.39</v>
+      </c>
+      <c r="H26" s="53" t="n">
+        <v>0.795088907705334</v>
+      </c>
+      <c r="I26" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J26" s="40"/>
+    </row>
+    <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="50" t="s">
+        <v>167</v>
+      </c>
+      <c r="C27" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="D27" s="51" t="n">
+        <f aca="false">'Market Comparison'!D28</f>
+        <v>33.41</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="F27" s="51" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="G27" s="54" t="n">
+        <v>-0.909999999999997</v>
+      </c>
+      <c r="H27" s="55" t="n">
+        <v>-0.027237354085603</v>
+      </c>
+      <c r="I27" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="J27" s="40"/>
+    </row>
+    <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="B28" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>175</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <f aca="false">'Market Comparison'!D29</f>
+        <v>33.41</v>
+      </c>
+      <c r="E28" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="F28" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="G28" s="52" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="H28" s="53" t="n">
+        <v>0.346902125112242</v>
+      </c>
+      <c r="I28" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J28" s="40"/>
+    </row>
+    <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B29" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <f aca="false">'Market Comparison'!D30</f>
+        <v>13.07</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>323</v>
+      </c>
+      <c r="F29" s="51" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="G29" s="52" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="H29" s="53" t="n">
+        <v>1.35654169854629</v>
+      </c>
+      <c r="I29" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J29" s="40"/>
+    </row>
+    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <f aca="false">'Market Comparison'!D31</f>
+        <v>13.07</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F30" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G30" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H30" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I30" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J30" s="40"/>
+    </row>
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B31" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <f aca="false">'Market Comparison'!D32</f>
+        <v>16.04</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F31" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G31" s="52" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="H31" s="53" t="n">
+        <v>0.932668329177057</v>
+      </c>
+      <c r="I31" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J31" s="40"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <f aca="false">'Market Comparison'!D33</f>
+        <v>16.04</v>
+      </c>
+      <c r="E32" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F32" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G32" s="52" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="H32" s="53" t="n">
+        <v>0.932668329177057</v>
+      </c>
+      <c r="I32" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J32" s="40"/>
+    </row>
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B33" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="D33" s="51" t="n">
+        <f aca="false">'Market Comparison'!D34</f>
+        <v>16.04</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F33" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G33" s="52" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="H33" s="53" t="n">
+        <v>0.932668329177057</v>
+      </c>
+      <c r="I33" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J33" s="40"/>
+    </row>
+    <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B34" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="51" t="n">
+        <f aca="false">'Market Comparison'!D35</f>
+        <v>16.04</v>
+      </c>
+      <c r="E34" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F34" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G34" s="52" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="H34" s="53" t="n">
+        <v>0.932668329177057</v>
+      </c>
+      <c r="I34" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J34" s="40"/>
+    </row>
+    <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B35" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <f aca="false">'Market Comparison'!D36</f>
+        <v>13.07</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F35" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G35" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H35" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I35" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J35" s="40"/>
+    </row>
+    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B36" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="51" t="n">
+        <f aca="false">'Market Comparison'!D37</f>
+        <v>16.04</v>
+      </c>
+      <c r="E36" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F36" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G36" s="52" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="H36" s="53" t="n">
+        <v>0.932668329177057</v>
+      </c>
+      <c r="I36" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J36" s="40"/>
+    </row>
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B37" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" s="51" t="n">
+        <f aca="false">'Market Comparison'!D38</f>
+        <v>13.07</v>
+      </c>
+      <c r="E37" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F37" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G37" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H37" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I37" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J37" s="40"/>
+    </row>
+    <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B38" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <f aca="false">'Market Comparison'!D39</f>
+        <v>13.07</v>
+      </c>
+      <c r="E38" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F38" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G38" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H38" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I38" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J38" s="40"/>
+    </row>
+    <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B39" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="D39" s="51" t="n">
+        <f aca="false">'Market Comparison'!D40</f>
+        <v>13.07</v>
+      </c>
+      <c r="E39" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F39" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G39" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H39" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I39" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J39" s="40"/>
+    </row>
+    <row r="40" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B40" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <f aca="false">'Market Comparison'!D41</f>
+        <v>13.07</v>
+      </c>
+      <c r="E40" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F40" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G40" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H40" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I40" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J40" s="40"/>
+    </row>
+    <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" s="51" t="n">
+        <f aca="false">'Market Comparison'!D42</f>
+        <v>13.07</v>
+      </c>
+      <c r="E41" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F41" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G41" s="52" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="H41" s="53" t="n">
+        <v>1.37184391736802</v>
+      </c>
+      <c r="I41" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J41" s="40"/>
+    </row>
+    <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B42" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="40" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="51" t="n">
+        <f aca="false">'Market Comparison'!D43</f>
+        <v>5.35</v>
+      </c>
+      <c r="E42" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F42" s="51" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="G42" s="52" t="n">
+        <v>29.1863636363636</v>
+      </c>
+      <c r="H42" s="53" t="n">
+        <v>5.4553950722175</v>
+      </c>
+      <c r="I42" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J42" s="40"/>
+    </row>
+    <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B43" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C43" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="51" t="n">
+        <f aca="false">'Market Comparison'!D44</f>
+        <v>2.67</v>
+      </c>
+      <c r="E43" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F43" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="G43" s="52" t="n">
+        <v>6.68454545454545</v>
+      </c>
+      <c r="H43" s="53" t="n">
+        <v>2.50357507660878</v>
+      </c>
+      <c r="I43" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J43" s="40"/>
+    </row>
+    <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B44" s="50" t="s">
+        <v>97</v>
+      </c>
+      <c r="C44" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" s="51" t="n">
+        <f aca="false">'Market Comparison'!D45</f>
+        <v>10.69</v>
+      </c>
+      <c r="E44" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F44" s="51" t="n">
+        <v>23.4090909090909</v>
+      </c>
+      <c r="G44" s="52" t="n">
+        <v>12.7190909090909</v>
+      </c>
+      <c r="H44" s="53" t="n">
+        <v>1.18981205884854</v>
+      </c>
+      <c r="I44" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J44" s="40"/>
+    </row>
+    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B45" s="50" t="s">
+        <v>99</v>
+      </c>
+      <c r="C45" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" s="51" t="n">
+        <f aca="false">'Market Comparison'!D46</f>
+        <v>2.67</v>
+      </c>
+      <c r="E45" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F45" s="51" t="n">
+        <v>22.7181818181818</v>
+      </c>
+      <c r="G45" s="52" t="n">
+        <v>20.0481818181818</v>
+      </c>
+      <c r="H45" s="53" t="n">
+        <v>7.50868232890705</v>
+      </c>
+      <c r="I45" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J45" s="40"/>
+    </row>
+    <row r="46" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B46" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" s="51" t="n">
+        <f aca="false">'Market Comparison'!D47</f>
+        <v>9.5</v>
+      </c>
+      <c r="E46" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F46" s="51" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G46" s="52" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H46" s="53" t="n">
+        <v>3.30526315789474</v>
+      </c>
+      <c r="I46" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J46" s="40"/>
+    </row>
+    <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B47" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="D47" s="51" t="n">
+        <f aca="false">'Market Comparison'!D48</f>
+        <v>10.69</v>
+      </c>
+      <c r="E47" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F47" s="51" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G47" s="52" t="n">
+        <v>30.21</v>
+      </c>
+      <c r="H47" s="53" t="n">
+        <v>2.82600561272217</v>
+      </c>
+      <c r="I47" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J47" s="40"/>
+    </row>
+    <row r="48" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B48" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="C48" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" s="51" t="n">
+        <f aca="false">'Market Comparison'!D49</f>
+        <v>5.35</v>
+      </c>
+      <c r="E48" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F48" s="51" t="n">
+        <v>20.9090909090909</v>
+      </c>
+      <c r="G48" s="52" t="n">
+        <v>15.5590909090909</v>
+      </c>
+      <c r="H48" s="53" t="n">
+        <v>2.90824129141886</v>
+      </c>
+      <c r="I48" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J48" s="40"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B49" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="C49" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="D49" s="51" t="n">
+        <f aca="false">'Market Comparison'!D50</f>
+        <v>5.35</v>
+      </c>
+      <c r="E49" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="F49" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="G49" s="52" t="n">
+        <v>4.00454545454545</v>
+      </c>
+      <c r="H49" s="53" t="n">
+        <v>0.748513169073917</v>
+      </c>
+      <c r="I49" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J49" s="40"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B50" s="50" t="s">
+        <v>115</v>
+      </c>
+      <c r="C50" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="D50" s="51" t="n">
+        <f aca="false">'Market Comparison'!D51</f>
+        <v>2.67</v>
+      </c>
+      <c r="E50" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F50" s="51" t="n">
+        <v>25.4454545454545</v>
+      </c>
+      <c r="G50" s="52" t="n">
+        <v>22.7754545454545</v>
+      </c>
+      <c r="H50" s="53" t="n">
+        <v>8.53013278855975</v>
+      </c>
+      <c r="I50" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J50" s="40"/>
+    </row>
+    <row r="51" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B51" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="D51" s="51" t="n">
+        <f aca="false">'Market Comparison'!D52</f>
+        <v>9.5</v>
+      </c>
+      <c r="E51" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F51" s="51" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G51" s="52" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H51" s="53" t="n">
+        <v>3.30526315789474</v>
+      </c>
+      <c r="I51" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J51" s="40"/>
+    </row>
+    <row r="52" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B52" s="50" t="s">
+        <v>121</v>
+      </c>
+      <c r="C52" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" s="51" t="n">
+        <f aca="false">'Market Comparison'!D53</f>
+        <v>2</v>
+      </c>
+      <c r="E52" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="F52" s="51" t="n">
+        <v>7.81818181818182</v>
+      </c>
+      <c r="G52" s="52" t="n">
+        <v>5.81818181818182</v>
+      </c>
+      <c r="H52" s="53" t="n">
+        <v>2.90909090909091</v>
+      </c>
+      <c r="I52" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J52" s="40"/>
+    </row>
+    <row r="53" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B53" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53" s="51" t="n">
+        <f aca="false">'Market Comparison'!D54</f>
+        <v>2.67</v>
+      </c>
+      <c r="E53" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F53" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G53" s="52" t="n">
+        <v>27.3209090909091</v>
+      </c>
+      <c r="H53" s="53" t="n">
+        <v>10.2325502213143</v>
+      </c>
+      <c r="I53" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J53" s="40"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B54" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C54" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="D54" s="51" t="n">
+        <f aca="false">'Market Comparison'!D55</f>
+        <v>4.01</v>
+      </c>
+      <c r="E54" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F54" s="51" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="G54" s="52" t="n">
+        <v>30.5263636363636</v>
+      </c>
+      <c r="H54" s="53" t="n">
+        <v>7.61255951031512</v>
+      </c>
+      <c r="I54" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J54" s="40"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B55" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="D55" s="51" t="n">
+        <f aca="false">'Market Comparison'!D56</f>
+        <v>10.69</v>
+      </c>
+      <c r="E55" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F55" s="51" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="G55" s="52" t="n">
+        <v>23.8463636363636</v>
+      </c>
+      <c r="H55" s="53" t="n">
+        <v>2.23071689769538</v>
+      </c>
+      <c r="I55" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J55" s="40"/>
+    </row>
+    <row r="56" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B56" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="C56" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="D56" s="51" t="n">
+        <f aca="false">'Market Comparison'!D57</f>
+        <v>10.69</v>
+      </c>
+      <c r="E56" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F56" s="51" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="G56" s="52" t="n">
+        <v>23.8463636363636</v>
+      </c>
+      <c r="H56" s="53" t="n">
+        <v>2.23071689769538</v>
+      </c>
+      <c r="I56" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J56" s="40"/>
+    </row>
+    <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B57" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="C57" s="40" t="s">
+        <v>136</v>
+      </c>
+      <c r="D57" s="51" t="n">
+        <f aca="false">'Market Comparison'!D58</f>
+        <v>10.69</v>
+      </c>
+      <c r="E57" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F57" s="51" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G57" s="52" t="n">
+        <v>30.21</v>
+      </c>
+      <c r="H57" s="53" t="n">
+        <v>2.82600561272217</v>
+      </c>
+      <c r="I57" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J57" s="40"/>
+    </row>
+    <row r="58" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B58" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="C58" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="D58" s="51" t="n">
+        <f aca="false">'Market Comparison'!D59</f>
+        <v>2.89</v>
+      </c>
+      <c r="E58" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F58" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G58" s="52" t="n">
+        <v>27.1009090909091</v>
+      </c>
+      <c r="H58" s="53" t="n">
+        <v>9.37747719408619</v>
+      </c>
+      <c r="I58" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J58" s="40"/>
+    </row>
+    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B59" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="C59" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="D59" s="51" t="n">
+        <f aca="false">'Market Comparison'!D60</f>
+        <v>1.94</v>
+      </c>
+      <c r="E59" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F59" s="51" t="n">
+        <v>45.4454545454546</v>
+      </c>
+      <c r="G59" s="52" t="n">
+        <v>43.5054545454546</v>
+      </c>
+      <c r="H59" s="53" t="n">
+        <v>22.4254920337395</v>
+      </c>
+      <c r="I59" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J59" s="40"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B60" s="50" t="s">
+        <v>149</v>
+      </c>
+      <c r="C60" s="40" t="s">
+        <v>150</v>
+      </c>
+      <c r="D60" s="51" t="n">
+        <f aca="false">'Market Comparison'!D61</f>
+        <v>10.69</v>
+      </c>
+      <c r="E60" s="50" t="s">
+        <v>322</v>
+      </c>
+      <c r="F60" s="51" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="G60" s="52" t="n">
+        <v>32.86</v>
+      </c>
+      <c r="H60" s="53" t="n">
+        <v>3.07390084190833</v>
+      </c>
+      <c r="I60" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J60" s="40"/>
+    </row>
+    <row r="61" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B61" s="50" t="s">
+        <v>155</v>
+      </c>
+      <c r="C61" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="D61" s="51" t="n">
+        <f aca="false">'Market Comparison'!D62</f>
+        <v>3.201</v>
+      </c>
+      <c r="E61" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F61" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G61" s="52" t="n">
+        <v>26.7899090909091</v>
+      </c>
+      <c r="H61" s="53" t="n">
+        <v>8.36923120615717</v>
+      </c>
+      <c r="I61" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J61" s="40"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B62" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="D62" s="51" t="n">
+        <f aca="false">'Market Comparison'!D63</f>
+        <v>5.35</v>
+      </c>
+      <c r="E62" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F62" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G62" s="52" t="n">
+        <v>24.6409090909091</v>
+      </c>
+      <c r="H62" s="53" t="n">
+        <v>4.60577740016992</v>
+      </c>
+      <c r="I62" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J62" s="40"/>
+    </row>
+    <row r="63" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B63" s="50" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="D63" s="51" t="n">
+        <f aca="false">'Market Comparison'!D64</f>
+        <v>2.67</v>
+      </c>
+      <c r="E63" s="50" t="s">
+        <v>321</v>
+      </c>
+      <c r="F63" s="51" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="G63" s="52" t="n">
+        <v>27.3209090909091</v>
+      </c>
+      <c r="H63" s="53" t="n">
+        <v>10.2325502213143</v>
+      </c>
+      <c r="I63" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J63" s="40"/>
+    </row>
+    <row r="64" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B64" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="D64" s="51" t="n">
+        <f aca="false">'Market Comparison'!D65</f>
+        <v>10.69</v>
+      </c>
+      <c r="E64" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="F64" s="51" t="n">
+        <v>27.2727272727273</v>
+      </c>
+      <c r="G64" s="52" t="n">
+        <v>16.5827272727273</v>
+      </c>
+      <c r="H64" s="53" t="n">
+        <v>1.55123735011481</v>
+      </c>
+      <c r="I64" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="J64" s="40"/>
+    </row>
+    <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="57" t="s">
+        <v>331</v>
+      </c>
+      <c r="B66" s="57"/>
+      <c r="C66" s="57"/>
+      <c r="D66" s="57"/>
+      <c r="E66" s="57"/>
+      <c r="F66" s="57"/>
+      <c r="G66" s="57"/>
+      <c r="H66" s="57"/>
+      <c r="I66" s="57"/>
+      <c r="J66" s="57"/>
+    </row>
+    <row r="67" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" s="49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" s="49" t="s">
+        <v>332</v>
+      </c>
+      <c r="D67" s="49" t="s">
+        <v>333</v>
+      </c>
+      <c r="E67" s="49" t="s">
+        <v>334</v>
+      </c>
+      <c r="F67" s="49" t="s">
+        <v>335</v>
+      </c>
+      <c r="G67" s="49" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B68" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="D68" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="E68" s="51" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="F68" s="52" t="n">
+        <v>7.35545454545455</v>
+      </c>
+      <c r="G68" s="53" t="n">
+        <v>0.440182797453893</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="B69" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C69" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="D69" s="51" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="E69" s="51" t="n">
+        <v>33.41</v>
+      </c>
+      <c r="F69" s="52" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="G69" s="53" t="n">
+        <v>0.365459443280455</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="50" t="s">
+        <v>159</v>
+      </c>
+      <c r="B70" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="C70" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="D70" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="E70" s="51" t="n">
+        <v>11.81</v>
+      </c>
+      <c r="F70" s="52" t="n">
+        <v>2.45545454545455</v>
+      </c>
+      <c r="G70" s="53" t="n">
+        <v>0.207913170656609</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="B71" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="C71" s="50" t="s">
+        <v>329</v>
+      </c>
+      <c r="D71" s="51" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="E71" s="51" t="n">
+        <v>11.81</v>
+      </c>
+      <c r="F71" s="52" t="n">
+        <v>2.45545454545455</v>
+      </c>
+      <c r="G71" s="53" t="n">
+        <v>0.207913170656609</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="50" t="s">
+        <v>79</v>
+      </c>
+      <c r="B72" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="C72" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="D72" s="51" t="n">
+        <v>28.3545454545455</v>
+      </c>
+      <c r="E72" s="51" t="n">
+        <v>33.41</v>
+      </c>
+      <c r="F72" s="52" t="n">
+        <v>5.05545454545455</v>
+      </c>
+      <c r="G72" s="53" t="n">
+        <v>0.151315610459579</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="D73" s="51" t="n">
+        <v>28.3545454545455</v>
+      </c>
+      <c r="E73" s="51" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="F73" s="52" t="n">
+        <v>1.34545454545455</v>
+      </c>
+      <c r="G73" s="53" t="n">
+        <v>0.0453014998469545</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="50" t="s">
+        <v>167</v>
+      </c>
+      <c r="B74" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="C74" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="D74" s="51" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E74" s="51" t="n">
+        <v>33.41</v>
+      </c>
+      <c r="F74" s="52" t="n">
+        <v>0.909999999999997</v>
+      </c>
+      <c r="G74" s="53" t="n">
+        <v>0.027237354085603</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A66:J66"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify Summary tab back to one block; color-code price source; highlight cheaper-competitor rows
Reverts to the single closest-competitor comparison block (like the
first draft) instead of duplicated 1200/1220 column sets. "Our Quoted
Price" is now whichever is higher of the 1200-stock or 1220-stock
price, per item - shown in bold blue when the 1220-stock price was the
one used, plain black when 1200-stock was used (e.g. the two
swing-stand items, which have no 1220 price at all). Rows where the
closest competitor is cheaper than us are now highlighted amber across
the whole row, in both the main table and the "more expensive" call-out
list. Recalculates clean with zero formula errors.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1715" uniqueCount="337">
   <si>
     <t xml:space="preserve">RSEA Code</t>
   </si>
@@ -993,18 +993,18 @@
     <t xml:space="preserve">Median of (our 1220-Stock quote ÷ cheapest − 1), ex GST — negative means our quote is cheaper</t>
   </si>
   <si>
-    <t xml:space="preserve">Summary — Closest-Priced Competitor &amp; Where We're More Expensive (1200 &amp; 1220 Stock)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For each of our 60 line items: the competitor (or RSEA) whose ex-GST price is CLOSEST to our quoted price — this can be either above or below ours — shown separately for the 1200-stock and 1220-stock quoted prices, with the $ and % gap to that closest price. This is a different question from "cheapest": closest tells you who's most directly comparable to us in the market; cheapest (separately reported, see the two call-out sections below) tells you who undercuts us the most. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
+    <t xml:space="preserve">Summary — Closest-Priced Competitor &amp; Where We're More Expensive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each of our 60 line items: "Our Quoted Price" below is whichever is HIGHER of our 1200-stock or 1220-stock quoted price (shown in blue bold when the 1220-stock price was the higher/used figure, plain black when the 1200-stock price was used — e.g. for items with no 1220-stock price at all, such as the swing-stand products). Against that price, this sheet shows the competitor (or RSEA) whose ex-GST price is CLOSEST to ours — above or below — with the $ and % gap. Rows shaded amber are ones where that closest competitor (or, in some cases, a different cheaper one — see the call-out list below) is actually cheaper than us. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
   </si>
   <si>
     <t xml:space="preserve">Our Quoted Price
-(ex GST, 1200 Stock)</t>
+(ex GST, higher of 1200/1220)</t>
   </si>
   <si>
     <t xml:space="preserve">Closest-Priced
-Competitor (1200)</t>
+Competitor (or RSEA)</t>
   </si>
   <si>
     <t xml:space="preserve">Their Price
@@ -1020,15 +1020,7 @@
   </si>
   <si>
     <t xml:space="preserve">Are We More
-Expensive? (1200)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest-Priced
-Competitor (1220)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Are We More
-Expensive? (1220)</t>
+Expensive?</t>
   </si>
   <si>
     <t xml:space="preserve">eSafety Supplies</t>
@@ -1040,9 +1032,6 @@
     <t xml:space="preserve">RSEA</t>
   </si>
   <si>
-    <t xml:space="preserve">N/A — no 1220 price</t>
-  </si>
-  <si>
     <t xml:space="preserve">Seton</t>
   </si>
   <si>
@@ -1070,7 +1059,7 @@
     <t xml:space="preserve">Safety Signs Australia</t>
   </si>
   <si>
-    <t xml:space="preserve">Items We're MORE EXPENSIVE On — 1200 Stock (7 of 60 items)</t>
+    <t xml:space="preserve">Items We're MORE EXPENSIVE On (our higher-of-1200/1220 quote vs the single cheapest alternative — 7 of 60 items)</t>
   </si>
   <si>
     <t xml:space="preserve">Cheapest Alternative</t>
@@ -1086,9 +1075,6 @@
   </si>
   <si>
     <t xml:space="preserve">% We're More Expensive By</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Items We're MORE EXPENSIVE On — 1220 Stock (7 of 60 items)</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1090,7 @@
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1241,7 +1227,22 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FF1F6FEB"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1262,7 +1263,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1290,13 +1291,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -1373,7 +1380,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="67">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1582,15 +1589,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1602,12 +1605,48 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1664,7 +1703,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1686,7 +1725,7 @@
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF1F6FEB"/>
       <rgbColor rgb="FF45B1E1"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
@@ -1718,9 +1757,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>405720</xdr:colOff>
+      <xdr:colOff>405360</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>262080</xdr:rowOff>
+      <xdr:rowOff>261720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1734,7 +1773,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2193480" cy="2339640"/>
+          <a:ext cx="2193120" cy="2339280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14104,23 +14143,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P84"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14136,12 +14170,6 @@
       <c r="H1" s="48"/>
       <c r="I1" s="48"/>
       <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
     </row>
     <row r="2" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="49" t="s">
@@ -14156,14 +14184,8 @@
       <c r="H2" s="49"/>
       <c r="I2" s="49"/>
       <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-    </row>
-    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="50" t="s">
         <v>212</v>
       </c>
@@ -14192,24 +14214,6 @@
         <v>318</v>
       </c>
       <c r="J4" s="50" t="s">
-        <v>217</v>
-      </c>
-      <c r="K4" s="50" t="s">
-        <v>319</v>
-      </c>
-      <c r="L4" s="50" t="s">
-        <v>315</v>
-      </c>
-      <c r="M4" s="50" t="s">
-        <v>316</v>
-      </c>
-      <c r="N4" s="50" t="s">
-        <v>317</v>
-      </c>
-      <c r="O4" s="50" t="s">
-        <v>320</v>
-      </c>
-      <c r="P4" s="50" t="s">
         <v>221</v>
       </c>
     </row>
@@ -14224,44 +14228,24 @@
         <v>8</v>
       </c>
       <c r="D5" s="52" t="n">
-        <f aca="false">'Market Comparison'!D6</f>
-        <v>16.71</v>
+        <v>16.93275</v>
       </c>
       <c r="E5" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F5" s="52" t="n">
+        <v>319</v>
+      </c>
+      <c r="F5" s="53" t="n">
         <v>20.05</v>
       </c>
-      <c r="G5" s="53" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="H5" s="54" t="n">
-        <v>0.199880311190904</v>
+      <c r="G5" s="54" t="n">
+        <v>3.11725</v>
+      </c>
+      <c r="H5" s="55" t="n">
+        <v>0.184095908815757</v>
       </c>
       <c r="I5" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J5" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F6="","",'Market Comparison'!F6)</f>
-        <v>16.93275</v>
-      </c>
-      <c r="K5" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="L5" s="52" t="n">
-        <v>20.05</v>
-      </c>
-      <c r="M5" s="53" t="n">
-        <v>3.11725</v>
-      </c>
-      <c r="N5" s="54" t="n">
-        <v>0.184095908815757</v>
-      </c>
-      <c r="O5" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P5" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J5" s="51"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
@@ -14273,45 +14257,25 @@
       <c r="C6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="52" t="n">
-        <f aca="false">'Market Comparison'!D7</f>
+      <c r="D6" s="56" t="n">
         <v>66.83</v>
       </c>
       <c r="E6" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F6" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F6" s="53" t="n">
         <v>122.718181818182</v>
       </c>
-      <c r="G6" s="53" t="n">
+      <c r="G6" s="54" t="n">
         <v>55.888181818182</v>
       </c>
-      <c r="H6" s="54" t="n">
+      <c r="H6" s="55" t="n">
         <v>0.836273856324735</v>
       </c>
       <c r="I6" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J6" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F7="","",'Market Comparison'!F7)</f>
-        <v/>
-      </c>
-      <c r="K6" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L6" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M6" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N6" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O6" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P6" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J6" s="51"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
@@ -14323,45 +14287,25 @@
       <c r="C7" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="52" t="n">
-        <f aca="false">'Market Comparison'!D8</f>
+      <c r="D7" s="56" t="n">
         <v>44.55</v>
       </c>
       <c r="E7" s="51" t="s">
-        <v>325</v>
-      </c>
-      <c r="F7" s="52" t="n">
+        <v>322</v>
+      </c>
+      <c r="F7" s="53" t="n">
         <v>128.75</v>
       </c>
-      <c r="G7" s="53" t="n">
+      <c r="G7" s="54" t="n">
         <v>84.2</v>
       </c>
-      <c r="H7" s="54" t="n">
+      <c r="H7" s="55" t="n">
         <v>1.89001122334456</v>
       </c>
       <c r="I7" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J7" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F8="","",'Market Comparison'!F8)</f>
-        <v/>
-      </c>
-      <c r="K7" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L7" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M7" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N7" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O7" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P7" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J7" s="51"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
@@ -14374,44 +14318,24 @@
         <v>14</v>
       </c>
       <c r="D8" s="52" t="n">
-        <f aca="false">'Market Comparison'!D9</f>
-        <v>44.55</v>
+        <v>45.144</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="F8" s="52" t="n">
+        <v>323</v>
+      </c>
+      <c r="F8" s="53" t="n">
         <v>69.245</v>
       </c>
-      <c r="G8" s="53" t="n">
-        <v>24.695</v>
-      </c>
-      <c r="H8" s="54" t="n">
-        <v>0.554320987654321</v>
+      <c r="G8" s="54" t="n">
+        <v>24.101</v>
+      </c>
+      <c r="H8" s="55" t="n">
+        <v>0.533869395711501</v>
       </c>
       <c r="I8" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J8" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F9="","",'Market Comparison'!F9)</f>
-        <v>45.144</v>
-      </c>
-      <c r="K8" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="L8" s="52" t="n">
-        <v>69.245</v>
-      </c>
-      <c r="M8" s="53" t="n">
-        <v>24.101</v>
-      </c>
-      <c r="N8" s="54" t="n">
-        <v>0.533869395711501</v>
-      </c>
-      <c r="O8" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P8" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J8" s="51"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
@@ -14424,44 +14348,24 @@
         <v>16</v>
       </c>
       <c r="D9" s="52" t="n">
-        <f aca="false">'Market Comparison'!D10</f>
-        <v>69.61</v>
+        <v>70.538125</v>
       </c>
       <c r="E9" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="F9" s="52" t="n">
+        <v>323</v>
+      </c>
+      <c r="F9" s="53" t="n">
         <v>81.4</v>
       </c>
-      <c r="G9" s="53" t="n">
-        <v>11.79</v>
-      </c>
-      <c r="H9" s="54" t="n">
-        <v>0.169372216635541</v>
+      <c r="G9" s="54" t="n">
+        <v>10.861875</v>
+      </c>
+      <c r="H9" s="55" t="n">
+        <v>0.153985876432072</v>
       </c>
       <c r="I9" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J9" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F10="","",'Market Comparison'!F10)</f>
-        <v>70.538125</v>
-      </c>
-      <c r="K9" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="L9" s="52" t="n">
-        <v>81.4</v>
-      </c>
-      <c r="M9" s="53" t="n">
-        <v>10.861875</v>
-      </c>
-      <c r="N9" s="54" t="n">
-        <v>0.153985876432072</v>
-      </c>
-      <c r="O9" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P9" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J9" s="51"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
@@ -14474,44 +14378,24 @@
         <v>18</v>
       </c>
       <c r="D10" s="52" t="n">
-        <f aca="false">'Market Comparison'!D11</f>
-        <v>33.41</v>
+        <v>33.8555</v>
       </c>
       <c r="E10" s="51" t="s">
-        <v>327</v>
-      </c>
-      <c r="F10" s="52" t="n">
+        <v>324</v>
+      </c>
+      <c r="F10" s="53" t="n">
         <v>44.209</v>
       </c>
-      <c r="G10" s="53" t="n">
-        <v>10.799</v>
-      </c>
-      <c r="H10" s="54" t="n">
-        <v>0.323226578868603</v>
+      <c r="G10" s="54" t="n">
+        <v>10.3535</v>
+      </c>
+      <c r="H10" s="55" t="n">
+        <v>0.305814417155263</v>
       </c>
       <c r="I10" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J10" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F11="","",'Market Comparison'!F11)</f>
-        <v>33.8555</v>
-      </c>
-      <c r="K10" s="51" t="s">
-        <v>327</v>
-      </c>
-      <c r="L10" s="52" t="n">
-        <v>44.209</v>
-      </c>
-      <c r="M10" s="53" t="n">
-        <v>10.3535</v>
-      </c>
-      <c r="N10" s="54" t="n">
-        <v>0.305814417155263</v>
-      </c>
-      <c r="O10" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P10" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J10" s="51"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
@@ -14524,94 +14408,54 @@
         <v>20</v>
       </c>
       <c r="D11" s="52" t="n">
-        <f aca="false">'Market Comparison'!D12</f>
-        <v>44.55</v>
+        <v>45.144</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F11" s="52" t="n">
+        <v>319</v>
+      </c>
+      <c r="F11" s="53" t="n">
         <v>70.36</v>
       </c>
-      <c r="G11" s="53" t="n">
-        <v>25.81</v>
-      </c>
-      <c r="H11" s="54" t="n">
-        <v>0.579349046015713</v>
+      <c r="G11" s="54" t="n">
+        <v>25.216</v>
+      </c>
+      <c r="H11" s="55" t="n">
+        <v>0.558568137515506</v>
       </c>
       <c r="I11" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J11" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F12="","",'Market Comparison'!F12)</f>
-        <v>45.144</v>
-      </c>
-      <c r="K11" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="L11" s="52" t="n">
-        <v>70.36</v>
-      </c>
-      <c r="M11" s="53" t="n">
-        <v>25.216</v>
-      </c>
-      <c r="N11" s="54" t="n">
-        <v>0.558568137515506</v>
-      </c>
-      <c r="O11" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P11" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J11" s="51"/>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="51" t="s">
+      <c r="A12" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B12" s="51" t="s">
+      <c r="B12" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="52" t="n">
-        <f aca="false">'Market Comparison'!D13</f>
-        <v>33.41</v>
-      </c>
-      <c r="E12" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="F12" s="52" t="n">
+      <c r="D12" s="59" t="n">
+        <v>33.8555</v>
+      </c>
+      <c r="E12" s="57" t="s">
+        <v>325</v>
+      </c>
+      <c r="F12" s="60" t="n">
         <v>33.1818181818182</v>
       </c>
-      <c r="G12" s="55" t="n">
-        <v>-0.228181818181795</v>
-      </c>
-      <c r="H12" s="56" t="n">
-        <v>-0.00682974612935634</v>
-      </c>
-      <c r="I12" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="J12" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F13="","",'Market Comparison'!F13)</f>
-        <v>33.8555</v>
-      </c>
-      <c r="K12" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="L12" s="52" t="n">
-        <v>33.1818181818182</v>
-      </c>
-      <c r="M12" s="55" t="n">
+      <c r="G12" s="61" t="n">
         <v>-0.673681818181798</v>
       </c>
-      <c r="N12" s="56" t="n">
+      <c r="H12" s="62" t="n">
         <v>-0.019898740771272</v>
       </c>
-      <c r="O12" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P12" s="41"/>
+      <c r="I12" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J12" s="57"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
@@ -14624,44 +14468,24 @@
         <v>82</v>
       </c>
       <c r="D13" s="52" t="n">
-        <f aca="false">'Market Comparison'!D14</f>
-        <v>25.06</v>
+        <v>25.394125</v>
       </c>
       <c r="E13" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F13" s="52" t="n">
+        <v>319</v>
+      </c>
+      <c r="F13" s="53" t="n">
         <v>43.09</v>
       </c>
-      <c r="G13" s="53" t="n">
-        <v>18.03</v>
-      </c>
-      <c r="H13" s="54" t="n">
-        <v>0.719473264166002</v>
+      <c r="G13" s="54" t="n">
+        <v>17.695875</v>
+      </c>
+      <c r="H13" s="55" t="n">
+        <v>0.696849172790951</v>
       </c>
       <c r="I13" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J13" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F14="","",'Market Comparison'!F14)</f>
-        <v>25.394125</v>
-      </c>
-      <c r="K13" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="L13" s="52" t="n">
-        <v>43.09</v>
-      </c>
-      <c r="M13" s="53" t="n">
-        <v>17.695875</v>
-      </c>
-      <c r="N13" s="54" t="n">
-        <v>0.696849172790951</v>
-      </c>
-      <c r="O13" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P13" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J13" s="51"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
@@ -14674,44 +14498,24 @@
         <v>102</v>
       </c>
       <c r="D14" s="52" t="n">
-        <f aca="false">'Market Comparison'!D15</f>
-        <v>8.35</v>
+        <v>8.461375</v>
       </c>
       <c r="E14" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F14" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F14" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G14" s="53" t="n">
-        <v>21.6409090909091</v>
-      </c>
-      <c r="H14" s="54" t="n">
-        <v>2.59172563962983</v>
+      <c r="G14" s="54" t="n">
+        <v>21.5295340909091</v>
+      </c>
+      <c r="H14" s="55" t="n">
+        <v>2.54444863759248</v>
       </c>
       <c r="I14" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J14" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F15="","",'Market Comparison'!F15)</f>
-        <v>8.461375</v>
-      </c>
-      <c r="K14" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="L14" s="52" t="n">
-        <v>29.9909090909091</v>
-      </c>
-      <c r="M14" s="53" t="n">
-        <v>21.5295340909091</v>
-      </c>
-      <c r="N14" s="54" t="n">
-        <v>2.54444863759248</v>
-      </c>
-      <c r="O14" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P14" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J14" s="51"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
@@ -14724,44 +14528,24 @@
         <v>108</v>
       </c>
       <c r="D15" s="52" t="n">
-        <f aca="false">'Market Comparison'!D16</f>
-        <v>15.59</v>
+        <v>15.81275</v>
       </c>
       <c r="E15" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F15" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F15" s="53" t="n">
         <v>40.9</v>
       </c>
-      <c r="G15" s="53" t="n">
-        <v>25.31</v>
-      </c>
-      <c r="H15" s="54" t="n">
-        <v>1.62347658755613</v>
+      <c r="G15" s="54" t="n">
+        <v>25.08725</v>
+      </c>
+      <c r="H15" s="55" t="n">
+        <v>1.58652037121943</v>
       </c>
       <c r="I15" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J15" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F16="","",'Market Comparison'!F16)</f>
-        <v>15.81275</v>
-      </c>
-      <c r="K15" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="L15" s="52" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="M15" s="53" t="n">
-        <v>25.08725</v>
-      </c>
-      <c r="N15" s="54" t="n">
-        <v>1.58652037121943</v>
-      </c>
-      <c r="O15" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P15" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J15" s="51"/>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="51" t="s">
@@ -14774,44 +14558,24 @@
         <v>118</v>
       </c>
       <c r="D16" s="52" t="n">
-        <f aca="false">'Market Comparison'!D17</f>
-        <v>8.35</v>
+        <v>8.461375</v>
       </c>
       <c r="E16" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F16" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F16" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G16" s="53" t="n">
-        <v>21.6409090909091</v>
-      </c>
-      <c r="H16" s="54" t="n">
-        <v>2.59172563962983</v>
+      <c r="G16" s="54" t="n">
+        <v>21.5295340909091</v>
+      </c>
+      <c r="H16" s="55" t="n">
+        <v>2.54444863759248</v>
       </c>
       <c r="I16" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J16" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F17="","",'Market Comparison'!F17)</f>
-        <v>8.461375</v>
-      </c>
-      <c r="K16" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="L16" s="52" t="n">
-        <v>29.9909090909091</v>
-      </c>
-      <c r="M16" s="53" t="n">
-        <v>21.5295340909091</v>
-      </c>
-      <c r="N16" s="54" t="n">
-        <v>2.54444863759248</v>
-      </c>
-      <c r="O16" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P16" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J16" s="51"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="51" t="s">
@@ -14824,94 +14588,54 @@
         <v>128</v>
       </c>
       <c r="D17" s="52" t="n">
-        <f aca="false">'Market Comparison'!D18</f>
-        <v>29.7</v>
+        <v>30.1455</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F17" s="52" t="n">
+        <v>327</v>
+      </c>
+      <c r="F17" s="53" t="n">
         <v>37.3909090909091</v>
       </c>
-      <c r="G17" s="53" t="n">
-        <v>7.6909090909091</v>
-      </c>
-      <c r="H17" s="54" t="n">
-        <v>0.258953168044077</v>
+      <c r="G17" s="54" t="n">
+        <v>7.2454090909091</v>
+      </c>
+      <c r="H17" s="55" t="n">
+        <v>0.240347948811899</v>
       </c>
       <c r="I17" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J17" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F18="","",'Market Comparison'!F18)</f>
+        <v>320</v>
+      </c>
+      <c r="J17" s="51"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="57" t="s">
+        <v>222</v>
+      </c>
+      <c r="B18" s="57" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="58" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="59" t="n">
         <v>30.1455</v>
       </c>
-      <c r="K17" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="L17" s="52" t="n">
-        <v>37.3909090909091</v>
-      </c>
-      <c r="M17" s="53" t="n">
-        <v>7.2454090909091</v>
-      </c>
-      <c r="N17" s="54" t="n">
-        <v>0.240347948811899</v>
-      </c>
-      <c r="O17" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P17" s="41"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="41" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="52" t="n">
-        <f aca="false">'Market Comparison'!D19</f>
-        <v>29.7</v>
-      </c>
-      <c r="E18" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F18" s="52" t="n">
+      <c r="E18" s="57" t="s">
+        <v>327</v>
+      </c>
+      <c r="F18" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="G18" s="55" t="n">
-        <v>-1.3454545454545</v>
-      </c>
-      <c r="H18" s="56" t="n">
-        <v>-0.0453014998469528</v>
-      </c>
-      <c r="I18" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="J18" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F19="","",'Market Comparison'!F19)</f>
-        <v>30.1455</v>
-      </c>
-      <c r="K18" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="L18" s="52" t="n">
-        <v>28.3545454545455</v>
-      </c>
-      <c r="M18" s="55" t="n">
+      <c r="G18" s="61" t="n">
         <v>-1.7909545454545</v>
       </c>
-      <c r="N18" s="56" t="n">
+      <c r="H18" s="62" t="n">
         <v>-0.0594103446768007</v>
       </c>
-      <c r="O18" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P18" s="41"/>
+      <c r="I18" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J18" s="57"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="51" t="s">
@@ -14924,94 +14648,54 @@
         <v>138</v>
       </c>
       <c r="D19" s="52" t="n">
-        <f aca="false">'Market Comparison'!D20</f>
-        <v>16.71</v>
+        <v>16.93275</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F19" s="52" t="n">
+        <v>327</v>
+      </c>
+      <c r="F19" s="53" t="n">
         <v>23.3090909090909</v>
       </c>
-      <c r="G19" s="53" t="n">
-        <v>6.5990909090909</v>
-      </c>
-      <c r="H19" s="54" t="n">
-        <v>0.394918666013818</v>
+      <c r="G19" s="54" t="n">
+        <v>6.3763409090909</v>
+      </c>
+      <c r="H19" s="55" t="n">
+        <v>0.376568537838857</v>
       </c>
       <c r="I19" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J19" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F20="","",'Market Comparison'!F20)</f>
-        <v>16.93275</v>
-      </c>
-      <c r="K19" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="L19" s="52" t="n">
-        <v>23.3090909090909</v>
-      </c>
-      <c r="M19" s="53" t="n">
-        <v>6.3763409090909</v>
-      </c>
-      <c r="N19" s="54" t="n">
-        <v>0.376568537838857</v>
-      </c>
-      <c r="O19" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P19" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J19" s="51"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="51" t="s">
+      <c r="A20" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B20" s="51" t="s">
+      <c r="B20" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="52" t="n">
-        <f aca="false">'Market Comparison'!D21</f>
-        <v>33.41</v>
-      </c>
-      <c r="E20" s="51" t="s">
-        <v>331</v>
-      </c>
-      <c r="F20" s="52" t="n">
+      <c r="D20" s="59" t="n">
+        <v>33.8555</v>
+      </c>
+      <c r="E20" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="F20" s="60" t="n">
         <v>28.99</v>
       </c>
-      <c r="G20" s="55" t="n">
-        <v>-4.42</v>
-      </c>
-      <c r="H20" s="56" t="n">
-        <v>-0.132295719844358</v>
-      </c>
-      <c r="I20" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="J20" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F21="","",'Market Comparison'!F21)</f>
-        <v>33.8555</v>
-      </c>
-      <c r="K20" s="51" t="s">
-        <v>331</v>
-      </c>
-      <c r="L20" s="52" t="n">
-        <v>28.99</v>
-      </c>
-      <c r="M20" s="55" t="n">
+      <c r="G20" s="61" t="n">
         <v>-4.8655</v>
       </c>
-      <c r="N20" s="56" t="n">
+      <c r="H20" s="62" t="n">
         <v>-0.14371372450562</v>
       </c>
-      <c r="O20" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P20" s="41"/>
+      <c r="I20" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J20" s="57"/>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="51" t="s">
@@ -15024,44 +14708,24 @@
         <v>148</v>
       </c>
       <c r="D21" s="52" t="n">
-        <f aca="false">'Market Comparison'!D22</f>
-        <v>11.81</v>
+        <v>12.03275</v>
       </c>
       <c r="E21" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F21" s="52" t="n">
+        <v>329</v>
+      </c>
+      <c r="F21" s="53" t="n">
         <v>21.2</v>
       </c>
-      <c r="G21" s="53" t="n">
-        <v>9.39</v>
-      </c>
-      <c r="H21" s="54" t="n">
-        <v>0.795088907705334</v>
+      <c r="G21" s="54" t="n">
+        <v>9.16725</v>
+      </c>
+      <c r="H21" s="55" t="n">
+        <v>0.761858261827097</v>
       </c>
       <c r="I21" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J21" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F22="","",'Market Comparison'!F22)</f>
-        <v>12.03275</v>
-      </c>
-      <c r="K21" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="L21" s="52" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="M21" s="53" t="n">
-        <v>9.16725</v>
-      </c>
-      <c r="N21" s="54" t="n">
-        <v>0.761858261827097</v>
-      </c>
-      <c r="O21" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P21" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J21" s="51"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="51" t="s">
@@ -15074,44 +14738,24 @@
         <v>152</v>
       </c>
       <c r="D22" s="52" t="n">
-        <f aca="false">'Market Comparison'!D23</f>
-        <v>11.81</v>
+        <v>12.03275</v>
       </c>
       <c r="E22" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F22" s="52" t="n">
+        <v>329</v>
+      </c>
+      <c r="F22" s="53" t="n">
         <v>21.2</v>
       </c>
-      <c r="G22" s="53" t="n">
-        <v>9.39</v>
-      </c>
-      <c r="H22" s="54" t="n">
-        <v>0.795088907705334</v>
+      <c r="G22" s="54" t="n">
+        <v>9.16725</v>
+      </c>
+      <c r="H22" s="55" t="n">
+        <v>0.761858261827097</v>
       </c>
       <c r="I22" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J22" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F23="","",'Market Comparison'!F23)</f>
-        <v>12.03275</v>
-      </c>
-      <c r="K22" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="L22" s="52" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="M22" s="53" t="n">
-        <v>9.16725</v>
-      </c>
-      <c r="N22" s="54" t="n">
-        <v>0.761858261827097</v>
-      </c>
-      <c r="O22" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P22" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J22" s="51"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="51" t="s">
@@ -15124,144 +14768,84 @@
         <v>154</v>
       </c>
       <c r="D23" s="52" t="n">
-        <f aca="false">'Market Comparison'!D24</f>
-        <v>5.9</v>
+        <v>6.011375</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F23" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F23" s="53" t="n">
         <v>34.5363636363636</v>
       </c>
-      <c r="G23" s="53" t="n">
-        <v>28.6363636363636</v>
-      </c>
-      <c r="H23" s="54" t="n">
-        <v>4.85362095531587</v>
+      <c r="G23" s="54" t="n">
+        <v>28.5249886363636</v>
+      </c>
+      <c r="H23" s="55" t="n">
+        <v>4.74516872368861</v>
       </c>
       <c r="I23" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J23" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F24="","",'Market Comparison'!F24)</f>
-        <v>6.011375</v>
-      </c>
-      <c r="K23" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="L23" s="52" t="n">
-        <v>34.5363636363636</v>
-      </c>
-      <c r="M23" s="53" t="n">
-        <v>28.5249886363636</v>
-      </c>
-      <c r="N23" s="54" t="n">
-        <v>4.74516872368861</v>
-      </c>
-      <c r="O23" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P23" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J23" s="51"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="51" t="s">
+      <c r="A24" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B24" s="51" t="s">
+      <c r="B24" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="D24" s="52" t="n">
-        <f aca="false">'Market Comparison'!D25</f>
-        <v>11.81</v>
-      </c>
-      <c r="E24" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F24" s="52" t="n">
+      <c r="D24" s="59" t="n">
+        <v>12.03275</v>
+      </c>
+      <c r="E24" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="F24" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="G24" s="55" t="n">
-        <v>-2.45545454545455</v>
-      </c>
-      <c r="H24" s="56" t="n">
-        <v>-0.207913170656609</v>
-      </c>
-      <c r="I24" s="57" t="s">
+      <c r="G24" s="61" t="n">
+        <v>-2.67820454545455</v>
+      </c>
+      <c r="H24" s="62" t="n">
+        <v>-0.222576264399622</v>
+      </c>
+      <c r="I24" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J24" s="57"/>
+    </row>
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="57" t="s">
+        <v>222</v>
+      </c>
+      <c r="B25" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C25" s="58" t="s">
+        <v>172</v>
+      </c>
+      <c r="D25" s="59" t="n">
+        <v>12.03275</v>
+      </c>
+      <c r="E25" s="57" t="s">
         <v>329</v>
       </c>
-      <c r="J24" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F25="","",'Market Comparison'!F25)</f>
-        <v>12.03275</v>
-      </c>
-      <c r="K24" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="L24" s="52" t="n">
+      <c r="F25" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="M24" s="55" t="n">
+      <c r="G25" s="61" t="n">
         <v>-2.67820454545455</v>
       </c>
-      <c r="N24" s="56" t="n">
+      <c r="H25" s="62" t="n">
         <v>-0.222576264399622</v>
       </c>
-      <c r="O24" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P24" s="41"/>
-    </row>
-    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>171</v>
-      </c>
-      <c r="C25" s="41" t="s">
-        <v>172</v>
-      </c>
-      <c r="D25" s="52" t="n">
-        <f aca="false">'Market Comparison'!D26</f>
-        <v>11.81</v>
-      </c>
-      <c r="E25" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F25" s="52" t="n">
-        <v>9.35454545454545</v>
-      </c>
-      <c r="G25" s="55" t="n">
-        <v>-2.45545454545455</v>
-      </c>
-      <c r="H25" s="56" t="n">
-        <v>-0.207913170656609</v>
-      </c>
-      <c r="I25" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="J25" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F26="","",'Market Comparison'!F26)</f>
-        <v>12.03275</v>
-      </c>
-      <c r="K25" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="L25" s="52" t="n">
-        <v>9.35454545454545</v>
-      </c>
-      <c r="M25" s="55" t="n">
-        <v>-2.67820454545455</v>
-      </c>
-      <c r="N25" s="56" t="n">
-        <v>-0.222576264399622</v>
-      </c>
-      <c r="O25" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P25" s="41"/>
+      <c r="I25" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J25" s="57"/>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="51" t="s">
@@ -15274,94 +14858,54 @@
         <v>173</v>
       </c>
       <c r="D26" s="52" t="n">
-        <f aca="false">'Market Comparison'!D27</f>
-        <v>11.81</v>
+        <v>12.03275</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F26" s="52" t="n">
+        <v>329</v>
+      </c>
+      <c r="F26" s="53" t="n">
         <v>21.2</v>
       </c>
-      <c r="G26" s="53" t="n">
-        <v>9.39</v>
-      </c>
-      <c r="H26" s="54" t="n">
-        <v>0.795088907705334</v>
+      <c r="G26" s="54" t="n">
+        <v>9.16725</v>
+      </c>
+      <c r="H26" s="55" t="n">
+        <v>0.761858261827097</v>
       </c>
       <c r="I26" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J26" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F27="","",'Market Comparison'!F27)</f>
-        <v>12.03275</v>
-      </c>
-      <c r="K26" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="L26" s="52" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="M26" s="53" t="n">
-        <v>9.16725</v>
-      </c>
-      <c r="N26" s="54" t="n">
-        <v>0.761858261827097</v>
-      </c>
-      <c r="O26" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P26" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J26" s="51"/>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="51" t="s">
+      <c r="A27" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="D27" s="52" t="n">
-        <f aca="false">'Market Comparison'!D28</f>
-        <v>33.41</v>
-      </c>
-      <c r="E27" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="F27" s="52" t="n">
+      <c r="D27" s="59" t="n">
+        <v>33.8555</v>
+      </c>
+      <c r="E27" s="57" t="s">
+        <v>325</v>
+      </c>
+      <c r="F27" s="60" t="n">
         <v>32.5</v>
       </c>
-      <c r="G27" s="55" t="n">
-        <v>-0.909999999999997</v>
-      </c>
-      <c r="H27" s="56" t="n">
-        <v>-0.027237354085603</v>
-      </c>
-      <c r="I27" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="J27" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F28="","",'Market Comparison'!F28)</f>
-        <v>33.8555</v>
-      </c>
-      <c r="K27" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="L27" s="52" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="M27" s="55" t="n">
+      <c r="G27" s="61" t="n">
         <v>-1.3555</v>
       </c>
-      <c r="N27" s="56" t="n">
+      <c r="H27" s="62" t="n">
         <v>-0.0400378077417258</v>
       </c>
-      <c r="O27" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="P27" s="41"/>
+      <c r="I27" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="J27" s="57"/>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="51" t="s">
@@ -15374,44 +14918,24 @@
         <v>175</v>
       </c>
       <c r="D28" s="52" t="n">
-        <f aca="false">'Market Comparison'!D29</f>
-        <v>33.41</v>
+        <v>33.8555</v>
       </c>
       <c r="E28" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="F28" s="52" t="n">
+        <v>325</v>
+      </c>
+      <c r="F28" s="53" t="n">
         <v>45</v>
       </c>
-      <c r="G28" s="53" t="n">
-        <v>11.59</v>
-      </c>
-      <c r="H28" s="54" t="n">
-        <v>0.346902125112242</v>
+      <c r="G28" s="54" t="n">
+        <v>11.1445</v>
+      </c>
+      <c r="H28" s="55" t="n">
+        <v>0.329178420049918</v>
       </c>
       <c r="I28" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J28" s="52" t="n">
-        <f aca="false">IF('Market Comparison'!F29="","",'Market Comparison'!F29)</f>
-        <v>33.8555</v>
-      </c>
-      <c r="K28" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="L28" s="52" t="n">
-        <v>45</v>
-      </c>
-      <c r="M28" s="53" t="n">
-        <v>11.1445</v>
-      </c>
-      <c r="N28" s="54" t="n">
-        <v>0.329178420049918</v>
-      </c>
-      <c r="O28" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="P28" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J28" s="51"/>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="51" t="s">
@@ -15423,45 +14947,25 @@
       <c r="C29" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="52" t="n">
-        <f aca="false">'Market Comparison'!D30</f>
+      <c r="D29" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E29" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="F29" s="52" t="n">
+        <v>323</v>
+      </c>
+      <c r="F29" s="53" t="n">
         <v>30.8</v>
       </c>
-      <c r="G29" s="53" t="n">
+      <c r="G29" s="54" t="n">
         <v>17.73</v>
       </c>
-      <c r="H29" s="54" t="n">
+      <c r="H29" s="55" t="n">
         <v>1.35654169854629</v>
       </c>
       <c r="I29" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J29" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F30="","",'Market Comparison'!F30)</f>
-        <v/>
-      </c>
-      <c r="K29" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L29" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M29" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N29" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O29" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P29" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J29" s="51"/>
     </row>
     <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="51" t="s">
@@ -15473,45 +14977,25 @@
       <c r="C30" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="D30" s="52" t="n">
-        <f aca="false">'Market Comparison'!D31</f>
+      <c r="D30" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E30" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F30" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F30" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G30" s="53" t="n">
+      <c r="G30" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H30" s="54" t="n">
+      <c r="H30" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I30" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J30" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F31="","",'Market Comparison'!F31)</f>
-        <v/>
-      </c>
-      <c r="K30" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L30" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M30" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N30" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O30" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P30" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J30" s="51"/>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="51" t="s">
@@ -15523,45 +15007,25 @@
       <c r="C31" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="52" t="n">
-        <f aca="false">'Market Comparison'!D32</f>
+      <c r="D31" s="56" t="n">
         <v>16.04</v>
       </c>
       <c r="E31" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F31" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F31" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G31" s="53" t="n">
+      <c r="G31" s="54" t="n">
         <v>14.96</v>
       </c>
-      <c r="H31" s="54" t="n">
+      <c r="H31" s="55" t="n">
         <v>0.932668329177057</v>
       </c>
       <c r="I31" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J31" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F32="","",'Market Comparison'!F32)</f>
-        <v/>
-      </c>
-      <c r="K31" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L31" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M31" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N31" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O31" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P31" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J31" s="51"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="51" t="s">
@@ -15573,45 +15037,25 @@
       <c r="C32" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="52" t="n">
-        <f aca="false">'Market Comparison'!D33</f>
+      <c r="D32" s="56" t="n">
         <v>16.04</v>
       </c>
       <c r="E32" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F32" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F32" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G32" s="53" t="n">
+      <c r="G32" s="54" t="n">
         <v>14.96</v>
       </c>
-      <c r="H32" s="54" t="n">
+      <c r="H32" s="55" t="n">
         <v>0.932668329177057</v>
       </c>
       <c r="I32" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J32" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F33="","",'Market Comparison'!F33)</f>
-        <v/>
-      </c>
-      <c r="K32" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L32" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M32" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N32" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O32" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P32" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J32" s="51"/>
     </row>
     <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="51" t="s">
@@ -15623,45 +15067,25 @@
       <c r="C33" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="D33" s="52" t="n">
-        <f aca="false">'Market Comparison'!D34</f>
+      <c r="D33" s="56" t="n">
         <v>16.04</v>
       </c>
       <c r="E33" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F33" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F33" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G33" s="53" t="n">
+      <c r="G33" s="54" t="n">
         <v>14.96</v>
       </c>
-      <c r="H33" s="54" t="n">
+      <c r="H33" s="55" t="n">
         <v>0.932668329177057</v>
       </c>
       <c r="I33" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J33" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F34="","",'Market Comparison'!F34)</f>
-        <v/>
-      </c>
-      <c r="K33" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L33" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M33" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N33" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O33" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P33" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J33" s="51"/>
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="51" t="s">
@@ -15673,45 +15097,25 @@
       <c r="C34" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="D34" s="52" t="n">
-        <f aca="false">'Market Comparison'!D35</f>
+      <c r="D34" s="56" t="n">
         <v>16.04</v>
       </c>
       <c r="E34" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F34" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F34" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G34" s="53" t="n">
+      <c r="G34" s="54" t="n">
         <v>14.96</v>
       </c>
-      <c r="H34" s="54" t="n">
+      <c r="H34" s="55" t="n">
         <v>0.932668329177057</v>
       </c>
       <c r="I34" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J34" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F35="","",'Market Comparison'!F35)</f>
-        <v/>
-      </c>
-      <c r="K34" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L34" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M34" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N34" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O34" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P34" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J34" s="51"/>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="51" t="s">
@@ -15723,45 +15127,25 @@
       <c r="C35" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="52" t="n">
-        <f aca="false">'Market Comparison'!D36</f>
+      <c r="D35" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E35" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F35" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F35" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G35" s="53" t="n">
+      <c r="G35" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H35" s="54" t="n">
+      <c r="H35" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I35" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J35" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F36="","",'Market Comparison'!F36)</f>
-        <v/>
-      </c>
-      <c r="K35" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L35" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M35" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N35" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O35" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P35" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J35" s="51"/>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="51" t="s">
@@ -15773,45 +15157,25 @@
       <c r="C36" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="52" t="n">
-        <f aca="false">'Market Comparison'!D37</f>
+      <c r="D36" s="56" t="n">
         <v>16.04</v>
       </c>
       <c r="E36" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F36" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F36" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G36" s="53" t="n">
+      <c r="G36" s="54" t="n">
         <v>14.96</v>
       </c>
-      <c r="H36" s="54" t="n">
+      <c r="H36" s="55" t="n">
         <v>0.932668329177057</v>
       </c>
       <c r="I36" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J36" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F37="","",'Market Comparison'!F37)</f>
-        <v/>
-      </c>
-      <c r="K36" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L36" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M36" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N36" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O36" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P36" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J36" s="51"/>
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="51" t="s">
@@ -15823,45 +15187,25 @@
       <c r="C37" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="D37" s="52" t="n">
-        <f aca="false">'Market Comparison'!D38</f>
+      <c r="D37" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E37" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F37" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F37" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G37" s="53" t="n">
+      <c r="G37" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H37" s="54" t="n">
+      <c r="H37" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I37" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J37" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F38="","",'Market Comparison'!F38)</f>
-        <v/>
-      </c>
-      <c r="K37" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L37" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M37" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N37" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O37" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P37" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J37" s="51"/>
     </row>
     <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="51" t="s">
@@ -15873,45 +15217,25 @@
       <c r="C38" s="41" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="52" t="n">
-        <f aca="false">'Market Comparison'!D39</f>
+      <c r="D38" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E38" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F38" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F38" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G38" s="53" t="n">
+      <c r="G38" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H38" s="54" t="n">
+      <c r="H38" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I38" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J38" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F39="","",'Market Comparison'!F39)</f>
-        <v/>
-      </c>
-      <c r="K38" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L38" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M38" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N38" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O38" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P38" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J38" s="51"/>
     </row>
     <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="51" t="s">
@@ -15923,45 +15247,25 @@
       <c r="C39" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="D39" s="52" t="n">
-        <f aca="false">'Market Comparison'!D40</f>
+      <c r="D39" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E39" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F39" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F39" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G39" s="53" t="n">
+      <c r="G39" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H39" s="54" t="n">
+      <c r="H39" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I39" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J39" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F40="","",'Market Comparison'!F40)</f>
-        <v/>
-      </c>
-      <c r="K39" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L39" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M39" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N39" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O39" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P39" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J39" s="51"/>
     </row>
     <row r="40" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="51" t="s">
@@ -15973,45 +15277,25 @@
       <c r="C40" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="D40" s="52" t="n">
-        <f aca="false">'Market Comparison'!D41</f>
+      <c r="D40" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E40" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F40" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F40" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G40" s="53" t="n">
+      <c r="G40" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H40" s="54" t="n">
+      <c r="H40" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I40" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J40" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F41="","",'Market Comparison'!F41)</f>
-        <v/>
-      </c>
-      <c r="K40" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L40" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M40" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N40" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O40" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P40" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J40" s="51"/>
     </row>
     <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="51" t="s">
@@ -16023,45 +15307,25 @@
       <c r="C41" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="D41" s="52" t="n">
-        <f aca="false">'Market Comparison'!D42</f>
+      <c r="D41" s="56" t="n">
         <v>13.07</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F41" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F41" s="53" t="n">
         <v>31</v>
       </c>
-      <c r="G41" s="53" t="n">
+      <c r="G41" s="54" t="n">
         <v>17.93</v>
       </c>
-      <c r="H41" s="54" t="n">
+      <c r="H41" s="55" t="n">
         <v>1.37184391736802</v>
       </c>
       <c r="I41" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J41" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F42="","",'Market Comparison'!F42)</f>
-        <v/>
-      </c>
-      <c r="K41" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L41" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M41" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N41" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O41" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P41" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J41" s="51"/>
     </row>
     <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="51" t="s">
@@ -16073,45 +15337,25 @@
       <c r="C42" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="52" t="n">
-        <f aca="false">'Market Comparison'!D43</f>
+      <c r="D42" s="56" t="n">
         <v>5.35</v>
       </c>
       <c r="E42" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F42" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F42" s="53" t="n">
         <v>34.5363636363636</v>
       </c>
-      <c r="G42" s="53" t="n">
+      <c r="G42" s="54" t="n">
         <v>29.1863636363636</v>
       </c>
-      <c r="H42" s="54" t="n">
+      <c r="H42" s="55" t="n">
         <v>5.4553950722175</v>
       </c>
       <c r="I42" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J42" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F43="","",'Market Comparison'!F43)</f>
-        <v/>
-      </c>
-      <c r="K42" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L42" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M42" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N42" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O42" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P42" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J42" s="51"/>
     </row>
     <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="51" t="s">
@@ -16123,45 +15367,25 @@
       <c r="C43" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="D43" s="52" t="n">
-        <f aca="false">'Market Comparison'!D44</f>
+      <c r="D43" s="56" t="n">
         <v>2.67</v>
       </c>
       <c r="E43" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F43" s="52" t="n">
+        <v>329</v>
+      </c>
+      <c r="F43" s="53" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="G43" s="53" t="n">
+      <c r="G43" s="54" t="n">
         <v>6.68454545454545</v>
       </c>
-      <c r="H43" s="54" t="n">
+      <c r="H43" s="55" t="n">
         <v>2.50357507660878</v>
       </c>
       <c r="I43" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J43" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F44="","",'Market Comparison'!F44)</f>
-        <v/>
-      </c>
-      <c r="K43" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L43" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M43" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N43" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O43" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P43" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J43" s="51"/>
     </row>
     <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="51" t="s">
@@ -16173,45 +15397,25 @@
       <c r="C44" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="D44" s="52" t="n">
-        <f aca="false">'Market Comparison'!D45</f>
+      <c r="D44" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E44" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F44" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F44" s="53" t="n">
         <v>23.4090909090909</v>
       </c>
-      <c r="G44" s="53" t="n">
+      <c r="G44" s="54" t="n">
         <v>12.7190909090909</v>
       </c>
-      <c r="H44" s="54" t="n">
+      <c r="H44" s="55" t="n">
         <v>1.18981205884854</v>
       </c>
       <c r="I44" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J44" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F45="","",'Market Comparison'!F45)</f>
-        <v/>
-      </c>
-      <c r="K44" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L44" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M44" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N44" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O44" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P44" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J44" s="51"/>
     </row>
     <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="51" t="s">
@@ -16223,45 +15427,25 @@
       <c r="C45" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="D45" s="52" t="n">
-        <f aca="false">'Market Comparison'!D46</f>
+      <c r="D45" s="56" t="n">
         <v>2.67</v>
       </c>
       <c r="E45" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F45" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F45" s="53" t="n">
         <v>22.7181818181818</v>
       </c>
-      <c r="G45" s="53" t="n">
+      <c r="G45" s="54" t="n">
         <v>20.0481818181818</v>
       </c>
-      <c r="H45" s="54" t="n">
+      <c r="H45" s="55" t="n">
         <v>7.50868232890704</v>
       </c>
       <c r="I45" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J45" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F46="","",'Market Comparison'!F46)</f>
-        <v/>
-      </c>
-      <c r="K45" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L45" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M45" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N45" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O45" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P45" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J45" s="51"/>
     </row>
     <row r="46" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="51" t="s">
@@ -16273,45 +15457,25 @@
       <c r="C46" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="D46" s="52" t="n">
-        <f aca="false">'Market Comparison'!D47</f>
+      <c r="D46" s="56" t="n">
         <v>9.5</v>
       </c>
       <c r="E46" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F46" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F46" s="53" t="n">
         <v>40.9</v>
       </c>
-      <c r="G46" s="53" t="n">
+      <c r="G46" s="54" t="n">
         <v>31.4</v>
       </c>
-      <c r="H46" s="54" t="n">
+      <c r="H46" s="55" t="n">
         <v>3.30526315789474</v>
       </c>
       <c r="I46" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J46" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F47="","",'Market Comparison'!F47)</f>
-        <v/>
-      </c>
-      <c r="K46" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L46" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M46" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N46" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O46" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P46" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J46" s="51"/>
     </row>
     <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="51" t="s">
@@ -16323,45 +15487,25 @@
       <c r="C47" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="D47" s="52" t="n">
-        <f aca="false">'Market Comparison'!D48</f>
+      <c r="D47" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E47" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F47" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F47" s="53" t="n">
         <v>40.9</v>
       </c>
-      <c r="G47" s="53" t="n">
+      <c r="G47" s="54" t="n">
         <v>30.21</v>
       </c>
-      <c r="H47" s="54" t="n">
+      <c r="H47" s="55" t="n">
         <v>2.82600561272217</v>
       </c>
       <c r="I47" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J47" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F48="","",'Market Comparison'!F48)</f>
-        <v/>
-      </c>
-      <c r="K47" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L47" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M47" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N47" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O47" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P47" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J47" s="51"/>
     </row>
     <row r="48" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="51" t="s">
@@ -16373,45 +15517,25 @@
       <c r="C48" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="D48" s="52" t="n">
-        <f aca="false">'Market Comparison'!D49</f>
+      <c r="D48" s="56" t="n">
         <v>5.35</v>
       </c>
       <c r="E48" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F48" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F48" s="53" t="n">
         <v>20.9090909090909</v>
       </c>
-      <c r="G48" s="53" t="n">
+      <c r="G48" s="54" t="n">
         <v>15.5590909090909</v>
       </c>
-      <c r="H48" s="54" t="n">
+      <c r="H48" s="55" t="n">
         <v>2.90824129141886</v>
       </c>
       <c r="I48" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J48" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F49="","",'Market Comparison'!F49)</f>
-        <v/>
-      </c>
-      <c r="K48" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L48" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M48" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N48" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O48" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P48" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J48" s="51"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="51" t="s">
@@ -16423,45 +15547,25 @@
       <c r="C49" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="52" t="n">
-        <f aca="false">'Market Comparison'!D50</f>
+      <c r="D49" s="56" t="n">
         <v>5.35</v>
       </c>
       <c r="E49" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="F49" s="52" t="n">
+        <v>329</v>
+      </c>
+      <c r="F49" s="53" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="G49" s="53" t="n">
+      <c r="G49" s="54" t="n">
         <v>4.00454545454545</v>
       </c>
-      <c r="H49" s="54" t="n">
+      <c r="H49" s="55" t="n">
         <v>0.748513169073916</v>
       </c>
       <c r="I49" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J49" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F50="","",'Market Comparison'!F50)</f>
-        <v/>
-      </c>
-      <c r="K49" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L49" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M49" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N49" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O49" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P49" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J49" s="51"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="51" t="s">
@@ -16473,45 +15577,25 @@
       <c r="C50" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="52" t="n">
-        <f aca="false">'Market Comparison'!D51</f>
+      <c r="D50" s="56" t="n">
         <v>2.67</v>
       </c>
       <c r="E50" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F50" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F50" s="53" t="n">
         <v>25.4454545454545</v>
       </c>
-      <c r="G50" s="53" t="n">
+      <c r="G50" s="54" t="n">
         <v>22.7754545454545</v>
       </c>
-      <c r="H50" s="54" t="n">
+      <c r="H50" s="55" t="n">
         <v>8.53013278855974</v>
       </c>
       <c r="I50" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J50" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F51="","",'Market Comparison'!F51)</f>
-        <v/>
-      </c>
-      <c r="K50" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L50" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M50" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N50" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O50" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P50" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J50" s="51"/>
     </row>
     <row r="51" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="51" t="s">
@@ -16523,45 +15607,25 @@
       <c r="C51" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="D51" s="52" t="n">
-        <f aca="false">'Market Comparison'!D52</f>
+      <c r="D51" s="56" t="n">
         <v>9.5</v>
       </c>
       <c r="E51" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F51" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F51" s="53" t="n">
         <v>40.9</v>
       </c>
-      <c r="G51" s="53" t="n">
+      <c r="G51" s="54" t="n">
         <v>31.4</v>
       </c>
-      <c r="H51" s="54" t="n">
+      <c r="H51" s="55" t="n">
         <v>3.30526315789474</v>
       </c>
       <c r="I51" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J51" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F52="","",'Market Comparison'!F52)</f>
-        <v/>
-      </c>
-      <c r="K51" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L51" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M51" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N51" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O51" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P51" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J51" s="51"/>
     </row>
     <row r="52" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="51" t="s">
@@ -16573,45 +15637,25 @@
       <c r="C52" s="41" t="s">
         <v>122</v>
       </c>
-      <c r="D52" s="52" t="n">
-        <f aca="false">'Market Comparison'!D53</f>
+      <c r="D52" s="56" t="n">
         <v>2</v>
       </c>
       <c r="E52" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="F52" s="52" t="n">
+        <v>325</v>
+      </c>
+      <c r="F52" s="53" t="n">
         <v>7.81818181818182</v>
       </c>
-      <c r="G52" s="53" t="n">
+      <c r="G52" s="54" t="n">
         <v>5.81818181818182</v>
       </c>
-      <c r="H52" s="54" t="n">
+      <c r="H52" s="55" t="n">
         <v>2.90909090909091</v>
       </c>
       <c r="I52" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J52" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F53="","",'Market Comparison'!F53)</f>
-        <v/>
-      </c>
-      <c r="K52" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L52" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M52" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N52" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O52" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P52" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J52" s="51"/>
     </row>
     <row r="53" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="51" t="s">
@@ -16623,45 +15667,25 @@
       <c r="C53" s="41" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="52" t="n">
-        <f aca="false">'Market Comparison'!D54</f>
+      <c r="D53" s="56" t="n">
         <v>2.67</v>
       </c>
       <c r="E53" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F53" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F53" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G53" s="53" t="n">
+      <c r="G53" s="54" t="n">
         <v>27.3209090909091</v>
       </c>
-      <c r="H53" s="54" t="n">
+      <c r="H53" s="55" t="n">
         <v>10.2325502213143</v>
       </c>
       <c r="I53" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J53" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F54="","",'Market Comparison'!F54)</f>
-        <v/>
-      </c>
-      <c r="K53" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L53" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M53" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N53" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O53" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P53" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J53" s="51"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="51" t="s">
@@ -16673,45 +15697,25 @@
       <c r="C54" s="41" t="s">
         <v>126</v>
       </c>
-      <c r="D54" s="52" t="n">
-        <f aca="false">'Market Comparison'!D55</f>
+      <c r="D54" s="56" t="n">
         <v>4.01</v>
       </c>
       <c r="E54" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F54" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F54" s="53" t="n">
         <v>34.5363636363636</v>
       </c>
-      <c r="G54" s="53" t="n">
+      <c r="G54" s="54" t="n">
         <v>30.5263636363636</v>
       </c>
-      <c r="H54" s="54" t="n">
+      <c r="H54" s="55" t="n">
         <v>7.61255951031511</v>
       </c>
       <c r="I54" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J54" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F55="","",'Market Comparison'!F55)</f>
-        <v/>
-      </c>
-      <c r="K54" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L54" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M54" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N54" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O54" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P54" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J54" s="51"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="51" t="s">
@@ -16723,45 +15727,25 @@
       <c r="C55" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="D55" s="52" t="n">
-        <f aca="false">'Market Comparison'!D56</f>
+      <c r="D55" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E55" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F55" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F55" s="53" t="n">
         <v>34.5363636363636</v>
       </c>
-      <c r="G55" s="53" t="n">
+      <c r="G55" s="54" t="n">
         <v>23.8463636363636</v>
       </c>
-      <c r="H55" s="54" t="n">
+      <c r="H55" s="55" t="n">
         <v>2.23071689769538</v>
       </c>
       <c r="I55" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J55" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F56="","",'Market Comparison'!F56)</f>
-        <v/>
-      </c>
-      <c r="K55" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L55" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M55" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N55" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O55" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P55" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J55" s="51"/>
     </row>
     <row r="56" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="51" t="s">
@@ -16773,45 +15757,25 @@
       <c r="C56" s="41" t="s">
         <v>134</v>
       </c>
-      <c r="D56" s="52" t="n">
-        <f aca="false">'Market Comparison'!D57</f>
+      <c r="D56" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E56" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F56" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F56" s="53" t="n">
         <v>34.5363636363636</v>
       </c>
-      <c r="G56" s="53" t="n">
+      <c r="G56" s="54" t="n">
         <v>23.8463636363636</v>
       </c>
-      <c r="H56" s="54" t="n">
+      <c r="H56" s="55" t="n">
         <v>2.23071689769538</v>
       </c>
       <c r="I56" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J56" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F57="","",'Market Comparison'!F57)</f>
-        <v/>
-      </c>
-      <c r="K56" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L56" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M56" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N56" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O56" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P56" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J56" s="51"/>
     </row>
     <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="51" t="s">
@@ -16823,45 +15787,25 @@
       <c r="C57" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="D57" s="52" t="n">
-        <f aca="false">'Market Comparison'!D58</f>
+      <c r="D57" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E57" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F57" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F57" s="53" t="n">
         <v>40.9</v>
       </c>
-      <c r="G57" s="53" t="n">
+      <c r="G57" s="54" t="n">
         <v>30.21</v>
       </c>
-      <c r="H57" s="54" t="n">
+      <c r="H57" s="55" t="n">
         <v>2.82600561272217</v>
       </c>
       <c r="I57" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J57" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F58="","",'Market Comparison'!F58)</f>
-        <v/>
-      </c>
-      <c r="K57" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L57" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M57" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N57" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O57" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P57" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J57" s="51"/>
     </row>
     <row r="58" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="51" t="s">
@@ -16873,45 +15817,25 @@
       <c r="C58" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="D58" s="52" t="n">
-        <f aca="false">'Market Comparison'!D59</f>
+      <c r="D58" s="56" t="n">
         <v>2.89</v>
       </c>
       <c r="E58" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F58" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F58" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G58" s="53" t="n">
+      <c r="G58" s="54" t="n">
         <v>27.1009090909091</v>
       </c>
-      <c r="H58" s="54" t="n">
+      <c r="H58" s="55" t="n">
         <v>9.37747719408619</v>
       </c>
       <c r="I58" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J58" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F59="","",'Market Comparison'!F59)</f>
-        <v/>
-      </c>
-      <c r="K58" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L58" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M58" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N58" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O58" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P58" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J58" s="51"/>
     </row>
     <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="51" t="s">
@@ -16923,45 +15847,25 @@
       <c r="C59" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="D59" s="52" t="n">
-        <f aca="false">'Market Comparison'!D60</f>
+      <c r="D59" s="56" t="n">
         <v>1.94</v>
       </c>
       <c r="E59" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F59" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F59" s="53" t="n">
         <v>45.4454545454545</v>
       </c>
-      <c r="G59" s="53" t="n">
+      <c r="G59" s="54" t="n">
         <v>43.5054545454545</v>
       </c>
-      <c r="H59" s="54" t="n">
+      <c r="H59" s="55" t="n">
         <v>22.4254920337394</v>
       </c>
       <c r="I59" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J59" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F60="","",'Market Comparison'!F60)</f>
-        <v/>
-      </c>
-      <c r="K59" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L59" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M59" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N59" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O59" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P59" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J59" s="51"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="51" t="s">
@@ -16973,45 +15877,25 @@
       <c r="C60" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="D60" s="52" t="n">
-        <f aca="false">'Market Comparison'!D61</f>
+      <c r="D60" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E60" s="51" t="s">
-        <v>325</v>
-      </c>
-      <c r="F60" s="52" t="n">
+        <v>322</v>
+      </c>
+      <c r="F60" s="53" t="n">
         <v>43.55</v>
       </c>
-      <c r="G60" s="53" t="n">
+      <c r="G60" s="54" t="n">
         <v>32.86</v>
       </c>
-      <c r="H60" s="54" t="n">
+      <c r="H60" s="55" t="n">
         <v>3.07390084190833</v>
       </c>
       <c r="I60" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J60" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F61="","",'Market Comparison'!F61)</f>
-        <v/>
-      </c>
-      <c r="K60" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L60" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M60" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N60" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O60" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P60" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J60" s="51"/>
     </row>
     <row r="61" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="51" t="s">
@@ -17023,45 +15907,25 @@
       <c r="C61" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="D61" s="52" t="n">
-        <f aca="false">'Market Comparison'!D62</f>
+      <c r="D61" s="56" t="n">
         <v>3.201</v>
       </c>
       <c r="E61" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F61" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F61" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G61" s="53" t="n">
+      <c r="G61" s="54" t="n">
         <v>26.7899090909091</v>
       </c>
-      <c r="H61" s="54" t="n">
+      <c r="H61" s="55" t="n">
         <v>8.36923120615717</v>
       </c>
       <c r="I61" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J61" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F62="","",'Market Comparison'!F62)</f>
-        <v/>
-      </c>
-      <c r="K61" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L61" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M61" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N61" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O61" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P61" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J61" s="51"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="51" t="s">
@@ -17073,45 +15937,25 @@
       <c r="C62" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="D62" s="52" t="n">
-        <f aca="false">'Market Comparison'!D63</f>
+      <c r="D62" s="56" t="n">
         <v>5.35</v>
       </c>
       <c r="E62" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F62" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F62" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G62" s="53" t="n">
+      <c r="G62" s="54" t="n">
         <v>24.6409090909091</v>
       </c>
-      <c r="H62" s="54" t="n">
+      <c r="H62" s="55" t="n">
         <v>4.60577740016993</v>
       </c>
       <c r="I62" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J62" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F63="","",'Market Comparison'!F63)</f>
-        <v/>
-      </c>
-      <c r="K62" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L62" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M62" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N62" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O62" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P62" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J62" s="51"/>
     </row>
     <row r="63" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="51" t="s">
@@ -17123,45 +15967,25 @@
       <c r="C63" s="41" t="s">
         <v>162</v>
       </c>
-      <c r="D63" s="52" t="n">
-        <f aca="false">'Market Comparison'!D64</f>
+      <c r="D63" s="56" t="n">
         <v>2.67</v>
       </c>
       <c r="E63" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F63" s="52" t="n">
+        <v>321</v>
+      </c>
+      <c r="F63" s="53" t="n">
         <v>29.9909090909091</v>
       </c>
-      <c r="G63" s="53" t="n">
+      <c r="G63" s="54" t="n">
         <v>27.3209090909091</v>
       </c>
-      <c r="H63" s="54" t="n">
+      <c r="H63" s="55" t="n">
         <v>10.2325502213143</v>
       </c>
       <c r="I63" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J63" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F64="","",'Market Comparison'!F64)</f>
-        <v/>
-      </c>
-      <c r="K63" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L63" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M63" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N63" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O63" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P63" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J63" s="51"/>
     </row>
     <row r="64" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="51" t="s">
@@ -17173,65 +15997,39 @@
       <c r="C64" s="41" t="s">
         <v>164</v>
       </c>
-      <c r="D64" s="52" t="n">
-        <f aca="false">'Market Comparison'!D65</f>
+      <c r="D64" s="56" t="n">
         <v>10.69</v>
       </c>
       <c r="E64" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="F64" s="52" t="n">
+        <v>330</v>
+      </c>
+      <c r="F64" s="53" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="G64" s="53" t="n">
+      <c r="G64" s="54" t="n">
         <v>16.5827272727273</v>
       </c>
-      <c r="H64" s="54" t="n">
+      <c r="H64" s="55" t="n">
         <v>1.55123735011481</v>
       </c>
       <c r="I64" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="J64" s="52" t="str">
-        <f aca="false">IF('Market Comparison'!F65="","",'Market Comparison'!F65)</f>
-        <v/>
-      </c>
-      <c r="K64" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="L64" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="M64" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="N64" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="O64" s="51" t="s">
-        <v>257</v>
-      </c>
-      <c r="P64" s="41"/>
+        <v>320</v>
+      </c>
+      <c r="J64" s="51"/>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="58" t="s">
-        <v>334</v>
-      </c>
-      <c r="B66" s="58"/>
-      <c r="C66" s="58"/>
-      <c r="D66" s="58"/>
-      <c r="E66" s="58"/>
-      <c r="F66" s="58"/>
-      <c r="G66" s="58"/>
-      <c r="H66" s="58"/>
-      <c r="I66" s="58"/>
-      <c r="J66" s="58"/>
-      <c r="K66" s="58"/>
-      <c r="L66" s="58"/>
-      <c r="M66" s="58"/>
-      <c r="N66" s="58"/>
-      <c r="O66" s="58"/>
-      <c r="P66" s="58"/>
+      <c r="A66" s="64" t="s">
+        <v>331</v>
+      </c>
+      <c r="B66" s="64"/>
+      <c r="C66" s="64"/>
+      <c r="D66" s="64"/>
+      <c r="E66" s="64"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="64"/>
+      <c r="H66" s="64"/>
+      <c r="I66" s="64"/>
+      <c r="J66" s="64"/>
     </row>
     <row r="67" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="50" t="s">
@@ -17241,392 +16039,187 @@
         <v>1</v>
       </c>
       <c r="C67" s="50" t="s">
+        <v>332</v>
+      </c>
+      <c r="D67" s="50" t="s">
+        <v>333</v>
+      </c>
+      <c r="E67" s="50" t="s">
+        <v>334</v>
+      </c>
+      <c r="F67" s="50" t="s">
         <v>335</v>
       </c>
-      <c r="D67" s="50" t="s">
+      <c r="G67" s="50" t="s">
         <v>336</v>
       </c>
-      <c r="E67" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="F67" s="50" t="s">
-        <v>338</v>
-      </c>
-      <c r="G67" s="50" t="s">
-        <v>339</v>
-      </c>
     </row>
     <row r="68" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="51" t="s">
+      <c r="A68" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="B68" s="41" t="s">
+      <c r="B68" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C68" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D68" s="52" t="n">
+      <c r="C68" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="D68" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E68" s="52" t="n">
-        <v>16.71</v>
-      </c>
-      <c r="F68" s="53" t="n">
-        <v>7.35545454545455</v>
-      </c>
-      <c r="G68" s="54" t="n">
-        <v>0.440182797453893</v>
+      <c r="E68" s="60" t="n">
+        <v>16.93275</v>
+      </c>
+      <c r="F68" s="65" t="n">
+        <v>7.57820454545455</v>
+      </c>
+      <c r="G68" s="66" t="n">
+        <v>0.447547181967167</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="51" t="s">
+      <c r="A69" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="B69" s="41" t="s">
+      <c r="B69" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D69" s="52" t="n">
+      <c r="C69" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="D69" s="60" t="n">
         <v>21.2</v>
       </c>
-      <c r="E69" s="52" t="n">
-        <v>33.41</v>
-      </c>
-      <c r="F69" s="53" t="n">
-        <v>12.21</v>
-      </c>
-      <c r="G69" s="54" t="n">
-        <v>0.365459443280455</v>
+      <c r="E69" s="60" t="n">
+        <v>33.8555</v>
+      </c>
+      <c r="F69" s="65" t="n">
+        <v>12.6555</v>
+      </c>
+      <c r="G69" s="66" t="n">
+        <v>0.373809277665372</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="51" t="s">
+      <c r="A70" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="B70" s="41" t="s">
+      <c r="B70" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D70" s="52" t="n">
+      <c r="C70" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="D70" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E70" s="52" t="n">
-        <v>11.81</v>
-      </c>
-      <c r="F70" s="53" t="n">
-        <v>2.45545454545455</v>
-      </c>
-      <c r="G70" s="54" t="n">
-        <v>0.207913170656609</v>
+      <c r="E70" s="60" t="n">
+        <v>12.03275</v>
+      </c>
+      <c r="F70" s="65" t="n">
+        <v>2.67820454545455</v>
+      </c>
+      <c r="G70" s="66" t="n">
+        <v>0.222576264399622</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="51" t="s">
+      <c r="A71" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="B71" s="41" t="s">
+      <c r="B71" s="58" t="s">
         <v>172</v>
       </c>
-      <c r="C71" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D71" s="52" t="n">
+      <c r="C71" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="D71" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E71" s="52" t="n">
-        <v>11.81</v>
-      </c>
-      <c r="F71" s="53" t="n">
-        <v>2.45545454545455</v>
-      </c>
-      <c r="G71" s="54" t="n">
-        <v>0.207913170656609</v>
+      <c r="E71" s="60" t="n">
+        <v>12.03275</v>
+      </c>
+      <c r="F71" s="65" t="n">
+        <v>2.67820454545455</v>
+      </c>
+      <c r="G71" s="66" t="n">
+        <v>0.222576264399622</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="51" t="s">
+      <c r="A72" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="B72" s="41" t="s">
+      <c r="B72" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="C72" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="D72" s="52" t="n">
+      <c r="C72" s="57" t="s">
+        <v>327</v>
+      </c>
+      <c r="D72" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E72" s="52" t="n">
-        <v>33.41</v>
-      </c>
-      <c r="F72" s="53" t="n">
-        <v>5.0554545454545</v>
-      </c>
-      <c r="G72" s="54" t="n">
-        <v>0.151315610459578</v>
+      <c r="E72" s="60" t="n">
+        <v>33.8555</v>
+      </c>
+      <c r="F72" s="65" t="n">
+        <v>5.5009545454545</v>
+      </c>
+      <c r="G72" s="66" t="n">
+        <v>0.162483334922081</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="51" t="s">
+      <c r="A73" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="B73" s="41" t="s">
+      <c r="B73" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="C73" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="D73" s="52" t="n">
+      <c r="C73" s="57" t="s">
+        <v>327</v>
+      </c>
+      <c r="D73" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E73" s="52" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="F73" s="53" t="n">
-        <v>1.3454545454545</v>
-      </c>
-      <c r="G73" s="54" t="n">
-        <v>0.0453014998469528</v>
+      <c r="E73" s="60" t="n">
+        <v>30.1455</v>
+      </c>
+      <c r="F73" s="65" t="n">
+        <v>1.7909545454545</v>
+      </c>
+      <c r="G73" s="66" t="n">
+        <v>0.0594103446768007</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="51" t="s">
+      <c r="A74" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="B74" s="41" t="s">
+      <c r="B74" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="C74" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="D74" s="52" t="n">
+      <c r="C74" s="57" t="s">
+        <v>325</v>
+      </c>
+      <c r="D74" s="60" t="n">
         <v>32.5</v>
       </c>
-      <c r="E74" s="52" t="n">
-        <v>33.41</v>
-      </c>
-      <c r="F74" s="53" t="n">
-        <v>0.909999999999997</v>
-      </c>
-      <c r="G74" s="54" t="n">
-        <v>0.027237354085603</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="58" t="s">
-        <v>340</v>
-      </c>
-      <c r="B76" s="58"/>
-      <c r="C76" s="58"/>
-      <c r="D76" s="58"/>
-      <c r="E76" s="58"/>
-      <c r="F76" s="58"/>
-      <c r="G76" s="58"/>
-      <c r="H76" s="58"/>
-      <c r="I76" s="58"/>
-      <c r="J76" s="58"/>
-      <c r="K76" s="58"/>
-      <c r="L76" s="58"/>
-      <c r="M76" s="58"/>
-      <c r="N76" s="58"/>
-      <c r="O76" s="58"/>
-      <c r="P76" s="58"/>
-    </row>
-    <row r="77" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="B77" s="50" t="s">
-        <v>1</v>
-      </c>
-      <c r="C77" s="50" t="s">
-        <v>335</v>
-      </c>
-      <c r="D77" s="50" t="s">
-        <v>336</v>
-      </c>
-      <c r="E77" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="F77" s="50" t="s">
-        <v>338</v>
-      </c>
-      <c r="G77" s="50" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="B78" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="C78" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D78" s="52" t="n">
-        <v>9.35454545454545</v>
-      </c>
-      <c r="E78" s="52" t="n">
-        <v>16.93275</v>
-      </c>
-      <c r="F78" s="53" t="n">
-        <v>7.57820454545455</v>
-      </c>
-      <c r="G78" s="54" t="n">
-        <v>0.447547181967167</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="51" t="s">
-        <v>141</v>
-      </c>
-      <c r="B79" s="41" t="s">
-        <v>142</v>
-      </c>
-      <c r="C79" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D79" s="52" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="E79" s="52" t="n">
+      <c r="E74" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F79" s="53" t="n">
-        <v>12.6555</v>
-      </c>
-      <c r="G79" s="54" t="n">
-        <v>0.373809277665372</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="51" t="s">
-        <v>159</v>
-      </c>
-      <c r="B80" s="41" t="s">
-        <v>160</v>
-      </c>
-      <c r="C80" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D80" s="52" t="n">
-        <v>9.35454545454545</v>
-      </c>
-      <c r="E80" s="52" t="n">
-        <v>12.03275</v>
-      </c>
-      <c r="F80" s="53" t="n">
-        <v>2.67820454545455</v>
-      </c>
-      <c r="G80" s="54" t="n">
-        <v>0.222576264399622</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="51" t="s">
-        <v>171</v>
-      </c>
-      <c r="B81" s="41" t="s">
-        <v>172</v>
-      </c>
-      <c r="C81" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="D81" s="52" t="n">
-        <v>9.35454545454545</v>
-      </c>
-      <c r="E81" s="52" t="n">
-        <v>12.03275</v>
-      </c>
-      <c r="F81" s="53" t="n">
-        <v>2.67820454545455</v>
-      </c>
-      <c r="G81" s="54" t="n">
-        <v>0.222576264399622</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="51" t="s">
-        <v>79</v>
-      </c>
-      <c r="B82" s="41" t="s">
-        <v>80</v>
-      </c>
-      <c r="C82" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="D82" s="52" t="n">
-        <v>28.3545454545455</v>
-      </c>
-      <c r="E82" s="52" t="n">
-        <v>33.8555</v>
-      </c>
-      <c r="F82" s="53" t="n">
-        <v>5.5009545454545</v>
-      </c>
-      <c r="G82" s="54" t="n">
-        <v>0.162483334922081</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="51" t="s">
-        <v>131</v>
-      </c>
-      <c r="B83" s="41" t="s">
-        <v>132</v>
-      </c>
-      <c r="C83" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="D83" s="52" t="n">
-        <v>28.3545454545455</v>
-      </c>
-      <c r="E83" s="52" t="n">
-        <v>30.1455</v>
-      </c>
-      <c r="F83" s="53" t="n">
-        <v>1.7909545454545</v>
-      </c>
-      <c r="G83" s="54" t="n">
-        <v>0.0594103446768007</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="51" t="s">
-        <v>167</v>
-      </c>
-      <c r="B84" s="41" t="s">
-        <v>168</v>
-      </c>
-      <c r="C84" s="51" t="s">
-        <v>328</v>
-      </c>
-      <c r="D84" s="52" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="E84" s="52" t="n">
-        <v>33.8555</v>
-      </c>
-      <c r="F84" s="53" t="n">
+      <c r="F74" s="65" t="n">
         <v>1.3555</v>
       </c>
-      <c r="G84" s="54" t="n">
+      <c r="G74" s="66" t="n">
         <v>0.0400378077417258</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A66:P66"/>
-    <mergeCell ref="A76:P76"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A66:J66"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Rework Summary tab to Us/Them column framing with Us-Them diff convention
- Headers now read Us (Our Quoted Price) and Them (Their Price) adjacently
- $ and % Difference now computed as Us - Them (positive/red = we're more
  expensive, negative/green = we're cheaper), reversing the prior Them-Us
  convention so the color coding reads correctly
- "Are We More Expensive?" flag and amber cheaper-row highlighting updated
  to match the new sign convention

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -996,27 +996,27 @@
     <t xml:space="preserve">Summary — Closest-Priced Competitor &amp; Where We're More Expensive</t>
   </si>
   <si>
-    <t xml:space="preserve">For each of our 60 line items: "Our Quoted Price" below is whichever is HIGHER of our 1200-stock or 1220-stock quoted price (shown in blue bold when the 1220-stock price was the higher/used figure, plain black when the 1200-stock price was used — e.g. for items with no 1220-stock price at all, such as the swing-stand products). Against that price, this sheet shows the competitor (or RSEA) whose ex-GST price is CLOSEST to ours — above or below — with the $ and % gap. Rows shaded amber are ones where that closest competitor (or, in some cases, a different cheaper one — see the call-out list below) is actually cheaper than us. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our Quoted Price
-(ex GST, higher of 1200/1220)</t>
+    <t xml:space="preserve">For each of our 60 line items: "Our Quoted Price" below is whichever is HIGHER of our 1200-stock or 1220-stock quoted price (shown in blue bold when the 1220-stock price was the higher/used figure, plain black when the 1200-stock price was used — e.g. for items with no 1220-stock price at all, such as the swing-stand products). Against that price, this sheet shows the competitor (or RSEA) whose ex-GST price is CLOSEST to ours — above or below — with the $ and % gap. Rows shaded amber are ones where that closest competitor (or, in some cases, a different cheaper one — see the call-out list below) is actually cheaper than us. "$ Difference" and "% Difference" are now expressed as Us − Them: a positive (red) figure means we are MORE expensive than that competitor; a negative (green) figure means we are cheaper. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Us
+(Our Quoted Price, ex GST)</t>
   </si>
   <si>
     <t xml:space="preserve">Closest-Priced
 Competitor (or RSEA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Their Price
-(ex GST)</t>
+    <t xml:space="preserve">Them
+(Their Price, ex GST)</t>
   </si>
   <si>
     <t xml:space="preserve">$ Difference
-(Them − Us)</t>
+(Us − Them)</t>
   </si>
   <si>
     <t xml:space="preserve">% Difference
-(vs Our Price)</t>
+(Us vs Them)</t>
   </si>
   <si>
     <t xml:space="preserve">Are We More
@@ -1233,9 +1233,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
+      <color rgb="FF1B7A4D"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1248,8 +1247,9 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF1B7A4D"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1380,7 +1380,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1633,20 +1633,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1757,9 +1749,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>405360</xdr:colOff>
+      <xdr:colOff>405000</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>261720</xdr:rowOff>
+      <xdr:rowOff>261360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1773,7 +1765,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2193120" cy="2339280"/>
+          <a:ext cx="2192760" cy="2338920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14237,10 +14229,10 @@
         <v>20.05</v>
       </c>
       <c r="G5" s="54" t="n">
-        <v>3.11725</v>
+        <v>-3.11725</v>
       </c>
       <c r="H5" s="55" t="n">
-        <v>0.184095908815757</v>
+        <v>-0.184095908815757</v>
       </c>
       <c r="I5" s="51" t="s">
         <v>320</v>
@@ -14267,10 +14259,10 @@
         <v>122.718181818182</v>
       </c>
       <c r="G6" s="54" t="n">
-        <v>55.888181818182</v>
+        <v>-55.888181818182</v>
       </c>
       <c r="H6" s="55" t="n">
-        <v>0.836273856324735</v>
+        <v>-0.836273856324735</v>
       </c>
       <c r="I6" s="51" t="s">
         <v>320</v>
@@ -14297,10 +14289,10 @@
         <v>128.75</v>
       </c>
       <c r="G7" s="54" t="n">
-        <v>84.2</v>
+        <v>-84.2</v>
       </c>
       <c r="H7" s="55" t="n">
-        <v>1.89001122334456</v>
+        <v>-1.89001122334456</v>
       </c>
       <c r="I7" s="51" t="s">
         <v>320</v>
@@ -14327,10 +14319,10 @@
         <v>69.245</v>
       </c>
       <c r="G8" s="54" t="n">
-        <v>24.101</v>
+        <v>-24.101</v>
       </c>
       <c r="H8" s="55" t="n">
-        <v>0.533869395711501</v>
+        <v>-0.533869395711501</v>
       </c>
       <c r="I8" s="51" t="s">
         <v>320</v>
@@ -14357,10 +14349,10 @@
         <v>81.4</v>
       </c>
       <c r="G9" s="54" t="n">
-        <v>10.861875</v>
+        <v>-10.861875</v>
       </c>
       <c r="H9" s="55" t="n">
-        <v>0.153985876432072</v>
+        <v>-0.153985876432072</v>
       </c>
       <c r="I9" s="51" t="s">
         <v>320</v>
@@ -14387,10 +14379,10 @@
         <v>44.209</v>
       </c>
       <c r="G10" s="54" t="n">
-        <v>10.3535</v>
+        <v>-10.3535</v>
       </c>
       <c r="H10" s="55" t="n">
-        <v>0.305814417155263</v>
+        <v>-0.305814417155263</v>
       </c>
       <c r="I10" s="51" t="s">
         <v>320</v>
@@ -14417,10 +14409,10 @@
         <v>70.36</v>
       </c>
       <c r="G11" s="54" t="n">
-        <v>25.216</v>
+        <v>-25.216</v>
       </c>
       <c r="H11" s="55" t="n">
-        <v>0.558568137515506</v>
+        <v>-0.558568137515506</v>
       </c>
       <c r="I11" s="51" t="s">
         <v>320</v>
@@ -14447,10 +14439,10 @@
         <v>33.1818181818182</v>
       </c>
       <c r="G12" s="61" t="n">
-        <v>-0.673681818181798</v>
+        <v>0.673681818181798</v>
       </c>
       <c r="H12" s="62" t="n">
-        <v>-0.019898740771272</v>
+        <v>0.019898740771272</v>
       </c>
       <c r="I12" s="63" t="s">
         <v>326</v>
@@ -14477,10 +14469,10 @@
         <v>43.09</v>
       </c>
       <c r="G13" s="54" t="n">
-        <v>17.695875</v>
+        <v>-17.695875</v>
       </c>
       <c r="H13" s="55" t="n">
-        <v>0.696849172790951</v>
+        <v>-0.696849172790951</v>
       </c>
       <c r="I13" s="51" t="s">
         <v>320</v>
@@ -14507,10 +14499,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G14" s="54" t="n">
-        <v>21.5295340909091</v>
+        <v>-21.5295340909091</v>
       </c>
       <c r="H14" s="55" t="n">
-        <v>2.54444863759248</v>
+        <v>-2.54444863759248</v>
       </c>
       <c r="I14" s="51" t="s">
         <v>320</v>
@@ -14537,10 +14529,10 @@
         <v>40.9</v>
       </c>
       <c r="G15" s="54" t="n">
-        <v>25.08725</v>
+        <v>-25.08725</v>
       </c>
       <c r="H15" s="55" t="n">
-        <v>1.58652037121943</v>
+        <v>-1.58652037121943</v>
       </c>
       <c r="I15" s="51" t="s">
         <v>320</v>
@@ -14567,10 +14559,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G16" s="54" t="n">
-        <v>21.5295340909091</v>
+        <v>-21.5295340909091</v>
       </c>
       <c r="H16" s="55" t="n">
-        <v>2.54444863759248</v>
+        <v>-2.54444863759248</v>
       </c>
       <c r="I16" s="51" t="s">
         <v>320</v>
@@ -14597,10 +14589,10 @@
         <v>37.3909090909091</v>
       </c>
       <c r="G17" s="54" t="n">
-        <v>7.2454090909091</v>
+        <v>-7.2454090909091</v>
       </c>
       <c r="H17" s="55" t="n">
-        <v>0.240347948811899</v>
+        <v>-0.240347948811899</v>
       </c>
       <c r="I17" s="51" t="s">
         <v>320</v>
@@ -14627,10 +14619,10 @@
         <v>28.3545454545455</v>
       </c>
       <c r="G18" s="61" t="n">
-        <v>-1.7909545454545</v>
+        <v>1.7909545454545</v>
       </c>
       <c r="H18" s="62" t="n">
-        <v>-0.0594103446768007</v>
+        <v>0.0594103446768007</v>
       </c>
       <c r="I18" s="63" t="s">
         <v>326</v>
@@ -14657,10 +14649,10 @@
         <v>23.3090909090909</v>
       </c>
       <c r="G19" s="54" t="n">
-        <v>6.3763409090909</v>
+        <v>-6.3763409090909</v>
       </c>
       <c r="H19" s="55" t="n">
-        <v>0.376568537838857</v>
+        <v>-0.376568537838857</v>
       </c>
       <c r="I19" s="51" t="s">
         <v>320</v>
@@ -14687,10 +14679,10 @@
         <v>28.99</v>
       </c>
       <c r="G20" s="61" t="n">
-        <v>-4.8655</v>
+        <v>4.8655</v>
       </c>
       <c r="H20" s="62" t="n">
-        <v>-0.14371372450562</v>
+        <v>0.14371372450562</v>
       </c>
       <c r="I20" s="63" t="s">
         <v>326</v>
@@ -14717,10 +14709,10 @@
         <v>21.2</v>
       </c>
       <c r="G21" s="54" t="n">
-        <v>9.16725</v>
+        <v>-9.16725</v>
       </c>
       <c r="H21" s="55" t="n">
-        <v>0.761858261827097</v>
+        <v>-0.761858261827097</v>
       </c>
       <c r="I21" s="51" t="s">
         <v>320</v>
@@ -14747,10 +14739,10 @@
         <v>21.2</v>
       </c>
       <c r="G22" s="54" t="n">
-        <v>9.16725</v>
+        <v>-9.16725</v>
       </c>
       <c r="H22" s="55" t="n">
-        <v>0.761858261827097</v>
+        <v>-0.761858261827097</v>
       </c>
       <c r="I22" s="51" t="s">
         <v>320</v>
@@ -14777,10 +14769,10 @@
         <v>34.5363636363636</v>
       </c>
       <c r="G23" s="54" t="n">
-        <v>28.5249886363636</v>
+        <v>-28.5249886363636</v>
       </c>
       <c r="H23" s="55" t="n">
-        <v>4.74516872368861</v>
+        <v>-4.74516872368861</v>
       </c>
       <c r="I23" s="51" t="s">
         <v>320</v>
@@ -14807,10 +14799,10 @@
         <v>9.35454545454545</v>
       </c>
       <c r="G24" s="61" t="n">
-        <v>-2.67820454545455</v>
+        <v>2.67820454545455</v>
       </c>
       <c r="H24" s="62" t="n">
-        <v>-0.222576264399622</v>
+        <v>0.222576264399622</v>
       </c>
       <c r="I24" s="63" t="s">
         <v>326</v>
@@ -14837,10 +14829,10 @@
         <v>9.35454545454545</v>
       </c>
       <c r="G25" s="61" t="n">
-        <v>-2.67820454545455</v>
+        <v>2.67820454545455</v>
       </c>
       <c r="H25" s="62" t="n">
-        <v>-0.222576264399622</v>
+        <v>0.222576264399622</v>
       </c>
       <c r="I25" s="63" t="s">
         <v>326</v>
@@ -14867,10 +14859,10 @@
         <v>21.2</v>
       </c>
       <c r="G26" s="54" t="n">
-        <v>9.16725</v>
+        <v>-9.16725</v>
       </c>
       <c r="H26" s="55" t="n">
-        <v>0.761858261827097</v>
+        <v>-0.761858261827097</v>
       </c>
       <c r="I26" s="51" t="s">
         <v>320</v>
@@ -14897,10 +14889,10 @@
         <v>32.5</v>
       </c>
       <c r="G27" s="61" t="n">
-        <v>-1.3555</v>
+        <v>1.3555</v>
       </c>
       <c r="H27" s="62" t="n">
-        <v>-0.0400378077417258</v>
+        <v>0.0400378077417258</v>
       </c>
       <c r="I27" s="63" t="s">
         <v>326</v>
@@ -14927,10 +14919,10 @@
         <v>45</v>
       </c>
       <c r="G28" s="54" t="n">
-        <v>11.1445</v>
+        <v>-11.1445</v>
       </c>
       <c r="H28" s="55" t="n">
-        <v>0.329178420049918</v>
+        <v>-0.329178420049918</v>
       </c>
       <c r="I28" s="51" t="s">
         <v>320</v>
@@ -14957,10 +14949,10 @@
         <v>30.8</v>
       </c>
       <c r="G29" s="54" t="n">
-        <v>17.73</v>
+        <v>-17.73</v>
       </c>
       <c r="H29" s="55" t="n">
-        <v>1.35654169854629</v>
+        <v>-1.35654169854629</v>
       </c>
       <c r="I29" s="51" t="s">
         <v>320</v>
@@ -14987,10 +14979,10 @@
         <v>31</v>
       </c>
       <c r="G30" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H30" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I30" s="51" t="s">
         <v>320</v>
@@ -15017,10 +15009,10 @@
         <v>31</v>
       </c>
       <c r="G31" s="54" t="n">
-        <v>14.96</v>
+        <v>-14.96</v>
       </c>
       <c r="H31" s="55" t="n">
-        <v>0.932668329177057</v>
+        <v>-0.932668329177057</v>
       </c>
       <c r="I31" s="51" t="s">
         <v>320</v>
@@ -15047,10 +15039,10 @@
         <v>31</v>
       </c>
       <c r="G32" s="54" t="n">
-        <v>14.96</v>
+        <v>-14.96</v>
       </c>
       <c r="H32" s="55" t="n">
-        <v>0.932668329177057</v>
+        <v>-0.932668329177057</v>
       </c>
       <c r="I32" s="51" t="s">
         <v>320</v>
@@ -15077,10 +15069,10 @@
         <v>31</v>
       </c>
       <c r="G33" s="54" t="n">
-        <v>14.96</v>
+        <v>-14.96</v>
       </c>
       <c r="H33" s="55" t="n">
-        <v>0.932668329177057</v>
+        <v>-0.932668329177057</v>
       </c>
       <c r="I33" s="51" t="s">
         <v>320</v>
@@ -15107,10 +15099,10 @@
         <v>31</v>
       </c>
       <c r="G34" s="54" t="n">
-        <v>14.96</v>
+        <v>-14.96</v>
       </c>
       <c r="H34" s="55" t="n">
-        <v>0.932668329177057</v>
+        <v>-0.932668329177057</v>
       </c>
       <c r="I34" s="51" t="s">
         <v>320</v>
@@ -15137,10 +15129,10 @@
         <v>31</v>
       </c>
       <c r="G35" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H35" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I35" s="51" t="s">
         <v>320</v>
@@ -15167,10 +15159,10 @@
         <v>31</v>
       </c>
       <c r="G36" s="54" t="n">
-        <v>14.96</v>
+        <v>-14.96</v>
       </c>
       <c r="H36" s="55" t="n">
-        <v>0.932668329177057</v>
+        <v>-0.932668329177057</v>
       </c>
       <c r="I36" s="51" t="s">
         <v>320</v>
@@ -15197,10 +15189,10 @@
         <v>31</v>
       </c>
       <c r="G37" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H37" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I37" s="51" t="s">
         <v>320</v>
@@ -15227,10 +15219,10 @@
         <v>31</v>
       </c>
       <c r="G38" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H38" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I38" s="51" t="s">
         <v>320</v>
@@ -15257,10 +15249,10 @@
         <v>31</v>
       </c>
       <c r="G39" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H39" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I39" s="51" t="s">
         <v>320</v>
@@ -15287,10 +15279,10 @@
         <v>31</v>
       </c>
       <c r="G40" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H40" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I40" s="51" t="s">
         <v>320</v>
@@ -15317,10 +15309,10 @@
         <v>31</v>
       </c>
       <c r="G41" s="54" t="n">
-        <v>17.93</v>
+        <v>-17.93</v>
       </c>
       <c r="H41" s="55" t="n">
-        <v>1.37184391736802</v>
+        <v>-1.37184391736802</v>
       </c>
       <c r="I41" s="51" t="s">
         <v>320</v>
@@ -15347,10 +15339,10 @@
         <v>34.5363636363636</v>
       </c>
       <c r="G42" s="54" t="n">
-        <v>29.1863636363636</v>
+        <v>-29.1863636363636</v>
       </c>
       <c r="H42" s="55" t="n">
-        <v>5.4553950722175</v>
+        <v>-5.4553950722175</v>
       </c>
       <c r="I42" s="51" t="s">
         <v>320</v>
@@ -15377,10 +15369,10 @@
         <v>9.35454545454545</v>
       </c>
       <c r="G43" s="54" t="n">
-        <v>6.68454545454545</v>
+        <v>-6.68454545454545</v>
       </c>
       <c r="H43" s="55" t="n">
-        <v>2.50357507660878</v>
+        <v>-2.50357507660878</v>
       </c>
       <c r="I43" s="51" t="s">
         <v>320</v>
@@ -15407,10 +15399,10 @@
         <v>23.4090909090909</v>
       </c>
       <c r="G44" s="54" t="n">
-        <v>12.7190909090909</v>
+        <v>-12.7190909090909</v>
       </c>
       <c r="H44" s="55" t="n">
-        <v>1.18981205884854</v>
+        <v>-1.18981205884854</v>
       </c>
       <c r="I44" s="51" t="s">
         <v>320</v>
@@ -15437,10 +15429,10 @@
         <v>22.7181818181818</v>
       </c>
       <c r="G45" s="54" t="n">
-        <v>20.0481818181818</v>
+        <v>-20.0481818181818</v>
       </c>
       <c r="H45" s="55" t="n">
-        <v>7.50868232890704</v>
+        <v>-7.50868232890704</v>
       </c>
       <c r="I45" s="51" t="s">
         <v>320</v>
@@ -15467,10 +15459,10 @@
         <v>40.9</v>
       </c>
       <c r="G46" s="54" t="n">
-        <v>31.4</v>
+        <v>-31.4</v>
       </c>
       <c r="H46" s="55" t="n">
-        <v>3.30526315789474</v>
+        <v>-3.30526315789474</v>
       </c>
       <c r="I46" s="51" t="s">
         <v>320</v>
@@ -15497,10 +15489,10 @@
         <v>40.9</v>
       </c>
       <c r="G47" s="54" t="n">
-        <v>30.21</v>
+        <v>-30.21</v>
       </c>
       <c r="H47" s="55" t="n">
-        <v>2.82600561272217</v>
+        <v>-2.82600561272217</v>
       </c>
       <c r="I47" s="51" t="s">
         <v>320</v>
@@ -15527,10 +15519,10 @@
         <v>20.9090909090909</v>
       </c>
       <c r="G48" s="54" t="n">
-        <v>15.5590909090909</v>
+        <v>-15.5590909090909</v>
       </c>
       <c r="H48" s="55" t="n">
-        <v>2.90824129141886</v>
+        <v>-2.90824129141886</v>
       </c>
       <c r="I48" s="51" t="s">
         <v>320</v>
@@ -15557,10 +15549,10 @@
         <v>9.35454545454545</v>
       </c>
       <c r="G49" s="54" t="n">
-        <v>4.00454545454545</v>
+        <v>-4.00454545454545</v>
       </c>
       <c r="H49" s="55" t="n">
-        <v>0.748513169073916</v>
+        <v>-0.748513169073916</v>
       </c>
       <c r="I49" s="51" t="s">
         <v>320</v>
@@ -15587,10 +15579,10 @@
         <v>25.4454545454545</v>
       </c>
       <c r="G50" s="54" t="n">
-        <v>22.7754545454545</v>
+        <v>-22.7754545454545</v>
       </c>
       <c r="H50" s="55" t="n">
-        <v>8.53013278855974</v>
+        <v>-8.53013278855974</v>
       </c>
       <c r="I50" s="51" t="s">
         <v>320</v>
@@ -15617,10 +15609,10 @@
         <v>40.9</v>
       </c>
       <c r="G51" s="54" t="n">
-        <v>31.4</v>
+        <v>-31.4</v>
       </c>
       <c r="H51" s="55" t="n">
-        <v>3.30526315789474</v>
+        <v>-3.30526315789474</v>
       </c>
       <c r="I51" s="51" t="s">
         <v>320</v>
@@ -15647,10 +15639,10 @@
         <v>7.81818181818182</v>
       </c>
       <c r="G52" s="54" t="n">
-        <v>5.81818181818182</v>
+        <v>-5.81818181818182</v>
       </c>
       <c r="H52" s="55" t="n">
-        <v>2.90909090909091</v>
+        <v>-2.90909090909091</v>
       </c>
       <c r="I52" s="51" t="s">
         <v>320</v>
@@ -15677,10 +15669,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G53" s="54" t="n">
-        <v>27.3209090909091</v>
+        <v>-27.3209090909091</v>
       </c>
       <c r="H53" s="55" t="n">
-        <v>10.2325502213143</v>
+        <v>-10.2325502213143</v>
       </c>
       <c r="I53" s="51" t="s">
         <v>320</v>
@@ -15707,10 +15699,10 @@
         <v>34.5363636363636</v>
       </c>
       <c r="G54" s="54" t="n">
-        <v>30.5263636363636</v>
+        <v>-30.5263636363636</v>
       </c>
       <c r="H54" s="55" t="n">
-        <v>7.61255951031511</v>
+        <v>-7.61255951031511</v>
       </c>
       <c r="I54" s="51" t="s">
         <v>320</v>
@@ -15737,10 +15729,10 @@
         <v>34.5363636363636</v>
       </c>
       <c r="G55" s="54" t="n">
-        <v>23.8463636363636</v>
+        <v>-23.8463636363636</v>
       </c>
       <c r="H55" s="55" t="n">
-        <v>2.23071689769538</v>
+        <v>-2.23071689769538</v>
       </c>
       <c r="I55" s="51" t="s">
         <v>320</v>
@@ -15767,10 +15759,10 @@
         <v>34.5363636363636</v>
       </c>
       <c r="G56" s="54" t="n">
-        <v>23.8463636363636</v>
+        <v>-23.8463636363636</v>
       </c>
       <c r="H56" s="55" t="n">
-        <v>2.23071689769538</v>
+        <v>-2.23071689769538</v>
       </c>
       <c r="I56" s="51" t="s">
         <v>320</v>
@@ -15797,10 +15789,10 @@
         <v>40.9</v>
       </c>
       <c r="G57" s="54" t="n">
-        <v>30.21</v>
+        <v>-30.21</v>
       </c>
       <c r="H57" s="55" t="n">
-        <v>2.82600561272217</v>
+        <v>-2.82600561272217</v>
       </c>
       <c r="I57" s="51" t="s">
         <v>320</v>
@@ -15827,10 +15819,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G58" s="54" t="n">
-        <v>27.1009090909091</v>
+        <v>-27.1009090909091</v>
       </c>
       <c r="H58" s="55" t="n">
-        <v>9.37747719408619</v>
+        <v>-9.37747719408619</v>
       </c>
       <c r="I58" s="51" t="s">
         <v>320</v>
@@ -15857,10 +15849,10 @@
         <v>45.4454545454545</v>
       </c>
       <c r="G59" s="54" t="n">
-        <v>43.5054545454545</v>
+        <v>-43.5054545454545</v>
       </c>
       <c r="H59" s="55" t="n">
-        <v>22.4254920337394</v>
+        <v>-22.4254920337394</v>
       </c>
       <c r="I59" s="51" t="s">
         <v>320</v>
@@ -15887,10 +15879,10 @@
         <v>43.55</v>
       </c>
       <c r="G60" s="54" t="n">
-        <v>32.86</v>
+        <v>-32.86</v>
       </c>
       <c r="H60" s="55" t="n">
-        <v>3.07390084190833</v>
+        <v>-3.07390084190833</v>
       </c>
       <c r="I60" s="51" t="s">
         <v>320</v>
@@ -15917,10 +15909,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G61" s="54" t="n">
-        <v>26.7899090909091</v>
+        <v>-26.7899090909091</v>
       </c>
       <c r="H61" s="55" t="n">
-        <v>8.36923120615717</v>
+        <v>-8.36923120615717</v>
       </c>
       <c r="I61" s="51" t="s">
         <v>320</v>
@@ -15947,10 +15939,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G62" s="54" t="n">
-        <v>24.6409090909091</v>
+        <v>-24.6409090909091</v>
       </c>
       <c r="H62" s="55" t="n">
-        <v>4.60577740016993</v>
+        <v>-4.60577740016993</v>
       </c>
       <c r="I62" s="51" t="s">
         <v>320</v>
@@ -15977,10 +15969,10 @@
         <v>29.9909090909091</v>
       </c>
       <c r="G63" s="54" t="n">
-        <v>27.3209090909091</v>
+        <v>-27.3209090909091</v>
       </c>
       <c r="H63" s="55" t="n">
-        <v>10.2325502213143</v>
+        <v>-10.2325502213143</v>
       </c>
       <c r="I63" s="51" t="s">
         <v>320</v>
@@ -16007,10 +15999,10 @@
         <v>27.2727272727273</v>
       </c>
       <c r="G64" s="54" t="n">
-        <v>16.5827272727273</v>
+        <v>-16.5827272727273</v>
       </c>
       <c r="H64" s="55" t="n">
-        <v>1.55123735011481</v>
+        <v>-1.55123735011481</v>
       </c>
       <c r="I64" s="51" t="s">
         <v>320</v>
@@ -16070,10 +16062,10 @@
       <c r="E68" s="60" t="n">
         <v>16.93275</v>
       </c>
-      <c r="F68" s="65" t="n">
+      <c r="F68" s="61" t="n">
         <v>7.57820454545455</v>
       </c>
-      <c r="G68" s="66" t="n">
+      <c r="G68" s="62" t="n">
         <v>0.447547181967167</v>
       </c>
     </row>
@@ -16093,10 +16085,10 @@
       <c r="E69" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F69" s="65" t="n">
+      <c r="F69" s="61" t="n">
         <v>12.6555</v>
       </c>
-      <c r="G69" s="66" t="n">
+      <c r="G69" s="62" t="n">
         <v>0.373809277665372</v>
       </c>
     </row>
@@ -16116,10 +16108,10 @@
       <c r="E70" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F70" s="65" t="n">
+      <c r="F70" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G70" s="66" t="n">
+      <c r="G70" s="62" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
@@ -16139,10 +16131,10 @@
       <c r="E71" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F71" s="65" t="n">
+      <c r="F71" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G71" s="66" t="n">
+      <c r="G71" s="62" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
@@ -16162,10 +16154,10 @@
       <c r="E72" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F72" s="65" t="n">
+      <c r="F72" s="61" t="n">
         <v>5.5009545454545</v>
       </c>
-      <c r="G72" s="66" t="n">
+      <c r="G72" s="62" t="n">
         <v>0.162483334922081</v>
       </c>
     </row>
@@ -16185,10 +16177,10 @@
       <c r="E73" s="60" t="n">
         <v>30.1455</v>
       </c>
-      <c r="F73" s="65" t="n">
+      <c r="F73" s="61" t="n">
         <v>1.7909545454545</v>
       </c>
-      <c r="G73" s="66" t="n">
+      <c r="G73" s="62" t="n">
         <v>0.0594103446768007</v>
       </c>
     </row>
@@ -16208,10 +16200,10 @@
       <c r="E74" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F74" s="65" t="n">
+      <c r="F74" s="61" t="n">
         <v>1.3555</v>
       </c>
-      <c r="G74" s="66" t="n">
+      <c r="G74" s="62" t="n">
         <v>0.0400378077417258</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorder Summary tab columns to Closest Competitor / Their Price / Our Price
Puts the closest-priced competitor's name and price ahead of our own
price in the main table, keeping the diff/pct math unchanged (Us - Them).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -999,16 +999,16 @@
     <t xml:space="preserve">For each of our 60 line items: "Our Quoted Price" below is whichever is HIGHER of our 1200-stock or 1220-stock quoted price (shown in blue bold when the 1220-stock price was the higher/used figure, plain black when the 1200-stock price was used — e.g. for items with no 1220-stock price at all, such as the swing-stand products). Against that price, this sheet shows the competitor (or RSEA) whose ex-GST price is CLOSEST to ours — above or below — with the $ and % gap. Rows shaded amber are ones where that closest competitor (or, in some cases, a different cheaper one — see the call-out list below) is actually cheaper than us. "$ Difference" and "% Difference" are now expressed as Us − Them: a positive (red) figure means we are MORE expensive than that competitor; a negative (green) figure means we are cheaper. Figures pulled from the 'Market Comparison' tab as of 15 October 2026 — re-run this summary if competitor prices there change. All $ / % figures compare ex-GST prices.</t>
   </si>
   <si>
-    <t xml:space="preserve">Us
-(Our Quoted Price, ex GST)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Closest-Priced
 Competitor (or RSEA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Them
-(Their Price, ex GST)</t>
+    <t xml:space="preserve">Their Price
+(ex GST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Our Price
+(ex GST, higher of 1200/1220)</t>
   </si>
   <si>
     <t xml:space="preserve">$ Difference
@@ -1589,11 +1589,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1617,11 +1617,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1749,9 +1749,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>405000</xdr:colOff>
+      <xdr:colOff>404640</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>261360</xdr:rowOff>
+      <xdr:rowOff>261000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1765,7 +1765,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2192760" cy="2338920"/>
+          <a:ext cx="2192400" cy="2338560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14141,9 +14141,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
@@ -14219,14 +14220,14 @@
       <c r="C5" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="52" t="n">
+      <c r="D5" s="51" t="s">
+        <v>319</v>
+      </c>
+      <c r="E5" s="52" t="n">
+        <v>20.05</v>
+      </c>
+      <c r="F5" s="53" t="n">
         <v>16.93275</v>
-      </c>
-      <c r="E5" s="51" t="s">
-        <v>319</v>
-      </c>
-      <c r="F5" s="53" t="n">
-        <v>20.05</v>
       </c>
       <c r="G5" s="54" t="n">
         <v>-3.11725</v>
@@ -14249,14 +14250,14 @@
       <c r="C6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="56" t="n">
+      <c r="D6" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E6" s="52" t="n">
+        <v>122.718181818182</v>
+      </c>
+      <c r="F6" s="56" t="n">
         <v>66.83</v>
-      </c>
-      <c r="E6" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F6" s="53" t="n">
-        <v>122.718181818182</v>
       </c>
       <c r="G6" s="54" t="n">
         <v>-55.888181818182</v>
@@ -14279,14 +14280,14 @@
       <c r="C7" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="56" t="n">
+      <c r="D7" s="51" t="s">
+        <v>322</v>
+      </c>
+      <c r="E7" s="52" t="n">
+        <v>128.75</v>
+      </c>
+      <c r="F7" s="56" t="n">
         <v>44.55</v>
-      </c>
-      <c r="E7" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="F7" s="53" t="n">
-        <v>128.75</v>
       </c>
       <c r="G7" s="54" t="n">
         <v>-84.2</v>
@@ -14309,14 +14310,14 @@
       <c r="C8" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="52" t="n">
+      <c r="D8" s="51" t="s">
+        <v>323</v>
+      </c>
+      <c r="E8" s="52" t="n">
+        <v>69.245</v>
+      </c>
+      <c r="F8" s="53" t="n">
         <v>45.144</v>
-      </c>
-      <c r="E8" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F8" s="53" t="n">
-        <v>69.245</v>
       </c>
       <c r="G8" s="54" t="n">
         <v>-24.101</v>
@@ -14339,14 +14340,14 @@
       <c r="C9" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="52" t="n">
+      <c r="D9" s="51" t="s">
+        <v>323</v>
+      </c>
+      <c r="E9" s="52" t="n">
+        <v>81.4</v>
+      </c>
+      <c r="F9" s="53" t="n">
         <v>70.538125</v>
-      </c>
-      <c r="E9" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F9" s="53" t="n">
-        <v>81.4</v>
       </c>
       <c r="G9" s="54" t="n">
         <v>-10.861875</v>
@@ -14369,14 +14370,14 @@
       <c r="C10" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="52" t="n">
+      <c r="D10" s="51" t="s">
+        <v>324</v>
+      </c>
+      <c r="E10" s="52" t="n">
+        <v>44.209</v>
+      </c>
+      <c r="F10" s="53" t="n">
         <v>33.8555</v>
-      </c>
-      <c r="E10" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="F10" s="53" t="n">
-        <v>44.209</v>
       </c>
       <c r="G10" s="54" t="n">
         <v>-10.3535</v>
@@ -14399,14 +14400,14 @@
       <c r="C11" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="52" t="n">
+      <c r="D11" s="51" t="s">
+        <v>319</v>
+      </c>
+      <c r="E11" s="52" t="n">
+        <v>70.36</v>
+      </c>
+      <c r="F11" s="53" t="n">
         <v>45.144</v>
-      </c>
-      <c r="E11" s="51" t="s">
-        <v>319</v>
-      </c>
-      <c r="F11" s="53" t="n">
-        <v>70.36</v>
       </c>
       <c r="G11" s="54" t="n">
         <v>-25.216</v>
@@ -14429,14 +14430,14 @@
       <c r="C12" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="59" t="n">
+      <c r="D12" s="57" t="s">
+        <v>325</v>
+      </c>
+      <c r="E12" s="59" t="n">
+        <v>33.1818181818182</v>
+      </c>
+      <c r="F12" s="60" t="n">
         <v>33.8555</v>
-      </c>
-      <c r="E12" s="57" t="s">
-        <v>325</v>
-      </c>
-      <c r="F12" s="60" t="n">
-        <v>33.1818181818182</v>
       </c>
       <c r="G12" s="61" t="n">
         <v>0.673681818181798</v>
@@ -14459,14 +14460,14 @@
       <c r="C13" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="52" t="n">
+      <c r="D13" s="51" t="s">
+        <v>319</v>
+      </c>
+      <c r="E13" s="52" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="F13" s="53" t="n">
         <v>25.394125</v>
-      </c>
-      <c r="E13" s="51" t="s">
-        <v>319</v>
-      </c>
-      <c r="F13" s="53" t="n">
-        <v>43.09</v>
       </c>
       <c r="G13" s="54" t="n">
         <v>-17.695875</v>
@@ -14489,14 +14490,14 @@
       <c r="C14" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="52" t="n">
+      <c r="D14" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E14" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F14" s="53" t="n">
         <v>8.461375</v>
-      </c>
-      <c r="E14" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F14" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G14" s="54" t="n">
         <v>-21.5295340909091</v>
@@ -14519,14 +14520,14 @@
       <c r="C15" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="D15" s="52" t="n">
+      <c r="D15" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E15" s="52" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="F15" s="53" t="n">
         <v>15.81275</v>
-      </c>
-      <c r="E15" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F15" s="53" t="n">
-        <v>40.9</v>
       </c>
       <c r="G15" s="54" t="n">
         <v>-25.08725</v>
@@ -14549,14 +14550,14 @@
       <c r="C16" s="41" t="s">
         <v>118</v>
       </c>
-      <c r="D16" s="52" t="n">
+      <c r="D16" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E16" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F16" s="53" t="n">
         <v>8.461375</v>
-      </c>
-      <c r="E16" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F16" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G16" s="54" t="n">
         <v>-21.5295340909091</v>
@@ -14579,14 +14580,14 @@
       <c r="C17" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="D17" s="52" t="n">
+      <c r="D17" s="51" t="s">
+        <v>327</v>
+      </c>
+      <c r="E17" s="52" t="n">
+        <v>37.3909090909091</v>
+      </c>
+      <c r="F17" s="53" t="n">
         <v>30.1455</v>
-      </c>
-      <c r="E17" s="51" t="s">
-        <v>327</v>
-      </c>
-      <c r="F17" s="53" t="n">
-        <v>37.3909090909091</v>
       </c>
       <c r="G17" s="54" t="n">
         <v>-7.2454090909091</v>
@@ -14609,14 +14610,14 @@
       <c r="C18" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="59" t="n">
+      <c r="D18" s="57" t="s">
+        <v>327</v>
+      </c>
+      <c r="E18" s="59" t="n">
+        <v>28.3545454545455</v>
+      </c>
+      <c r="F18" s="60" t="n">
         <v>30.1455</v>
-      </c>
-      <c r="E18" s="57" t="s">
-        <v>327</v>
-      </c>
-      <c r="F18" s="60" t="n">
-        <v>28.3545454545455</v>
       </c>
       <c r="G18" s="61" t="n">
         <v>1.7909545454545</v>
@@ -14639,14 +14640,14 @@
       <c r="C19" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="D19" s="52" t="n">
+      <c r="D19" s="51" t="s">
+        <v>327</v>
+      </c>
+      <c r="E19" s="52" t="n">
+        <v>23.3090909090909</v>
+      </c>
+      <c r="F19" s="53" t="n">
         <v>16.93275</v>
-      </c>
-      <c r="E19" s="51" t="s">
-        <v>327</v>
-      </c>
-      <c r="F19" s="53" t="n">
-        <v>23.3090909090909</v>
       </c>
       <c r="G19" s="54" t="n">
         <v>-6.3763409090909</v>
@@ -14669,14 +14670,14 @@
       <c r="C20" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="59" t="n">
+      <c r="D20" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="E20" s="59" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F20" s="60" t="n">
         <v>33.8555</v>
-      </c>
-      <c r="E20" s="57" t="s">
-        <v>328</v>
-      </c>
-      <c r="F20" s="60" t="n">
-        <v>28.99</v>
       </c>
       <c r="G20" s="61" t="n">
         <v>4.8655</v>
@@ -14699,14 +14700,14 @@
       <c r="C21" s="41" t="s">
         <v>148</v>
       </c>
-      <c r="D21" s="52" t="n">
+      <c r="D21" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="E21" s="52" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="F21" s="53" t="n">
         <v>12.03275</v>
-      </c>
-      <c r="E21" s="51" t="s">
-        <v>329</v>
-      </c>
-      <c r="F21" s="53" t="n">
-        <v>21.2</v>
       </c>
       <c r="G21" s="54" t="n">
         <v>-9.16725</v>
@@ -14729,14 +14730,14 @@
       <c r="C22" s="41" t="s">
         <v>152</v>
       </c>
-      <c r="D22" s="52" t="n">
+      <c r="D22" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="E22" s="52" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="F22" s="53" t="n">
         <v>12.03275</v>
-      </c>
-      <c r="E22" s="51" t="s">
-        <v>329</v>
-      </c>
-      <c r="F22" s="53" t="n">
-        <v>21.2</v>
       </c>
       <c r="G22" s="54" t="n">
         <v>-9.16725</v>
@@ -14759,14 +14760,14 @@
       <c r="C23" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="D23" s="52" t="n">
+      <c r="D23" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E23" s="52" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="F23" s="53" t="n">
         <v>6.011375</v>
-      </c>
-      <c r="E23" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F23" s="53" t="n">
-        <v>34.5363636363636</v>
       </c>
       <c r="G23" s="54" t="n">
         <v>-28.5249886363636</v>
@@ -14789,14 +14790,14 @@
       <c r="C24" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="D24" s="59" t="n">
+      <c r="D24" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="E24" s="59" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="F24" s="60" t="n">
         <v>12.03275</v>
-      </c>
-      <c r="E24" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="F24" s="60" t="n">
-        <v>9.35454545454545</v>
       </c>
       <c r="G24" s="61" t="n">
         <v>2.67820454545455</v>
@@ -14819,14 +14820,14 @@
       <c r="C25" s="58" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="59" t="n">
+      <c r="D25" s="57" t="s">
+        <v>329</v>
+      </c>
+      <c r="E25" s="59" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="F25" s="60" t="n">
         <v>12.03275</v>
-      </c>
-      <c r="E25" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="F25" s="60" t="n">
-        <v>9.35454545454545</v>
       </c>
       <c r="G25" s="61" t="n">
         <v>2.67820454545455</v>
@@ -14849,14 +14850,14 @@
       <c r="C26" s="41" t="s">
         <v>173</v>
       </c>
-      <c r="D26" s="52" t="n">
+      <c r="D26" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="E26" s="52" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="F26" s="53" t="n">
         <v>12.03275</v>
-      </c>
-      <c r="E26" s="51" t="s">
-        <v>329</v>
-      </c>
-      <c r="F26" s="53" t="n">
-        <v>21.2</v>
       </c>
       <c r="G26" s="54" t="n">
         <v>-9.16725</v>
@@ -14879,14 +14880,14 @@
       <c r="C27" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="D27" s="59" t="n">
+      <c r="D27" s="57" t="s">
+        <v>325</v>
+      </c>
+      <c r="E27" s="59" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="F27" s="60" t="n">
         <v>33.8555</v>
-      </c>
-      <c r="E27" s="57" t="s">
-        <v>325</v>
-      </c>
-      <c r="F27" s="60" t="n">
-        <v>32.5</v>
       </c>
       <c r="G27" s="61" t="n">
         <v>1.3555</v>
@@ -14909,14 +14910,14 @@
       <c r="C28" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="D28" s="52" t="n">
+      <c r="D28" s="51" t="s">
+        <v>325</v>
+      </c>
+      <c r="E28" s="52" t="n">
+        <v>45</v>
+      </c>
+      <c r="F28" s="53" t="n">
         <v>33.8555</v>
-      </c>
-      <c r="E28" s="51" t="s">
-        <v>325</v>
-      </c>
-      <c r="F28" s="53" t="n">
-        <v>45</v>
       </c>
       <c r="G28" s="54" t="n">
         <v>-11.1445</v>
@@ -14939,14 +14940,14 @@
       <c r="C29" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="56" t="n">
+      <c r="D29" s="51" t="s">
+        <v>323</v>
+      </c>
+      <c r="E29" s="52" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F29" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E29" s="51" t="s">
-        <v>323</v>
-      </c>
-      <c r="F29" s="53" t="n">
-        <v>30.8</v>
       </c>
       <c r="G29" s="54" t="n">
         <v>-17.73</v>
@@ -14969,14 +14970,14 @@
       <c r="C30" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="D30" s="56" t="n">
+      <c r="D30" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E30" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F30" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E30" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F30" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G30" s="54" t="n">
         <v>-17.93</v>
@@ -14999,14 +15000,14 @@
       <c r="C31" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="56" t="n">
+      <c r="D31" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E31" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F31" s="56" t="n">
         <v>16.04</v>
-      </c>
-      <c r="E31" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F31" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G31" s="54" t="n">
         <v>-14.96</v>
@@ -15029,14 +15030,14 @@
       <c r="C32" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="56" t="n">
+      <c r="D32" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E32" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F32" s="56" t="n">
         <v>16.04</v>
-      </c>
-      <c r="E32" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F32" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G32" s="54" t="n">
         <v>-14.96</v>
@@ -15059,14 +15060,14 @@
       <c r="C33" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="D33" s="56" t="n">
+      <c r="D33" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E33" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F33" s="56" t="n">
         <v>16.04</v>
-      </c>
-      <c r="E33" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F33" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G33" s="54" t="n">
         <v>-14.96</v>
@@ -15089,14 +15090,14 @@
       <c r="C34" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="D34" s="56" t="n">
+      <c r="D34" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E34" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F34" s="56" t="n">
         <v>16.04</v>
-      </c>
-      <c r="E34" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F34" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G34" s="54" t="n">
         <v>-14.96</v>
@@ -15119,14 +15120,14 @@
       <c r="C35" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="56" t="n">
+      <c r="D35" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E35" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F35" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E35" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F35" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G35" s="54" t="n">
         <v>-17.93</v>
@@ -15149,14 +15150,14 @@
       <c r="C36" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="56" t="n">
+      <c r="D36" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E36" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F36" s="56" t="n">
         <v>16.04</v>
-      </c>
-      <c r="E36" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F36" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G36" s="54" t="n">
         <v>-14.96</v>
@@ -15179,14 +15180,14 @@
       <c r="C37" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="D37" s="56" t="n">
+      <c r="D37" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E37" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F37" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E37" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F37" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G37" s="54" t="n">
         <v>-17.93</v>
@@ -15209,14 +15210,14 @@
       <c r="C38" s="41" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="56" t="n">
+      <c r="D38" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E38" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F38" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E38" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F38" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G38" s="54" t="n">
         <v>-17.93</v>
@@ -15239,14 +15240,14 @@
       <c r="C39" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="D39" s="56" t="n">
+      <c r="D39" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E39" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F39" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E39" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F39" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G39" s="54" t="n">
         <v>-17.93</v>
@@ -15269,14 +15270,14 @@
       <c r="C40" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="D40" s="56" t="n">
+      <c r="D40" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E40" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F40" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E40" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F40" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G40" s="54" t="n">
         <v>-17.93</v>
@@ -15299,14 +15300,14 @@
       <c r="C41" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="D41" s="56" t="n">
+      <c r="D41" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E41" s="52" t="n">
+        <v>31</v>
+      </c>
+      <c r="F41" s="56" t="n">
         <v>13.07</v>
-      </c>
-      <c r="E41" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F41" s="53" t="n">
-        <v>31</v>
       </c>
       <c r="G41" s="54" t="n">
         <v>-17.93</v>
@@ -15329,14 +15330,14 @@
       <c r="C42" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="56" t="n">
+      <c r="D42" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E42" s="52" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="F42" s="56" t="n">
         <v>5.35</v>
-      </c>
-      <c r="E42" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F42" s="53" t="n">
-        <v>34.5363636363636</v>
       </c>
       <c r="G42" s="54" t="n">
         <v>-29.1863636363636</v>
@@ -15359,14 +15360,14 @@
       <c r="C43" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="D43" s="56" t="n">
+      <c r="D43" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="E43" s="52" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="F43" s="56" t="n">
         <v>2.67</v>
-      </c>
-      <c r="E43" s="51" t="s">
-        <v>329</v>
-      </c>
-      <c r="F43" s="53" t="n">
-        <v>9.35454545454545</v>
       </c>
       <c r="G43" s="54" t="n">
         <v>-6.68454545454545</v>
@@ -15389,14 +15390,14 @@
       <c r="C44" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="D44" s="56" t="n">
+      <c r="D44" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E44" s="52" t="n">
+        <v>23.4090909090909</v>
+      </c>
+      <c r="F44" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E44" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F44" s="53" t="n">
-        <v>23.4090909090909</v>
       </c>
       <c r="G44" s="54" t="n">
         <v>-12.7190909090909</v>
@@ -15419,14 +15420,14 @@
       <c r="C45" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="D45" s="56" t="n">
+      <c r="D45" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E45" s="52" t="n">
+        <v>22.7181818181818</v>
+      </c>
+      <c r="F45" s="56" t="n">
         <v>2.67</v>
-      </c>
-      <c r="E45" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F45" s="53" t="n">
-        <v>22.7181818181818</v>
       </c>
       <c r="G45" s="54" t="n">
         <v>-20.0481818181818</v>
@@ -15449,14 +15450,14 @@
       <c r="C46" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="D46" s="56" t="n">
+      <c r="D46" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E46" s="52" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="F46" s="56" t="n">
         <v>9.5</v>
-      </c>
-      <c r="E46" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F46" s="53" t="n">
-        <v>40.9</v>
       </c>
       <c r="G46" s="54" t="n">
         <v>-31.4</v>
@@ -15479,14 +15480,14 @@
       <c r="C47" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="D47" s="56" t="n">
+      <c r="D47" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E47" s="52" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="F47" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E47" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F47" s="53" t="n">
-        <v>40.9</v>
       </c>
       <c r="G47" s="54" t="n">
         <v>-30.21</v>
@@ -15509,14 +15510,14 @@
       <c r="C48" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="D48" s="56" t="n">
+      <c r="D48" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E48" s="52" t="n">
+        <v>20.9090909090909</v>
+      </c>
+      <c r="F48" s="56" t="n">
         <v>5.35</v>
-      </c>
-      <c r="E48" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F48" s="53" t="n">
-        <v>20.9090909090909</v>
       </c>
       <c r="G48" s="54" t="n">
         <v>-15.5590909090909</v>
@@ -15539,14 +15540,14 @@
       <c r="C49" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="56" t="n">
+      <c r="D49" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="E49" s="52" t="n">
+        <v>9.35454545454545</v>
+      </c>
+      <c r="F49" s="56" t="n">
         <v>5.35</v>
-      </c>
-      <c r="E49" s="51" t="s">
-        <v>329</v>
-      </c>
-      <c r="F49" s="53" t="n">
-        <v>9.35454545454545</v>
       </c>
       <c r="G49" s="54" t="n">
         <v>-4.00454545454545</v>
@@ -15569,14 +15570,14 @@
       <c r="C50" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="56" t="n">
+      <c r="D50" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E50" s="52" t="n">
+        <v>25.4454545454545</v>
+      </c>
+      <c r="F50" s="56" t="n">
         <v>2.67</v>
-      </c>
-      <c r="E50" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F50" s="53" t="n">
-        <v>25.4454545454545</v>
       </c>
       <c r="G50" s="54" t="n">
         <v>-22.7754545454545</v>
@@ -15599,14 +15600,14 @@
       <c r="C51" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="D51" s="56" t="n">
+      <c r="D51" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E51" s="52" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="F51" s="56" t="n">
         <v>9.5</v>
-      </c>
-      <c r="E51" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F51" s="53" t="n">
-        <v>40.9</v>
       </c>
       <c r="G51" s="54" t="n">
         <v>-31.4</v>
@@ -15629,14 +15630,14 @@
       <c r="C52" s="41" t="s">
         <v>122</v>
       </c>
-      <c r="D52" s="56" t="n">
+      <c r="D52" s="51" t="s">
+        <v>325</v>
+      </c>
+      <c r="E52" s="52" t="n">
+        <v>7.81818181818182</v>
+      </c>
+      <c r="F52" s="56" t="n">
         <v>2</v>
-      </c>
-      <c r="E52" s="51" t="s">
-        <v>325</v>
-      </c>
-      <c r="F52" s="53" t="n">
-        <v>7.81818181818182</v>
       </c>
       <c r="G52" s="54" t="n">
         <v>-5.81818181818182</v>
@@ -15659,14 +15660,14 @@
       <c r="C53" s="41" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="56" t="n">
+      <c r="D53" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E53" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F53" s="56" t="n">
         <v>2.67</v>
-      </c>
-      <c r="E53" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F53" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G53" s="54" t="n">
         <v>-27.3209090909091</v>
@@ -15689,14 +15690,14 @@
       <c r="C54" s="41" t="s">
         <v>126</v>
       </c>
-      <c r="D54" s="56" t="n">
+      <c r="D54" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E54" s="52" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="F54" s="56" t="n">
         <v>4.01</v>
-      </c>
-      <c r="E54" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F54" s="53" t="n">
-        <v>34.5363636363636</v>
       </c>
       <c r="G54" s="54" t="n">
         <v>-30.5263636363636</v>
@@ -15719,14 +15720,14 @@
       <c r="C55" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="D55" s="56" t="n">
+      <c r="D55" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E55" s="52" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="F55" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E55" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F55" s="53" t="n">
-        <v>34.5363636363636</v>
       </c>
       <c r="G55" s="54" t="n">
         <v>-23.8463636363636</v>
@@ -15749,14 +15750,14 @@
       <c r="C56" s="41" t="s">
         <v>134</v>
       </c>
-      <c r="D56" s="56" t="n">
+      <c r="D56" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E56" s="52" t="n">
+        <v>34.5363636363636</v>
+      </c>
+      <c r="F56" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E56" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F56" s="53" t="n">
-        <v>34.5363636363636</v>
       </c>
       <c r="G56" s="54" t="n">
         <v>-23.8463636363636</v>
@@ -15779,14 +15780,14 @@
       <c r="C57" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="D57" s="56" t="n">
+      <c r="D57" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E57" s="52" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="F57" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E57" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F57" s="53" t="n">
-        <v>40.9</v>
       </c>
       <c r="G57" s="54" t="n">
         <v>-30.21</v>
@@ -15809,14 +15810,14 @@
       <c r="C58" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="D58" s="56" t="n">
+      <c r="D58" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E58" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F58" s="56" t="n">
         <v>2.89</v>
-      </c>
-      <c r="E58" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F58" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G58" s="54" t="n">
         <v>-27.1009090909091</v>
@@ -15839,14 +15840,14 @@
       <c r="C59" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="D59" s="56" t="n">
+      <c r="D59" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E59" s="52" t="n">
+        <v>45.4454545454545</v>
+      </c>
+      <c r="F59" s="56" t="n">
         <v>1.94</v>
-      </c>
-      <c r="E59" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F59" s="53" t="n">
-        <v>45.4454545454545</v>
       </c>
       <c r="G59" s="54" t="n">
         <v>-43.5054545454545</v>
@@ -15869,14 +15870,14 @@
       <c r="C60" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="D60" s="56" t="n">
+      <c r="D60" s="51" t="s">
+        <v>322</v>
+      </c>
+      <c r="E60" s="52" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="F60" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E60" s="51" t="s">
-        <v>322</v>
-      </c>
-      <c r="F60" s="53" t="n">
-        <v>43.55</v>
       </c>
       <c r="G60" s="54" t="n">
         <v>-32.86</v>
@@ -15899,14 +15900,14 @@
       <c r="C61" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="D61" s="56" t="n">
+      <c r="D61" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E61" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F61" s="56" t="n">
         <v>3.201</v>
-      </c>
-      <c r="E61" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F61" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G61" s="54" t="n">
         <v>-26.7899090909091</v>
@@ -15929,14 +15930,14 @@
       <c r="C62" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="D62" s="56" t="n">
+      <c r="D62" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E62" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F62" s="56" t="n">
         <v>5.35</v>
-      </c>
-      <c r="E62" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F62" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G62" s="54" t="n">
         <v>-24.6409090909091</v>
@@ -15959,14 +15960,14 @@
       <c r="C63" s="41" t="s">
         <v>162</v>
       </c>
-      <c r="D63" s="56" t="n">
+      <c r="D63" s="51" t="s">
+        <v>321</v>
+      </c>
+      <c r="E63" s="52" t="n">
+        <v>29.9909090909091</v>
+      </c>
+      <c r="F63" s="56" t="n">
         <v>2.67</v>
-      </c>
-      <c r="E63" s="51" t="s">
-        <v>321</v>
-      </c>
-      <c r="F63" s="53" t="n">
-        <v>29.9909090909091</v>
       </c>
       <c r="G63" s="54" t="n">
         <v>-27.3209090909091</v>
@@ -15989,14 +15990,14 @@
       <c r="C64" s="41" t="s">
         <v>164</v>
       </c>
-      <c r="D64" s="56" t="n">
+      <c r="D64" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="E64" s="52" t="n">
+        <v>27.2727272727273</v>
+      </c>
+      <c r="F64" s="56" t="n">
         <v>10.69</v>
-      </c>
-      <c r="E64" s="51" t="s">
-        <v>330</v>
-      </c>
-      <c r="F64" s="53" t="n">
-        <v>27.2727272727273</v>
       </c>
       <c r="G64" s="54" t="n">
         <v>-16.5827272727273</v>
@@ -16056,10 +16057,10 @@
       <c r="C68" s="57" t="s">
         <v>329</v>
       </c>
-      <c r="D68" s="60" t="n">
+      <c r="D68" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E68" s="60" t="n">
+      <c r="E68" s="59" t="n">
         <v>16.93275</v>
       </c>
       <c r="F68" s="61" t="n">
@@ -16079,10 +16080,10 @@
       <c r="C69" s="57" t="s">
         <v>329</v>
       </c>
-      <c r="D69" s="60" t="n">
+      <c r="D69" s="59" t="n">
         <v>21.2</v>
       </c>
-      <c r="E69" s="60" t="n">
+      <c r="E69" s="59" t="n">
         <v>33.8555</v>
       </c>
       <c r="F69" s="61" t="n">
@@ -16102,10 +16103,10 @@
       <c r="C70" s="57" t="s">
         <v>329</v>
       </c>
-      <c r="D70" s="60" t="n">
+      <c r="D70" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E70" s="60" t="n">
+      <c r="E70" s="59" t="n">
         <v>12.03275</v>
       </c>
       <c r="F70" s="61" t="n">
@@ -16125,10 +16126,10 @@
       <c r="C71" s="57" t="s">
         <v>329</v>
       </c>
-      <c r="D71" s="60" t="n">
+      <c r="D71" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E71" s="60" t="n">
+      <c r="E71" s="59" t="n">
         <v>12.03275</v>
       </c>
       <c r="F71" s="61" t="n">
@@ -16148,10 +16149,10 @@
       <c r="C72" s="57" t="s">
         <v>327</v>
       </c>
-      <c r="D72" s="60" t="n">
+      <c r="D72" s="59" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E72" s="60" t="n">
+      <c r="E72" s="59" t="n">
         <v>33.8555</v>
       </c>
       <c r="F72" s="61" t="n">
@@ -16171,10 +16172,10 @@
       <c r="C73" s="57" t="s">
         <v>327</v>
       </c>
-      <c r="D73" s="60" t="n">
+      <c r="D73" s="59" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E73" s="60" t="n">
+      <c r="E73" s="59" t="n">
         <v>30.1455</v>
       </c>
       <c r="F73" s="61" t="n">
@@ -16194,10 +16195,10 @@
       <c r="C74" s="57" t="s">
         <v>325</v>
       </c>
-      <c r="D74" s="60" t="n">
+      <c r="D74" s="59" t="n">
         <v>32.5</v>
       </c>
-      <c r="E74" s="60" t="n">
+      <c r="E74" s="59" t="n">
         <v>33.8555</v>
       </c>
       <c r="F74" s="61" t="n">

</xml_diff>

<commit_message>
Correct row 16 Advanced Group match to exact size/material
Replaced an approximate self-adhesive-vinyl match (wrong size and
material) with the correct 450x300mm metal "Confined Space Entry By
Permit Only" sign confirmed via the exact product URL ($38.45 inc GST).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -869,7 +869,7 @@
     <t xml:space="preserve">Generic site/warehouse danger sign - no comparable product found at any of the 9 researched retailers (out of scope: these retailers focus on road/traffic signage).</t>
   </si>
   <si>
-    <t xml:space="preserve">No metal-sign equivalent found at the 9 researched retailers for this specific size/material. See RSEA 685265 (Poly, Confined Space Entry By Permit) below for comparable market data.</t>
+    <t xml:space="preserve">Advanced Group: 'Confined Space Entry By Permit Only - Danger Signs - Metal (colorbond steel) - 450 x 300' (832249), $38.45 Inc GST; exact size and material match.</t>
   </si>
   <si>
     <t xml:space="preserve">Generic site/warehouse safety sign - no comparable product found at any of the 9 researched retailers.</t>
@@ -1070,6 +1070,9 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
+    <t xml:space="preserve">Advanced Group</t>
+  </si>
+  <si>
     <t xml:space="preserve">SafetyXpress</t>
   </si>
   <si>
@@ -1080,9 +1083,6 @@
   </si>
   <si>
     <t xml:space="preserve">Safety Signs Australia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advanced Group</t>
   </si>
   <si>
     <t xml:space="preserve">Items We're MORE EXPENSIVE On (our higher-of-1200/1220 quote vs the single cheapest alternative — 7 of 60 items)</t>
@@ -1775,9 +1775,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>403920</xdr:colOff>
+      <xdr:colOff>402480</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>260280</xdr:rowOff>
+      <xdr:rowOff>258840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1791,7 +1791,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2191680" cy="2337840"/>
+          <a:ext cx="2190240" cy="2336400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8800,19 +8800,24 @@
       <c r="AA16" s="45" t="n">
         <v>44.41</v>
       </c>
-      <c r="AB16" s="45"/>
-      <c r="AC16" s="45"/>
+      <c r="AB16" s="45" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="AC16" s="45" t="n">
+        <f aca="false">AB16/1.1</f>
+        <v>34.9545454545455</v>
+      </c>
       <c r="AD16" s="11" t="n">
         <f aca="false">IF(COUNT(I16,J16,M16,O16,Q16,S16,U16,V16,Y16,AA16,AC16)=0,"N/A",MIN(I16,J16,M16,O16,Q16,S16,U16,V16,Y16,AA16,AC16))</f>
-        <v>40.9</v>
+        <v>34.9545454545455</v>
       </c>
       <c r="AE16" s="43" t="n">
         <f aca="false">IF(OR(D16="",AD16="",AD16="N/A"),"N/A",D16/AD16-1)</f>
-        <v>-0.618826405867971</v>
+        <v>-0.553992197659298</v>
       </c>
       <c r="AF16" s="43" t="n">
         <f aca="false">IF(OR(F16="",AD16="",AD16="N/A"),"N/A",F16/AD16-1)</f>
-        <v>-0.613380195599022</v>
+        <v>-0.547619635890767</v>
       </c>
       <c r="AG16" s="41" t="s">
         <v>269</v>
@@ -14255,7 +14260,7 @@
       <c r="C69" s="35"/>
       <c r="D69" s="46" t="n">
         <f aca="false">COUNTIF(J6:J65,"&gt;0")+COUNTIF(M6:M65,"&gt;0")+COUNTIF(O6:O65,"&gt;0")+COUNTIF(Q6:Q65,"&gt;0")+COUNTIF(S6:S65,"&gt;0")+COUNTIF(U6:U65,"&gt;0")+COUNTIF(V6:V65,"&gt;0")+COUNTIF(Y6:Y65,"&gt;0")+COUNTIF(AA6:AA65,"&gt;0")+COUNTIF(AC6:AC65,"&gt;0")</f>
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14288,7 +14293,7 @@
       <c r="C72" s="35"/>
       <c r="D72" s="47" t="n">
         <f aca="false">AVERAGE(AE6:AE65)</f>
-        <v>-0.502826801988701</v>
+        <v>-0.50174623185189</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14332,7 +14337,7 @@
       <c r="C76" s="35"/>
       <c r="D76" s="47" t="n">
         <f aca="false">AVERAGE(AF6:AF65)</f>
-        <v>-0.186068097813109</v>
+        <v>-0.183078981462734</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14763,19 +14768,19 @@
         <v>108</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="E15" s="52" t="n">
-        <v>40.9</v>
+        <v>34.9545454545455</v>
       </c>
       <c r="F15" s="53" t="n">
         <v>15.81275</v>
       </c>
       <c r="G15" s="54" t="n">
-        <v>-25.08725</v>
+        <v>-19.1417954545455</v>
       </c>
       <c r="H15" s="55" t="n">
-        <v>-0.613380195599022</v>
+        <v>-0.547619635890768</v>
       </c>
       <c r="I15" s="51" t="s">
         <v>327</v>
@@ -14823,7 +14828,7 @@
         <v>128</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E17" s="52" t="n">
         <v>37.3909090909091</v>
@@ -14853,7 +14858,7 @@
         <v>132</v>
       </c>
       <c r="D18" s="57" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E18" s="59" t="n">
         <v>28.3545454545455</v>
@@ -14883,7 +14888,7 @@
         <v>138</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E19" s="52" t="n">
         <v>23.3090909090909</v>
@@ -14913,7 +14918,7 @@
         <v>142</v>
       </c>
       <c r="D20" s="57" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E20" s="59" t="n">
         <v>28.99</v>
@@ -14943,7 +14948,7 @@
         <v>148</v>
       </c>
       <c r="D21" s="51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E21" s="52" t="n">
         <v>21.2</v>
@@ -14973,7 +14978,7 @@
         <v>152</v>
       </c>
       <c r="D22" s="51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E22" s="52" t="n">
         <v>21.2</v>
@@ -15033,7 +15038,7 @@
         <v>160</v>
       </c>
       <c r="D24" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E24" s="59" t="n">
         <v>9.35454545454545</v>
@@ -15063,7 +15068,7 @@
         <v>172</v>
       </c>
       <c r="D25" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E25" s="59" t="n">
         <v>9.35454545454545</v>
@@ -15093,7 +15098,7 @@
         <v>173</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E26" s="52" t="n">
         <v>21.2</v>
@@ -15213,7 +15218,7 @@
         <v>52</v>
       </c>
       <c r="D30" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E30" s="52" t="n">
         <v>31</v>
@@ -15243,7 +15248,7 @@
         <v>54</v>
       </c>
       <c r="D31" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E31" s="52" t="n">
         <v>31</v>
@@ -15273,7 +15278,7 @@
         <v>56</v>
       </c>
       <c r="D32" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E32" s="52" t="n">
         <v>31</v>
@@ -15303,7 +15308,7 @@
         <v>58</v>
       </c>
       <c r="D33" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E33" s="52" t="n">
         <v>31</v>
@@ -15333,7 +15338,7 @@
         <v>60</v>
       </c>
       <c r="D34" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E34" s="52" t="n">
         <v>31</v>
@@ -15363,7 +15368,7 @@
         <v>62</v>
       </c>
       <c r="D35" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E35" s="52" t="n">
         <v>31</v>
@@ -15393,7 +15398,7 @@
         <v>64</v>
       </c>
       <c r="D36" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E36" s="52" t="n">
         <v>31</v>
@@ -15423,7 +15428,7 @@
         <v>66</v>
       </c>
       <c r="D37" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E37" s="52" t="n">
         <v>31</v>
@@ -15453,7 +15458,7 @@
         <v>68</v>
       </c>
       <c r="D38" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E38" s="52" t="n">
         <v>31</v>
@@ -15483,7 +15488,7 @@
         <v>70</v>
       </c>
       <c r="D39" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E39" s="52" t="n">
         <v>31</v>
@@ -15513,7 +15518,7 @@
         <v>72</v>
       </c>
       <c r="D40" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E40" s="52" t="n">
         <v>31</v>
@@ -15543,7 +15548,7 @@
         <v>74</v>
       </c>
       <c r="D41" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E41" s="52" t="n">
         <v>31</v>
@@ -15573,7 +15578,7 @@
         <v>5</v>
       </c>
       <c r="D42" s="51" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E42" s="52" t="n">
         <v>32.6363636363636</v>
@@ -15603,7 +15608,7 @@
         <v>96</v>
       </c>
       <c r="D43" s="51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E43" s="52" t="n">
         <v>9.35454545454545</v>
@@ -15633,7 +15638,7 @@
         <v>98</v>
       </c>
       <c r="D44" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E44" s="52" t="n">
         <v>23.4090909090909</v>
@@ -15693,7 +15698,7 @@
         <v>104</v>
       </c>
       <c r="D46" s="51" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E46" s="52" t="n">
         <v>25.5818181818182</v>
@@ -15753,7 +15758,7 @@
         <v>110</v>
       </c>
       <c r="D48" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E48" s="52" t="n">
         <v>20.9090909090909</v>
@@ -15783,7 +15788,7 @@
         <v>112</v>
       </c>
       <c r="D49" s="51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E49" s="52" t="n">
         <v>9.35454545454545</v>
@@ -16023,7 +16028,7 @@
         <v>136</v>
       </c>
       <c r="D57" s="51" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E57" s="52" t="n">
         <v>38.8636363636364</v>
@@ -16203,7 +16208,7 @@
         <v>162</v>
       </c>
       <c r="D63" s="51" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E63" s="52" t="n">
         <v>27.9727272727273</v>
@@ -16233,7 +16238,7 @@
         <v>164</v>
       </c>
       <c r="D64" s="51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E64" s="52" t="n">
         <v>27.2727272727273</v>
@@ -16297,7 +16302,7 @@
         <v>8</v>
       </c>
       <c r="C68" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D68" s="59" t="n">
         <v>9.35454545454545</v>
@@ -16320,7 +16325,7 @@
         <v>142</v>
       </c>
       <c r="C69" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D69" s="59" t="n">
         <v>21.2</v>
@@ -16343,7 +16348,7 @@
         <v>160</v>
       </c>
       <c r="C70" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D70" s="59" t="n">
         <v>9.35454545454545</v>
@@ -16366,7 +16371,7 @@
         <v>172</v>
       </c>
       <c r="C71" s="57" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D71" s="59" t="n">
         <v>9.35454545454545</v>
@@ -16389,7 +16394,7 @@
         <v>80</v>
       </c>
       <c r="C72" s="57" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D72" s="59" t="n">
         <v>28.3545454545455</v>
@@ -16412,7 +16417,7 @@
         <v>132</v>
       </c>
       <c r="C73" s="57" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D73" s="59" t="n">
         <v>28.3545454545455</v>

</xml_diff>

<commit_message>
Format Market Comparison figures as currency; highlight N/A in red
- Every dollar-figure cell (234 were missing it, mostly the prices
  added in the last re-check pass) now uses \$#,##0.00 formatting
- All 370 literal "N/A" cells recolored red
- Added conditional formatting to the Cheapest/vs-Cheapest columns
  so any cell that evaluates to "N/A" turns red automatically, not
  just the ones that currently do

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -1140,15 +1140,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00_);[RED]&quot;($&quot;#,##0.00\)"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1248,13 +1249,21 @@
     <font>
       <i val="true"/>
       <sz val="11"/>
-      <color rgb="FF9B9B9B"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
       <sz val="11"/>
+      <color rgb="FF9B9B9B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1438,7 +1447,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1619,7 +1628,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1631,31 +1648,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1671,23 +1688,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1700,7 +1717,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1723,6 +1740,11 @@
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
     </dxf>
   </dxfs>
   <colors>
@@ -1799,9 +1821,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>401400</xdr:colOff>
+      <xdr:colOff>401040</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>257760</xdr:rowOff>
+      <xdr:rowOff>257400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1815,7 +1837,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2189160" cy="2335320"/>
+          <a:ext cx="2188800" cy="2334960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8684,23 +8706,23 @@
       <c r="M15" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N15" s="42" t="n">
+      <c r="N15" s="46" t="n">
         <v>35.7</v>
       </c>
-      <c r="O15" s="42" t="n">
+      <c r="O15" s="46" t="n">
         <f aca="false">N15/1.1</f>
         <v>32.4545454545455</v>
       </c>
-      <c r="P15" s="42" t="n">
+      <c r="P15" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q15" s="42" t="n">
+      <c r="Q15" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R15" s="42" t="n">
+      <c r="R15" s="46" t="n">
         <v>25</v>
       </c>
-      <c r="S15" s="42" t="n">
+      <c r="S15" s="46" t="n">
         <f aca="false">R15/1.1</f>
         <v>22.7272727272727</v>
       </c>
@@ -8716,10 +8738,10 @@
       <c r="W15" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X15" s="42" t="n">
+      <c r="X15" s="46" t="n">
         <v>35.07</v>
       </c>
-      <c r="Y15" s="42" t="n">
+      <c r="Y15" s="46" t="n">
         <f aca="false">X15/1.1</f>
         <v>31.8818181818182</v>
       </c>
@@ -8793,29 +8815,29 @@
       <c r="K16" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L16" s="42" t="n">
+      <c r="L16" s="46" t="n">
         <v>48.29</v>
       </c>
-      <c r="M16" s="42" t="n">
+      <c r="M16" s="46" t="n">
         <v>43.9</v>
       </c>
-      <c r="N16" s="42" t="n">
+      <c r="N16" s="46" t="n">
         <v>39.95</v>
       </c>
-      <c r="O16" s="42" t="n">
+      <c r="O16" s="46" t="n">
         <f aca="false">N16/1.1</f>
         <v>36.3181818181818</v>
       </c>
-      <c r="P16" s="42" t="n">
+      <c r="P16" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q16" s="42" t="n">
+      <c r="Q16" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R16" s="42" t="n">
+      <c r="R16" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="S16" s="42" t="n">
+      <c r="S16" s="46" t="n">
         <f aca="false">R16/1.1</f>
         <v>25</v>
       </c>
@@ -8825,17 +8847,17 @@
       <c r="U16" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="V16" s="42" t="n">
+      <c r="V16" s="46" t="n">
         <v>21.9</v>
       </c>
-      <c r="W16" s="42" t="n">
+      <c r="W16" s="46" t="n">
         <f aca="false">V16*1.1</f>
         <v>24.09</v>
       </c>
-      <c r="X16" s="42" t="n">
+      <c r="X16" s="46" t="n">
         <v>42.75</v>
       </c>
-      <c r="Y16" s="42" t="n">
+      <c r="Y16" s="46" t="n">
         <f aca="false">X16/1.1</f>
         <v>38.8636363636364</v>
       </c>
@@ -8909,29 +8931,29 @@
       <c r="K17" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L17" s="42" t="n">
+      <c r="L17" s="46" t="n">
         <v>53.63</v>
       </c>
-      <c r="M17" s="42" t="n">
+      <c r="M17" s="46" t="n">
         <v>48.75</v>
       </c>
-      <c r="N17" s="42" t="n">
+      <c r="N17" s="46" t="n">
         <v>35.7</v>
       </c>
-      <c r="O17" s="42" t="n">
+      <c r="O17" s="46" t="n">
         <f aca="false">N17/1.1</f>
         <v>32.4545454545455</v>
       </c>
-      <c r="P17" s="42" t="n">
+      <c r="P17" s="46" t="n">
         <v>11.55</v>
       </c>
-      <c r="Q17" s="42" t="n">
+      <c r="Q17" s="46" t="n">
         <v>10.5</v>
       </c>
-      <c r="R17" s="42" t="n">
+      <c r="R17" s="46" t="n">
         <v>25</v>
       </c>
-      <c r="S17" s="42" t="n">
+      <c r="S17" s="46" t="n">
         <f aca="false">R17/1.1</f>
         <v>22.7272727272727</v>
       </c>
@@ -8947,10 +8969,10 @@
       <c r="W17" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X17" s="42" t="n">
+      <c r="X17" s="46" t="n">
         <v>35.07</v>
       </c>
-      <c r="Y17" s="42" t="n">
+      <c r="Y17" s="46" t="n">
         <f aca="false">X17/1.1</f>
         <v>31.8818181818182</v>
       </c>
@@ -9030,10 +9052,10 @@
       <c r="M18" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N18" s="42" t="n">
+      <c r="N18" s="46" t="n">
         <v>49.5</v>
       </c>
-      <c r="O18" s="42" t="n">
+      <c r="O18" s="46" t="n">
         <f aca="false">N18/1.1</f>
         <v>45</v>
       </c>
@@ -9141,10 +9163,10 @@
       <c r="K19" s="11" t="n">
         <v>99.23</v>
       </c>
-      <c r="L19" s="42" t="n">
+      <c r="L19" s="46" t="n">
         <v>61.59</v>
       </c>
-      <c r="M19" s="42" t="n">
+      <c r="M19" s="46" t="n">
         <v>55.99</v>
       </c>
       <c r="N19" s="11" t="n">
@@ -9394,10 +9416,10 @@
       <c r="Q21" s="11" t="n">
         <v>40.91</v>
       </c>
-      <c r="R21" s="42" t="n">
+      <c r="R21" s="46" t="n">
         <v>37.07</v>
       </c>
-      <c r="S21" s="42" t="n">
+      <c r="S21" s="46" t="n">
         <f aca="false">R21/1.1</f>
         <v>33.7</v>
       </c>
@@ -9723,36 +9745,36 @@
       <c r="K24" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L24" s="42" t="n">
+      <c r="L24" s="46" t="n">
         <v>43.15</v>
       </c>
-      <c r="M24" s="42" t="n">
+      <c r="M24" s="46" t="n">
         <v>39.23</v>
       </c>
-      <c r="N24" s="42" t="n">
+      <c r="N24" s="46" t="n">
         <v>35.75</v>
       </c>
-      <c r="O24" s="42" t="n">
+      <c r="O24" s="46" t="n">
         <f aca="false">N24/1.1</f>
         <v>32.5</v>
       </c>
-      <c r="P24" s="42" t="n">
+      <c r="P24" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q24" s="42" t="n">
+      <c r="Q24" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R24" s="42" t="n">
+      <c r="R24" s="46" t="n">
         <v>25</v>
       </c>
-      <c r="S24" s="42" t="n">
+      <c r="S24" s="46" t="n">
         <f aca="false">R24/1.1</f>
         <v>22.7272727272727</v>
       </c>
-      <c r="T24" s="42" t="n">
+      <c r="T24" s="46" t="n">
         <v>33.19</v>
       </c>
-      <c r="U24" s="42" t="n">
+      <c r="U24" s="46" t="n">
         <f aca="false">T24/1.1</f>
         <v>30.1727272727273</v>
       </c>
@@ -9762,10 +9784,10 @@
       <c r="W24" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X24" s="42" t="n">
+      <c r="X24" s="46" t="n">
         <v>35.9</v>
       </c>
-      <c r="Y24" s="42" t="n">
+      <c r="Y24" s="46" t="n">
         <f aca="false">X24/1.1</f>
         <v>32.6363636363636</v>
       </c>
@@ -9838,10 +9860,10 @@
       <c r="K25" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L25" s="42" t="n">
+      <c r="L25" s="46" t="n">
         <v>46.29</v>
       </c>
-      <c r="M25" s="42" t="n">
+      <c r="M25" s="46" t="n">
         <v>42.08</v>
       </c>
       <c r="N25" s="11" t="n">
@@ -10070,10 +10092,10 @@
       <c r="K27" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L27" s="42" t="n">
+      <c r="L27" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M27" s="42" t="n">
+      <c r="M27" s="46" t="n">
         <v>35.98</v>
       </c>
       <c r="N27" s="11" t="n">
@@ -10238,10 +10260,10 @@
       <c r="AA28" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB28" s="42" t="n">
+      <c r="AB28" s="46" t="n">
         <v>90.08</v>
       </c>
-      <c r="AC28" s="42" t="n">
+      <c r="AC28" s="46" t="n">
         <f aca="false">AB28/1.1</f>
         <v>81.8909090909091</v>
       </c>
@@ -10470,10 +10492,10 @@
       <c r="AA30" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB30" s="42" t="n">
+      <c r="AB30" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC30" s="42" t="n">
+      <c r="AC30" s="46" t="n">
         <f aca="false">AB30/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10565,10 +10587,10 @@
         <f aca="false">T31/1.1</f>
         <v>42.8545454545455</v>
       </c>
-      <c r="V31" s="42" t="n">
+      <c r="V31" s="46" t="n">
         <v>28</v>
       </c>
-      <c r="W31" s="42" t="n">
+      <c r="W31" s="46" t="n">
         <f aca="false">V31*1.1</f>
         <v>30.8</v>
       </c>
@@ -10585,8 +10607,8 @@
       <c r="AA31" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB31" s="42"/>
-      <c r="AC31" s="42"/>
+      <c r="AB31" s="47"/>
+      <c r="AC31" s="47"/>
       <c r="AD31" s="11" t="n">
         <f aca="false">IF(COUNT(I31,J31,M31,O31,Q31,S31,U31,V31,Y31,AA31,AC31)=0,"N/A",MIN(I31,J31,M31,O31,Q31,S31,U31,V31,Y31,AA31,AC31))</f>
         <v>28</v>
@@ -10695,10 +10717,10 @@
       <c r="AA32" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB32" s="42" t="n">
+      <c r="AB32" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC32" s="42" t="n">
+      <c r="AC32" s="46" t="n">
         <f aca="false">AB32/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10765,10 +10787,10 @@
       <c r="M33" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N33" s="42" t="n">
+      <c r="N33" s="46" t="n">
         <v>51</v>
       </c>
-      <c r="O33" s="42" t="n">
+      <c r="O33" s="46" t="n">
         <f aca="false">N33/1.1</f>
         <v>46.3636363636364</v>
       </c>
@@ -10792,10 +10814,10 @@
         <f aca="false">T33/1.1</f>
         <v>53.4909090909091</v>
       </c>
-      <c r="V33" s="42" t="n">
+      <c r="V33" s="46" t="n">
         <v>51.5</v>
       </c>
-      <c r="W33" s="42" t="n">
+      <c r="W33" s="46" t="n">
         <f aca="false">V33*1.1</f>
         <v>56.65</v>
       </c>
@@ -10812,10 +10834,10 @@
       <c r="AA33" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB33" s="42" t="n">
+      <c r="AB33" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC33" s="42" t="n">
+      <c r="AC33" s="46" t="n">
         <f aca="false">AB33/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10928,10 +10950,10 @@
       <c r="AA34" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB34" s="42" t="n">
+      <c r="AB34" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC34" s="42" t="n">
+      <c r="AC34" s="46" t="n">
         <f aca="false">AB34/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11044,10 +11066,10 @@
       <c r="AA35" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB35" s="42" t="n">
+      <c r="AB35" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC35" s="42" t="n">
+      <c r="AC35" s="46" t="n">
         <f aca="false">AB35/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11161,10 +11183,10 @@
       <c r="AA36" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB36" s="42" t="n">
+      <c r="AB36" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC36" s="42" t="n">
+      <c r="AC36" s="46" t="n">
         <f aca="false">AB36/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11275,10 +11297,10 @@
       <c r="AA37" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB37" s="42" t="n">
+      <c r="AB37" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC37" s="42" t="n">
+      <c r="AC37" s="46" t="n">
         <f aca="false">AB37/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11390,10 +11412,10 @@
       <c r="AA38" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB38" s="42" t="n">
+      <c r="AB38" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC38" s="42" t="n">
+      <c r="AC38" s="46" t="n">
         <f aca="false">AB38/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11506,10 +11528,10 @@
       <c r="AA39" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB39" s="42" t="n">
+      <c r="AB39" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC39" s="42" t="n">
+      <c r="AC39" s="46" t="n">
         <f aca="false">AB39/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11622,10 +11644,10 @@
       <c r="AA40" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB40" s="42" t="n">
+      <c r="AB40" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC40" s="42" t="n">
+      <c r="AC40" s="46" t="n">
         <f aca="false">AB40/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11738,10 +11760,10 @@
       <c r="AA41" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB41" s="42" t="n">
+      <c r="AB41" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC41" s="42" t="n">
+      <c r="AC41" s="46" t="n">
         <f aca="false">AB41/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11854,10 +11876,10 @@
       <c r="AA42" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB42" s="42" t="n">
+      <c r="AB42" s="46" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC42" s="42" t="n">
+      <c r="AC42" s="46" t="n">
         <f aca="false">AB42/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11929,16 +11951,16 @@
       <c r="O43" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P43" s="42" t="n">
+      <c r="P43" s="46" t="n">
         <v>22.05</v>
       </c>
-      <c r="Q43" s="42" t="n">
+      <c r="Q43" s="46" t="n">
         <v>20.05</v>
       </c>
-      <c r="R43" s="42" t="n">
+      <c r="R43" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="S43" s="42" t="n">
+      <c r="S43" s="46" t="n">
         <f aca="false">R43/1.1</f>
         <v>25</v>
       </c>
@@ -11954,19 +11976,19 @@
       <c r="W43" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X43" s="42" t="n">
+      <c r="X43" s="46" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y43" s="42" t="n">
+      <c r="Y43" s="46" t="n">
         <f aca="false">X43/1.1</f>
         <v>29.0545454545455</v>
       </c>
-      <c r="Z43" s="42"/>
-      <c r="AA43" s="42"/>
-      <c r="AB43" s="42" t="n">
+      <c r="Z43" s="47"/>
+      <c r="AA43" s="47"/>
+      <c r="AB43" s="46" t="n">
         <v>35.9</v>
       </c>
-      <c r="AC43" s="42" t="n">
+      <c r="AC43" s="46" t="n">
         <f aca="false">AB43/1.1</f>
         <v>32.6363636363636</v>
       </c>
@@ -12045,10 +12067,10 @@
       <c r="Q44" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="R44" s="42" t="n">
+      <c r="R44" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S44" s="42" t="n">
+      <c r="S44" s="46" t="n">
         <f aca="false">R44/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -12181,10 +12203,10 @@
       <c r="W45" s="11" t="n">
         <v>26.5</v>
       </c>
-      <c r="X45" s="42" t="n">
+      <c r="X45" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y45" s="42" t="n">
+      <c r="Y45" s="46" t="n">
         <f aca="false">X45/1.1</f>
         <v>41.6</v>
       </c>
@@ -12258,16 +12280,16 @@
       <c r="K46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L46" s="42" t="n">
+      <c r="L46" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M46" s="42" t="n">
+      <c r="M46" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N46" s="42" t="n">
+      <c r="N46" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="O46" s="42" t="n">
+      <c r="O46" s="46" t="n">
         <f aca="false">N46/1.1</f>
         <v>25</v>
       </c>
@@ -12277,10 +12299,10 @@
       <c r="Q46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R46" s="42" t="n">
+      <c r="R46" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S46" s="42" t="n">
+      <c r="S46" s="46" t="n">
         <f aca="false">R46/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -12296,10 +12318,10 @@
       <c r="W46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X46" s="42" t="n">
+      <c r="X46" s="46" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y46" s="42" t="n">
+      <c r="Y46" s="46" t="n">
         <f aca="false">X46/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -12373,50 +12395,50 @@
       <c r="K47" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L47" s="42" t="n">
+      <c r="L47" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M47" s="42" t="n">
+      <c r="M47" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N47" s="42" t="n">
+      <c r="N47" s="46" t="n">
         <v>42.5</v>
       </c>
-      <c r="O47" s="42" t="n">
+      <c r="O47" s="46" t="n">
         <f aca="false">N47/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P47" s="42" t="n">
+      <c r="P47" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q47" s="42" t="n">
+      <c r="Q47" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R47" s="42" t="n">
+      <c r="R47" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="S47" s="42" t="n">
+      <c r="S47" s="46" t="n">
         <f aca="false">R47/1.1</f>
         <v>27.2727272727273</v>
       </c>
-      <c r="T47" s="42" t="n">
+      <c r="T47" s="46" t="n">
         <v>28.66</v>
       </c>
-      <c r="U47" s="42" t="n">
+      <c r="U47" s="46" t="n">
         <f aca="false">T47/1.1</f>
         <v>26.0545454545455</v>
       </c>
-      <c r="V47" s="42" t="n">
+      <c r="V47" s="46" t="n">
         <v>36.5</v>
       </c>
-      <c r="W47" s="42" t="n">
+      <c r="W47" s="46" t="n">
         <f aca="false">V47*1.1</f>
         <v>40.15</v>
       </c>
-      <c r="X47" s="42" t="n">
+      <c r="X47" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y47" s="42" t="n">
+      <c r="Y47" s="46" t="n">
         <f aca="false">X47/1.1</f>
         <v>41.6</v>
       </c>
@@ -12490,43 +12512,43 @@
       <c r="K48" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L48" s="42" t="n">
+      <c r="L48" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M48" s="42" t="n">
+      <c r="M48" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N48" s="42" t="n">
+      <c r="N48" s="46" t="n">
         <v>42.5</v>
       </c>
-      <c r="O48" s="42" t="n">
+      <c r="O48" s="46" t="n">
         <f aca="false">N48/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P48" s="42" t="n">
+      <c r="P48" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q48" s="42" t="n">
+      <c r="Q48" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R48" s="42" t="n">
+      <c r="R48" s="46" t="n">
         <v>33.5</v>
       </c>
-      <c r="S48" s="42" t="n">
+      <c r="S48" s="46" t="n">
         <f aca="false">R48/1.1</f>
         <v>30.4545454545455</v>
       </c>
-      <c r="T48" s="42" t="n">
+      <c r="T48" s="46" t="n">
         <v>18.41</v>
       </c>
-      <c r="U48" s="42" t="n">
+      <c r="U48" s="46" t="n">
         <f aca="false">T48/1.1</f>
         <v>16.7363636363636</v>
       </c>
-      <c r="V48" s="42" t="n">
+      <c r="V48" s="46" t="n">
         <v>28.5</v>
       </c>
-      <c r="W48" s="42" t="n">
+      <c r="W48" s="46" t="n">
         <f aca="false">V48*1.1</f>
         <v>31.35</v>
       </c>
@@ -12612,17 +12634,17 @@
       <c r="M49" s="11" t="n">
         <v>31.52</v>
       </c>
-      <c r="N49" s="42" t="n">
+      <c r="N49" s="46" t="n">
         <v>35.4</v>
       </c>
-      <c r="O49" s="42" t="n">
+      <c r="O49" s="46" t="n">
         <f aca="false">N49/1.1</f>
         <v>32.1818181818182</v>
       </c>
-      <c r="P49" s="42" t="n">
+      <c r="P49" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q49" s="42" t="n">
+      <c r="Q49" s="46" t="n">
         <v>22</v>
       </c>
       <c r="R49" s="11" t="n">
@@ -12646,10 +12668,10 @@
       <c r="W49" s="11" t="n">
         <v>21.9</v>
       </c>
-      <c r="X49" s="42" t="n">
+      <c r="X49" s="46" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y49" s="42" t="n">
+      <c r="Y49" s="46" t="n">
         <f aca="false">X49/1.1</f>
         <v>29.0545454545455</v>
       </c>
@@ -12840,43 +12862,43 @@
       <c r="K51" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L51" s="42" t="n">
+      <c r="L51" s="46" t="n">
         <v>34.67</v>
       </c>
-      <c r="M51" s="42" t="n">
+      <c r="M51" s="46" t="n">
         <v>31.52</v>
       </c>
-      <c r="N51" s="42" t="n">
+      <c r="N51" s="46" t="n">
         <v>28.3</v>
       </c>
-      <c r="O51" s="42" t="n">
+      <c r="O51" s="46" t="n">
         <f aca="false">N51/1.1</f>
         <v>25.7272727272727</v>
       </c>
-      <c r="P51" s="42" t="n">
+      <c r="P51" s="46" t="n">
         <v>11.55</v>
       </c>
-      <c r="Q51" s="42" t="n">
+      <c r="Q51" s="46" t="n">
         <v>10.5</v>
       </c>
-      <c r="R51" s="42" t="n">
+      <c r="R51" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S51" s="42" t="n">
+      <c r="S51" s="46" t="n">
         <f aca="false">R51/1.1</f>
         <v>20.4545454545455</v>
       </c>
-      <c r="T51" s="42" t="n">
+      <c r="T51" s="46" t="n">
         <v>33.04</v>
       </c>
-      <c r="U51" s="42" t="n">
+      <c r="U51" s="46" t="n">
         <f aca="false">T51/1.1</f>
         <v>30.0363636363636</v>
       </c>
-      <c r="V51" s="42" t="n">
+      <c r="V51" s="46" t="n">
         <v>19.5</v>
       </c>
-      <c r="W51" s="42" t="n">
+      <c r="W51" s="46" t="n">
         <f aca="false">V51*1.1</f>
         <v>21.45</v>
       </c>
@@ -12956,29 +12978,29 @@
       <c r="K52" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L52" s="42" t="n">
+      <c r="L52" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M52" s="42" t="n">
+      <c r="M52" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N52" s="42" t="n">
+      <c r="N52" s="46" t="n">
         <v>42.5</v>
       </c>
-      <c r="O52" s="42" t="n">
+      <c r="O52" s="46" t="n">
         <f aca="false">N52/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P52" s="42" t="n">
+      <c r="P52" s="46" t="n">
         <v>45.15</v>
       </c>
-      <c r="Q52" s="42" t="n">
+      <c r="Q52" s="46" t="n">
         <v>41.05</v>
       </c>
-      <c r="R52" s="42" t="n">
+      <c r="R52" s="46" t="n">
         <v>33.5</v>
       </c>
-      <c r="S52" s="42" t="n">
+      <c r="S52" s="46" t="n">
         <f aca="false">R52/1.1</f>
         <v>30.4545454545455</v>
       </c>
@@ -12988,17 +13010,17 @@
       <c r="U52" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="V52" s="42" t="n">
+      <c r="V52" s="46" t="n">
         <v>26.5</v>
       </c>
-      <c r="W52" s="42" t="n">
+      <c r="W52" s="46" t="n">
         <f aca="false">V52*1.1</f>
         <v>29.15</v>
       </c>
-      <c r="X52" s="42" t="n">
+      <c r="X52" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y52" s="42" t="n">
+      <c r="Y52" s="46" t="n">
         <f aca="false">X52/1.1</f>
         <v>41.6</v>
       </c>
@@ -13178,16 +13200,16 @@
       <c r="K54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L54" s="42" t="n">
+      <c r="L54" s="46" t="n">
         <v>34.67</v>
       </c>
-      <c r="M54" s="42" t="n">
+      <c r="M54" s="46" t="n">
         <v>31.52</v>
       </c>
-      <c r="N54" s="42" t="n">
+      <c r="N54" s="46" t="n">
         <v>28.3</v>
       </c>
-      <c r="O54" s="42" t="n">
+      <c r="O54" s="46" t="n">
         <f aca="false">N54/1.1</f>
         <v>25.7272727272727</v>
       </c>
@@ -13197,10 +13219,10 @@
       <c r="Q54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R54" s="42" t="n">
+      <c r="R54" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S54" s="42" t="n">
+      <c r="S54" s="46" t="n">
         <f aca="false">R54/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -13216,10 +13238,10 @@
       <c r="W54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X54" s="42" t="n">
+      <c r="X54" s="46" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y54" s="42" t="n">
+      <c r="Y54" s="46" t="n">
         <f aca="false">X54/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -13311,10 +13333,10 @@
       <c r="Q55" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R55" s="42" t="n">
+      <c r="R55" s="46" t="n">
         <v>23</v>
       </c>
-      <c r="S55" s="42" t="n">
+      <c r="S55" s="46" t="n">
         <f aca="false">R55/1.1</f>
         <v>20.9090909090909</v>
       </c>
@@ -13342,8 +13364,8 @@
       <c r="AA55" s="42" t="s">
         <v>309</v>
       </c>
-      <c r="AB55" s="42"/>
-      <c r="AC55" s="42"/>
+      <c r="AB55" s="47"/>
+      <c r="AC55" s="47"/>
       <c r="AD55" s="11" t="n">
         <f aca="false">IF(COUNT(I55,J55,M55,O55,Q55,S55,U55,V55,Y55,AA55,AC55)=0,"N/A",MIN(I55,J55,M55,O55,Q55,S55,U55,V55,Y55,AA55,AC55))</f>
         <v>20.9090909090909</v>
@@ -13412,16 +13434,16 @@
       <c r="O56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P56" s="42" t="n">
+      <c r="P56" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q56" s="42" t="n">
+      <c r="Q56" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R56" s="42" t="n">
+      <c r="R56" s="46" t="n">
         <v>33.5</v>
       </c>
-      <c r="S56" s="42" t="n">
+      <c r="S56" s="46" t="n">
         <f aca="false">R56/1.1</f>
         <v>30.4545454545455</v>
       </c>
@@ -13437,10 +13459,10 @@
       <c r="W56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X56" s="42" t="n">
+      <c r="X56" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y56" s="42" t="n">
+      <c r="Y56" s="46" t="n">
         <f aca="false">X56/1.1</f>
         <v>41.6</v>
       </c>
@@ -13450,8 +13472,8 @@
       <c r="AA56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB56" s="42"/>
-      <c r="AC56" s="42"/>
+      <c r="AB56" s="47"/>
+      <c r="AC56" s="47"/>
       <c r="AD56" s="11" t="n">
         <f aca="false">IF(COUNT(I56,J56,M56,O56,Q56,S56,U56,V56,Y56,AA56,AC56)=0,"N/A",MIN(I56,J56,M56,O56,Q56,S56,U56,V56,Y56,AA56,AC56))</f>
         <v>22</v>
@@ -13508,10 +13530,10 @@
       <c r="K57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L57" s="42" t="n">
+      <c r="L57" s="46" t="n">
         <v>39.47</v>
       </c>
-      <c r="M57" s="42" t="n">
+      <c r="M57" s="46" t="n">
         <v>35.88</v>
       </c>
       <c r="N57" s="42" t="s">
@@ -13526,10 +13548,10 @@
       <c r="Q57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R57" s="42" t="n">
+      <c r="R57" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="S57" s="42" t="n">
+      <c r="S57" s="46" t="n">
         <f aca="false">R57/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -13545,10 +13567,10 @@
       <c r="W57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X57" s="42" t="n">
+      <c r="X57" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y57" s="42" t="n">
+      <c r="Y57" s="46" t="n">
         <f aca="false">X57/1.1</f>
         <v>41.6</v>
       </c>
@@ -13628,23 +13650,23 @@
       <c r="M58" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N58" s="42" t="n">
+      <c r="N58" s="46" t="n">
         <v>42.5</v>
       </c>
-      <c r="O58" s="42" t="n">
+      <c r="O58" s="46" t="n">
         <f aca="false">N58/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P58" s="42" t="n">
+      <c r="P58" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q58" s="42" t="n">
+      <c r="Q58" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R58" s="42" t="n">
+      <c r="R58" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="S58" s="42" t="n">
+      <c r="S58" s="46" t="n">
         <f aca="false">R58/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -13660,10 +13682,10 @@
       <c r="W58" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X58" s="42" t="n">
+      <c r="X58" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y58" s="42" t="n">
+      <c r="Y58" s="46" t="n">
         <f aca="false">X58/1.1</f>
         <v>41.6</v>
       </c>
@@ -13743,10 +13765,10 @@
       <c r="M59" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N59" s="42" t="n">
+      <c r="N59" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="O59" s="42" t="n">
+      <c r="O59" s="46" t="n">
         <f aca="false">N59/1.1</f>
         <v>25</v>
       </c>
@@ -13756,10 +13778,10 @@
       <c r="Q59" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R59" s="42" t="n">
+      <c r="R59" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="S59" s="42" t="n">
+      <c r="S59" s="46" t="n">
         <f aca="false">R59/1.1</f>
         <v>20</v>
       </c>
@@ -13887,10 +13909,10 @@
       <c r="W60" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X60" s="42" t="n">
+      <c r="X60" s="46" t="n">
         <v>41.4</v>
       </c>
-      <c r="Y60" s="42" t="n">
+      <c r="Y60" s="46" t="n">
         <f aca="false">X60/1.1</f>
         <v>37.6363636363636</v>
       </c>
@@ -13964,16 +13986,16 @@
       <c r="K61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L61" s="42" t="n">
+      <c r="L61" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M61" s="42" t="n">
+      <c r="M61" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N61" s="42" t="n">
+      <c r="N61" s="46" t="n">
         <v>42.5</v>
       </c>
-      <c r="O61" s="42" t="n">
+      <c r="O61" s="46" t="n">
         <f aca="false">N61/1.1</f>
         <v>38.6363636363636</v>
       </c>
@@ -13983,10 +14005,10 @@
       <c r="Q61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R61" s="42" t="n">
+      <c r="R61" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="S61" s="42" t="n">
+      <c r="S61" s="46" t="n">
         <f aca="false">R61/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -14002,10 +14024,10 @@
       <c r="W61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X61" s="42" t="n">
+      <c r="X61" s="46" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y61" s="42" t="n">
+      <c r="Y61" s="46" t="n">
         <f aca="false">X61/1.1</f>
         <v>41.6</v>
       </c>
@@ -14079,29 +14101,29 @@
       <c r="K62" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L62" s="42" t="n">
+      <c r="L62" s="46" t="n">
         <v>39.47</v>
       </c>
-      <c r="M62" s="42" t="n">
+      <c r="M62" s="46" t="n">
         <v>35.88</v>
       </c>
-      <c r="N62" s="42" t="n">
+      <c r="N62" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="O62" s="42" t="n">
+      <c r="O62" s="46" t="n">
         <f aca="false">N62/1.1</f>
         <v>25</v>
       </c>
-      <c r="P62" s="42" t="n">
+      <c r="P62" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q62" s="42" t="n">
+      <c r="Q62" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R62" s="42" t="n">
+      <c r="R62" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S62" s="42" t="n">
+      <c r="S62" s="46" t="n">
         <f aca="false">R62/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -14117,10 +14139,10 @@
       <c r="W62" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X62" s="42" t="n">
+      <c r="X62" s="46" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y62" s="42" t="n">
+      <c r="Y62" s="46" t="n">
         <f aca="false">X62/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -14194,10 +14216,10 @@
       <c r="K63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L63" s="42" t="n">
+      <c r="L63" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M63" s="42" t="n">
+      <c r="M63" s="46" t="n">
         <v>35.98</v>
       </c>
       <c r="N63" s="42" t="s">
@@ -14206,16 +14228,16 @@
       <c r="O63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P63" s="42" t="n">
+      <c r="P63" s="46" t="n">
         <v>22.6</v>
       </c>
-      <c r="Q63" s="42" t="n">
+      <c r="Q63" s="46" t="n">
         <v>20.55</v>
       </c>
-      <c r="R63" s="42" t="n">
+      <c r="R63" s="46" t="n">
         <v>23</v>
       </c>
-      <c r="S63" s="42" t="n">
+      <c r="S63" s="46" t="n">
         <f aca="false">R63/1.1</f>
         <v>20.9090909090909</v>
       </c>
@@ -14231,10 +14253,10 @@
       <c r="W63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X63" s="42" t="n">
+      <c r="X63" s="46" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y63" s="42" t="n">
+      <c r="Y63" s="46" t="n">
         <f aca="false">X63/1.1</f>
         <v>29.0545454545455</v>
       </c>
@@ -14308,29 +14330,29 @@
       <c r="K64" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L64" s="42" t="n">
+      <c r="L64" s="46" t="n">
         <v>39.58</v>
       </c>
-      <c r="M64" s="42" t="n">
+      <c r="M64" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="N64" s="42" t="n">
+      <c r="N64" s="46" t="n">
         <v>27.5</v>
       </c>
-      <c r="O64" s="42" t="n">
+      <c r="O64" s="46" t="n">
         <f aca="false">N64/1.1</f>
         <v>25</v>
       </c>
-      <c r="P64" s="42" t="n">
+      <c r="P64" s="46" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q64" s="42" t="n">
+      <c r="Q64" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="R64" s="42" t="n">
+      <c r="R64" s="46" t="n">
         <v>22.5</v>
       </c>
-      <c r="S64" s="42" t="n">
+      <c r="S64" s="46" t="n">
         <f aca="false">R64/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -14346,10 +14368,10 @@
       <c r="W64" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X64" s="42" t="n">
+      <c r="X64" s="46" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y64" s="42" t="n">
+      <c r="Y64" s="46" t="n">
         <f aca="false">X64/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -14423,10 +14445,10 @@
       <c r="K65" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L65" s="42" t="n">
+      <c r="L65" s="46" t="n">
         <v>39.47</v>
       </c>
-      <c r="M65" s="42" t="n">
+      <c r="M65" s="46" t="n">
         <v>35.88</v>
       </c>
       <c r="N65" s="11" t="n">
@@ -14511,7 +14533,7 @@
       </c>
       <c r="B68" s="35"/>
       <c r="C68" s="35"/>
-      <c r="D68" s="46" t="n">
+      <c r="D68" s="48" t="n">
         <f aca="false">COUNTA(B6:B65)</f>
         <v>60</v>
       </c>
@@ -14522,7 +14544,7 @@
       </c>
       <c r="B69" s="35"/>
       <c r="C69" s="35"/>
-      <c r="D69" s="46" t="n">
+      <c r="D69" s="48" t="n">
         <f aca="false">COUNTIF(J6:J65,"&gt;0")+COUNTIF(M6:M65,"&gt;0")+COUNTIF(O6:O65,"&gt;0")+COUNTIF(Q6:Q65,"&gt;0")+COUNTIF(S6:S65,"&gt;0")+COUNTIF(U6:U65,"&gt;0")+COUNTIF(V6:V65,"&gt;0")+COUNTIF(Y6:Y65,"&gt;0")+COUNTIF(AA6:AA65,"&gt;0")+COUNTIF(AC6:AC65,"&gt;0")</f>
         <v>407</v>
       </c>
@@ -14533,7 +14555,7 @@
       </c>
       <c r="B70" s="35"/>
       <c r="C70" s="35"/>
-      <c r="D70" s="46" t="n">
+      <c r="D70" s="48" t="n">
         <f aca="false">COUNTIF(AE6:AE65,"&lt;0")</f>
         <v>53</v>
       </c>
@@ -14544,7 +14566,7 @@
       </c>
       <c r="B71" s="35"/>
       <c r="C71" s="35"/>
-      <c r="D71" s="46" t="n">
+      <c r="D71" s="48" t="n">
         <f aca="false">COUNTIF(AE6:AE65,"&gt;0")</f>
         <v>7</v>
       </c>
@@ -14555,7 +14577,7 @@
       </c>
       <c r="B72" s="35"/>
       <c r="C72" s="35"/>
-      <c r="D72" s="47" t="n">
+      <c r="D72" s="49" t="n">
         <f aca="false">AVERAGE(AE6:AE65)</f>
         <v>-0.454866678565887</v>
       </c>
@@ -14566,7 +14588,7 @@
       </c>
       <c r="B73" s="35"/>
       <c r="C73" s="35"/>
-      <c r="D73" s="47" t="n">
+      <c r="D73" s="49" t="n">
         <f aca="false">MEDIAN(AE6:AE65)</f>
         <v>-0.523652597402597</v>
       </c>
@@ -14577,7 +14599,7 @@
       </c>
       <c r="B74" s="35"/>
       <c r="C74" s="35"/>
-      <c r="D74" s="46" t="n">
+      <c r="D74" s="48" t="n">
         <f aca="false">COUNTIF(AF6:AF65,"&lt;0")</f>
         <v>15</v>
       </c>
@@ -14588,7 +14610,7 @@
       </c>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
-      <c r="D75" s="46" t="n">
+      <c r="D75" s="48" t="n">
         <f aca="false">COUNTIF(AF6:AF65,"&gt;0")</f>
         <v>7</v>
       </c>
@@ -14599,7 +14621,7 @@
       </c>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
-      <c r="D76" s="47" t="n">
+      <c r="D76" s="49" t="n">
         <f aca="false">AVERAGE(AF6:AF65)</f>
         <v>-0.137849955170021</v>
       </c>
@@ -14610,7 +14632,7 @@
       </c>
       <c r="B77" s="35"/>
       <c r="C77" s="35"/>
-      <c r="D77" s="47" t="n">
+      <c r="D77" s="49" t="n">
         <f aca="false">MEDIAN(AF6:AF65)</f>
         <v>-0.240924975181021</v>
       </c>
@@ -14631,6 +14653,21 @@
     <mergeCell ref="A76:C76"/>
     <mergeCell ref="A77:C77"/>
   </mergeCells>
+  <conditionalFormatting sqref="AD6:AD65">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>EXACT(AD6,"N/A")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE6:AE65">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>EXACT(AE6,"N/A")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF6:AF65">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>EXACT(AF6,"N/A")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -14662,62 +14699,62 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="50" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
     </row>
     <row r="2" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="51" t="s">
         <v>332</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="52" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="52" t="s">
         <v>333</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="52" t="s">
         <v>334</v>
       </c>
-      <c r="F4" s="50" t="s">
+      <c r="F4" s="52" t="s">
         <v>335</v>
       </c>
-      <c r="G4" s="50" t="s">
+      <c r="G4" s="52" t="s">
         <v>336</v>
       </c>
-      <c r="H4" s="50" t="s">
+      <c r="H4" s="52" t="s">
         <v>337</v>
       </c>
-      <c r="I4" s="50" t="s">
+      <c r="I4" s="52" t="s">
         <v>338</v>
       </c>
-      <c r="J4" s="50" t="s">
+      <c r="J4" s="52" t="s">
         <v>221</v>
       </c>
     </row>
@@ -14737,13 +14774,13 @@
       <c r="E5" s="11" t="n">
         <v>20.05</v>
       </c>
-      <c r="F5" s="51" t="n">
+      <c r="F5" s="53" t="n">
         <v>16.93275</v>
       </c>
-      <c r="G5" s="52" t="n">
+      <c r="G5" s="54" t="n">
         <v>-3.11725</v>
       </c>
-      <c r="H5" s="53" t="n">
+      <c r="H5" s="55" t="n">
         <v>-0.155473815461347</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -14766,13 +14803,13 @@
       <c r="E6" s="11" t="n">
         <v>122.718181818182</v>
       </c>
-      <c r="F6" s="54" t="n">
+      <c r="F6" s="56" t="n">
         <v>66.83</v>
       </c>
-      <c r="G6" s="52" t="n">
+      <c r="G6" s="54" t="n">
         <v>-55.888181818182</v>
       </c>
-      <c r="H6" s="53" t="n">
+      <c r="H6" s="55" t="n">
         <v>-0.455418919919995</v>
       </c>
       <c r="I6" s="1" t="s">
@@ -14795,13 +14832,13 @@
       <c r="E7" s="11" t="n">
         <v>128.75</v>
       </c>
-      <c r="F7" s="54" t="n">
+      <c r="F7" s="56" t="n">
         <v>44.55</v>
       </c>
-      <c r="G7" s="52" t="n">
+      <c r="G7" s="54" t="n">
         <v>-84.2</v>
       </c>
-      <c r="H7" s="53" t="n">
+      <c r="H7" s="55" t="n">
         <v>-0.653980582524272</v>
       </c>
       <c r="I7" s="1" t="s">
@@ -14824,13 +14861,13 @@
       <c r="E8" s="11" t="n">
         <v>69.245</v>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="53" t="n">
         <v>45.144</v>
       </c>
-      <c r="G8" s="52" t="n">
+      <c r="G8" s="54" t="n">
         <v>-24.101</v>
       </c>
-      <c r="H8" s="53" t="n">
+      <c r="H8" s="55" t="n">
         <v>-0.348054011119937</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -14853,13 +14890,13 @@
       <c r="E9" s="11" t="n">
         <v>81.4</v>
       </c>
-      <c r="F9" s="51" t="n">
+      <c r="F9" s="53" t="n">
         <v>70.538125</v>
       </c>
-      <c r="G9" s="52" t="n">
+      <c r="G9" s="54" t="n">
         <v>-10.861875</v>
       </c>
-      <c r="H9" s="53" t="n">
+      <c r="H9" s="55" t="n">
         <v>-0.133438267813268</v>
       </c>
       <c r="I9" s="1" t="s">
@@ -14882,13 +14919,13 @@
       <c r="E10" s="11" t="n">
         <v>44.209</v>
       </c>
-      <c r="F10" s="51" t="n">
+      <c r="F10" s="53" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G10" s="52" t="n">
+      <c r="G10" s="54" t="n">
         <v>-10.3535</v>
       </c>
-      <c r="H10" s="53" t="n">
+      <c r="H10" s="55" t="n">
         <v>-0.234194394806487</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -14911,13 +14948,13 @@
       <c r="E11" s="11" t="n">
         <v>70.36</v>
       </c>
-      <c r="F11" s="51" t="n">
+      <c r="F11" s="53" t="n">
         <v>45.144</v>
       </c>
-      <c r="G11" s="52" t="n">
+      <c r="G11" s="54" t="n">
         <v>-25.216</v>
       </c>
-      <c r="H11" s="53" t="n">
+      <c r="H11" s="55" t="n">
         <v>-0.358385446276293</v>
       </c>
       <c r="I11" s="1" t="s">
@@ -14925,34 +14962,34 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="55" t="s">
+      <c r="A12" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="56" t="s">
+      <c r="C12" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="55" t="s">
+      <c r="D12" s="57" t="s">
         <v>345</v>
       </c>
-      <c r="E12" s="57" t="n">
+      <c r="E12" s="59" t="n">
         <v>33.1818181818182</v>
       </c>
-      <c r="F12" s="58" t="n">
+      <c r="F12" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G12" s="59" t="n">
+      <c r="G12" s="61" t="n">
         <v>0.673681818181798</v>
       </c>
-      <c r="H12" s="60" t="n">
+      <c r="H12" s="62" t="n">
         <v>0.0203027397260268</v>
       </c>
-      <c r="I12" s="61" t="s">
+      <c r="I12" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J12" s="55"/>
+      <c r="J12" s="57"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -14970,13 +15007,13 @@
       <c r="E13" s="11" t="n">
         <v>43.09</v>
       </c>
-      <c r="F13" s="51" t="n">
+      <c r="F13" s="53" t="n">
         <v>25.394125</v>
       </c>
-      <c r="G13" s="52" t="n">
+      <c r="G13" s="54" t="n">
         <v>-17.695875</v>
       </c>
-      <c r="H13" s="53" t="n">
+      <c r="H13" s="55" t="n">
         <v>-0.410672429798097</v>
       </c>
       <c r="I13" s="1" t="s">
@@ -14999,13 +15036,13 @@
       <c r="E14" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F14" s="51" t="n">
+      <c r="F14" s="53" t="n">
         <v>8.461375</v>
       </c>
-      <c r="G14" s="52" t="n">
+      <c r="G14" s="54" t="n">
         <v>-13.538625</v>
       </c>
-      <c r="H14" s="53" t="n">
+      <c r="H14" s="55" t="n">
         <v>-0.615392045454545</v>
       </c>
       <c r="I14" s="1" t="s">
@@ -15028,13 +15065,13 @@
       <c r="E15" s="11" t="n">
         <v>21.9</v>
       </c>
-      <c r="F15" s="51" t="n">
+      <c r="F15" s="53" t="n">
         <v>15.81275</v>
       </c>
-      <c r="G15" s="52" t="n">
+      <c r="G15" s="54" t="n">
         <v>-6.08725</v>
       </c>
-      <c r="H15" s="53" t="n">
+      <c r="H15" s="55" t="n">
         <v>-0.277956621004566</v>
       </c>
       <c r="I15" s="1" t="s">
@@ -15057,13 +15094,13 @@
       <c r="E16" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="F16" s="51" t="n">
+      <c r="F16" s="53" t="n">
         <v>8.461375</v>
       </c>
-      <c r="G16" s="52" t="n">
+      <c r="G16" s="54" t="n">
         <v>-2.038625</v>
       </c>
-      <c r="H16" s="53" t="n">
+      <c r="H16" s="55" t="n">
         <v>-0.194154761904762</v>
       </c>
       <c r="I16" s="1" t="s">
@@ -15086,13 +15123,13 @@
       <c r="E17" s="11" t="n">
         <v>37.3909090909091</v>
       </c>
-      <c r="F17" s="51" t="n">
+      <c r="F17" s="53" t="n">
         <v>30.1455</v>
       </c>
-      <c r="G17" s="52" t="n">
+      <c r="G17" s="54" t="n">
         <v>-7.2454090909091</v>
       </c>
-      <c r="H17" s="53" t="n">
+      <c r="H17" s="55" t="n">
         <v>-0.193774617067834</v>
       </c>
       <c r="I17" s="1" t="s">
@@ -15100,34 +15137,34 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="55" t="s">
+      <c r="A18" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B18" s="55" t="s">
+      <c r="B18" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="C18" s="56" t="s">
+      <c r="C18" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="55" t="s">
+      <c r="D18" s="57" t="s">
         <v>347</v>
       </c>
-      <c r="E18" s="57" t="n">
+      <c r="E18" s="59" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="F18" s="58" t="n">
+      <c r="F18" s="60" t="n">
         <v>30.1455</v>
       </c>
-      <c r="G18" s="59" t="n">
+      <c r="G18" s="61" t="n">
         <v>1.7909545454545</v>
       </c>
-      <c r="H18" s="60" t="n">
+      <c r="H18" s="62" t="n">
         <v>0.0631628727156122</v>
       </c>
-      <c r="I18" s="61" t="s">
+      <c r="I18" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J18" s="55"/>
+      <c r="J18" s="57"/>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -15145,13 +15182,13 @@
       <c r="E19" s="11" t="n">
         <v>23.3090909090909</v>
       </c>
-      <c r="F19" s="51" t="n">
+      <c r="F19" s="53" t="n">
         <v>16.93275</v>
       </c>
-      <c r="G19" s="52" t="n">
+      <c r="G19" s="54" t="n">
         <v>-6.3763409090909</v>
       </c>
-      <c r="H19" s="53" t="n">
+      <c r="H19" s="55" t="n">
         <v>-0.273555967238689</v>
       </c>
       <c r="I19" s="1" t="s">
@@ -15159,34 +15196,34 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="55" t="s">
+      <c r="A20" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="56" t="s">
+      <c r="C20" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="55" t="s">
+      <c r="D20" s="57" t="s">
         <v>348</v>
       </c>
-      <c r="E20" s="57" t="n">
+      <c r="E20" s="59" t="n">
         <v>33.7</v>
       </c>
-      <c r="F20" s="58" t="n">
+      <c r="F20" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G20" s="59" t="n">
+      <c r="G20" s="61" t="n">
         <v>0.155499999999996</v>
       </c>
-      <c r="H20" s="60" t="n">
+      <c r="H20" s="62" t="n">
         <v>0.00461424332344203</v>
       </c>
-      <c r="I20" s="61" t="s">
+      <c r="I20" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J20" s="55"/>
+      <c r="J20" s="57"/>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
@@ -15204,13 +15241,13 @@
       <c r="E21" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F21" s="51" t="n">
+      <c r="F21" s="53" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G21" s="52" t="n">
+      <c r="G21" s="54" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H21" s="53" t="n">
+      <c r="H21" s="55" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I21" s="1" t="s">
@@ -15233,13 +15270,13 @@
       <c r="E22" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F22" s="51" t="n">
+      <c r="F22" s="53" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G22" s="52" t="n">
+      <c r="G22" s="54" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H22" s="53" t="n">
+      <c r="H22" s="55" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I22" s="1" t="s">
@@ -15262,13 +15299,13 @@
       <c r="E23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F23" s="51" t="n">
+      <c r="F23" s="53" t="n">
         <v>6.011375</v>
       </c>
-      <c r="G23" s="52" t="n">
+      <c r="G23" s="54" t="n">
         <v>-15.988625</v>
       </c>
-      <c r="H23" s="53" t="n">
+      <c r="H23" s="55" t="n">
         <v>-0.726755681818182</v>
       </c>
       <c r="I23" s="1" t="s">
@@ -15276,64 +15313,64 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="C24" s="56" t="s">
+      <c r="C24" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="D24" s="55" t="s">
+      <c r="D24" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="E24" s="57" t="n">
+      <c r="E24" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F24" s="58" t="n">
+      <c r="F24" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G24" s="59" t="n">
+      <c r="G24" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="H24" s="60" t="n">
+      <c r="H24" s="62" t="n">
         <v>0.286299805636541</v>
       </c>
-      <c r="I24" s="61" t="s">
+      <c r="I24" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J24" s="55"/>
+      <c r="J24" s="57"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="C25" s="56" t="s">
+      <c r="C25" s="58" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="55" t="s">
+      <c r="D25" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="E25" s="57" t="n">
+      <c r="E25" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F25" s="58" t="n">
+      <c r="F25" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G25" s="59" t="n">
+      <c r="G25" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="H25" s="60" t="n">
+      <c r="H25" s="62" t="n">
         <v>0.286299805636541</v>
       </c>
-      <c r="I25" s="61" t="s">
+      <c r="I25" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J25" s="55"/>
+      <c r="J25" s="57"/>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
@@ -15351,13 +15388,13 @@
       <c r="E26" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F26" s="51" t="n">
+      <c r="F26" s="53" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G26" s="52" t="n">
+      <c r="G26" s="54" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H26" s="53" t="n">
+      <c r="H26" s="55" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I26" s="1" t="s">
@@ -15365,34 +15402,34 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="55" t="s">
+      <c r="A27" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="B27" s="55" t="s">
+      <c r="B27" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="C27" s="56" t="s">
+      <c r="C27" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="D27" s="55" t="s">
+      <c r="D27" s="57" t="s">
         <v>345</v>
       </c>
-      <c r="E27" s="57" t="n">
+      <c r="E27" s="59" t="n">
         <v>32.5</v>
       </c>
-      <c r="F27" s="58" t="n">
+      <c r="F27" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G27" s="59" t="n">
+      <c r="G27" s="61" t="n">
         <v>1.3555</v>
       </c>
-      <c r="H27" s="60" t="n">
+      <c r="H27" s="62" t="n">
         <v>0.0417076923076923</v>
       </c>
-      <c r="I27" s="61" t="s">
+      <c r="I27" s="63" t="s">
         <v>346</v>
       </c>
-      <c r="J27" s="55"/>
+      <c r="J27" s="57"/>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -15410,13 +15447,13 @@
       <c r="E28" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="F28" s="51" t="n">
+      <c r="F28" s="53" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G28" s="52" t="n">
+      <c r="G28" s="54" t="n">
         <v>-11.1445</v>
       </c>
-      <c r="H28" s="53" t="n">
+      <c r="H28" s="55" t="n">
         <v>-0.247655555555556</v>
       </c>
       <c r="I28" s="1" t="s">
@@ -15439,13 +15476,13 @@
       <c r="E29" s="11" t="n">
         <v>30.8</v>
       </c>
-      <c r="F29" s="54" t="n">
+      <c r="F29" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G29" s="52" t="n">
+      <c r="G29" s="54" t="n">
         <v>-17.73</v>
       </c>
-      <c r="H29" s="53" t="n">
+      <c r="H29" s="55" t="n">
         <v>-0.575649350649351</v>
       </c>
       <c r="I29" s="1" t="s">
@@ -15468,13 +15505,13 @@
       <c r="E30" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="F30" s="54" t="n">
+      <c r="F30" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G30" s="52" t="n">
+      <c r="G30" s="54" t="n">
         <v>-14.93</v>
       </c>
-      <c r="H30" s="53" t="n">
+      <c r="H30" s="55" t="n">
         <v>-0.533214285714286</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -15497,13 +15534,13 @@
       <c r="E31" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F31" s="54" t="n">
+      <c r="F31" s="56" t="n">
         <v>16.04</v>
       </c>
-      <c r="G31" s="52" t="n">
+      <c r="G31" s="54" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H31" s="53" t="n">
+      <c r="H31" s="55" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I31" s="1" t="s">
@@ -15526,13 +15563,13 @@
       <c r="E32" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F32" s="54" t="n">
+      <c r="F32" s="56" t="n">
         <v>16.04</v>
       </c>
-      <c r="G32" s="52" t="n">
+      <c r="G32" s="54" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H32" s="53" t="n">
+      <c r="H32" s="55" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I32" s="1" t="s">
@@ -15555,13 +15592,13 @@
       <c r="E33" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F33" s="54" t="n">
+      <c r="F33" s="56" t="n">
         <v>16.04</v>
       </c>
-      <c r="G33" s="52" t="n">
+      <c r="G33" s="54" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H33" s="53" t="n">
+      <c r="H33" s="55" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I33" s="1" t="s">
@@ -15584,13 +15621,13 @@
       <c r="E34" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F34" s="54" t="n">
+      <c r="F34" s="56" t="n">
         <v>16.04</v>
       </c>
-      <c r="G34" s="52" t="n">
+      <c r="G34" s="54" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H34" s="53" t="n">
+      <c r="H34" s="55" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I34" s="1" t="s">
@@ -15613,13 +15650,13 @@
       <c r="E35" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F35" s="54" t="n">
+      <c r="F35" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G35" s="52" t="n">
+      <c r="G35" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H35" s="53" t="n">
+      <c r="H35" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I35" s="1" t="s">
@@ -15642,13 +15679,13 @@
       <c r="E36" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F36" s="54" t="n">
+      <c r="F36" s="56" t="n">
         <v>16.04</v>
       </c>
-      <c r="G36" s="52" t="n">
+      <c r="G36" s="54" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H36" s="53" t="n">
+      <c r="H36" s="55" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I36" s="1" t="s">
@@ -15671,13 +15708,13 @@
       <c r="E37" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F37" s="54" t="n">
+      <c r="F37" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G37" s="52" t="n">
+      <c r="G37" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H37" s="53" t="n">
+      <c r="H37" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I37" s="1" t="s">
@@ -15700,13 +15737,13 @@
       <c r="E38" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F38" s="54" t="n">
+      <c r="F38" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G38" s="52" t="n">
+      <c r="G38" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H38" s="53" t="n">
+      <c r="H38" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I38" s="1" t="s">
@@ -15729,13 +15766,13 @@
       <c r="E39" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F39" s="54" t="n">
+      <c r="F39" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G39" s="52" t="n">
+      <c r="G39" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H39" s="53" t="n">
+      <c r="H39" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I39" s="1" t="s">
@@ -15758,13 +15795,13 @@
       <c r="E40" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F40" s="54" t="n">
+      <c r="F40" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G40" s="52" t="n">
+      <c r="G40" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H40" s="53" t="n">
+      <c r="H40" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I40" s="1" t="s">
@@ -15787,13 +15824,13 @@
       <c r="E41" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F41" s="54" t="n">
+      <c r="F41" s="56" t="n">
         <v>13.07</v>
       </c>
-      <c r="G41" s="52" t="n">
+      <c r="G41" s="54" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H41" s="53" t="n">
+      <c r="H41" s="55" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I41" s="1" t="s">
@@ -15816,13 +15853,13 @@
       <c r="E42" s="11" t="n">
         <v>20.05</v>
       </c>
-      <c r="F42" s="54" t="n">
+      <c r="F42" s="56" t="n">
         <v>5.35</v>
       </c>
-      <c r="G42" s="52" t="n">
+      <c r="G42" s="54" t="n">
         <v>-14.7</v>
       </c>
-      <c r="H42" s="53" t="n">
+      <c r="H42" s="55" t="n">
         <v>-0.733167082294264</v>
       </c>
       <c r="I42" s="1" t="s">
@@ -15845,13 +15882,13 @@
       <c r="E43" s="11" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F43" s="54" t="n">
+      <c r="F43" s="56" t="n">
         <v>2.67</v>
       </c>
-      <c r="G43" s="52" t="n">
+      <c r="G43" s="54" t="n">
         <v>-6.68454545454545</v>
       </c>
-      <c r="H43" s="53" t="n">
+      <c r="H43" s="55" t="n">
         <v>-0.714577259475219</v>
       </c>
       <c r="I43" s="1" t="s">
@@ -15874,13 +15911,13 @@
       <c r="E44" s="11" t="n">
         <v>23.4090909090909</v>
       </c>
-      <c r="F44" s="54" t="n">
+      <c r="F44" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G44" s="52" t="n">
+      <c r="G44" s="54" t="n">
         <v>-12.7190909090909</v>
       </c>
-      <c r="H44" s="53" t="n">
+      <c r="H44" s="55" t="n">
         <v>-0.543339805825243</v>
       </c>
       <c r="I44" s="1" t="s">
@@ -15903,13 +15940,13 @@
       <c r="E45" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F45" s="54" t="n">
+      <c r="F45" s="56" t="n">
         <v>2.67</v>
       </c>
-      <c r="G45" s="52" t="n">
+      <c r="G45" s="54" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H45" s="53" t="n">
+      <c r="H45" s="55" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I45" s="1" t="s">
@@ -15932,13 +15969,13 @@
       <c r="E46" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F46" s="54" t="n">
+      <c r="F46" s="56" t="n">
         <v>9.5</v>
       </c>
-      <c r="G46" s="52" t="n">
+      <c r="G46" s="54" t="n">
         <v>-12.5</v>
       </c>
-      <c r="H46" s="53" t="n">
+      <c r="H46" s="55" t="n">
         <v>-0.568181818181818</v>
       </c>
       <c r="I46" s="1" t="s">
@@ -15961,13 +15998,13 @@
       <c r="E47" s="11" t="n">
         <v>16.7363636363636</v>
       </c>
-      <c r="F47" s="54" t="n">
+      <c r="F47" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G47" s="52" t="n">
+      <c r="G47" s="54" t="n">
         <v>-6.0463636363636</v>
       </c>
-      <c r="H47" s="53" t="n">
+      <c r="H47" s="55" t="n">
         <v>-0.36127104834329</v>
       </c>
       <c r="I47" s="1" t="s">
@@ -15990,13 +16027,13 @@
       <c r="E48" s="11" t="n">
         <v>20.9090909090909</v>
       </c>
-      <c r="F48" s="54" t="n">
+      <c r="F48" s="56" t="n">
         <v>5.35</v>
       </c>
-      <c r="G48" s="52" t="n">
+      <c r="G48" s="54" t="n">
         <v>-15.5590909090909</v>
       </c>
-      <c r="H48" s="53" t="n">
+      <c r="H48" s="55" t="n">
         <v>-0.744130434782609</v>
       </c>
       <c r="I48" s="1" t="s">
@@ -16019,13 +16056,13 @@
       <c r="E49" s="11" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F49" s="54" t="n">
+      <c r="F49" s="56" t="n">
         <v>5.35</v>
       </c>
-      <c r="G49" s="52" t="n">
+      <c r="G49" s="54" t="n">
         <v>-4.00454545454545</v>
       </c>
-      <c r="H49" s="53" t="n">
+      <c r="H49" s="55" t="n">
         <v>-0.428085519922254</v>
       </c>
       <c r="I49" s="1" t="s">
@@ -16048,13 +16085,13 @@
       <c r="E50" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="F50" s="54" t="n">
+      <c r="F50" s="56" t="n">
         <v>2.67</v>
       </c>
-      <c r="G50" s="52" t="n">
+      <c r="G50" s="54" t="n">
         <v>-7.83</v>
       </c>
-      <c r="H50" s="53" t="n">
+      <c r="H50" s="55" t="n">
         <v>-0.745714285714286</v>
       </c>
       <c r="I50" s="1" t="s">
@@ -16077,13 +16114,13 @@
       <c r="E51" s="11" t="n">
         <v>26.5</v>
       </c>
-      <c r="F51" s="54" t="n">
+      <c r="F51" s="56" t="n">
         <v>9.5</v>
       </c>
-      <c r="G51" s="52" t="n">
+      <c r="G51" s="54" t="n">
         <v>-17</v>
       </c>
-      <c r="H51" s="53" t="n">
+      <c r="H51" s="55" t="n">
         <v>-0.641509433962264</v>
       </c>
       <c r="I51" s="1" t="s">
@@ -16106,13 +16143,13 @@
       <c r="E52" s="11" t="n">
         <v>7.81818181818182</v>
       </c>
-      <c r="F52" s="54" t="n">
+      <c r="F52" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G52" s="52" t="n">
+      <c r="G52" s="54" t="n">
         <v>-5.81818181818182</v>
       </c>
-      <c r="H52" s="53" t="n">
+      <c r="H52" s="55" t="n">
         <v>-0.744186046511628</v>
       </c>
       <c r="I52" s="1" t="s">
@@ -16135,13 +16172,13 @@
       <c r="E53" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F53" s="54" t="n">
+      <c r="F53" s="56" t="n">
         <v>2.67</v>
       </c>
-      <c r="G53" s="52" t="n">
+      <c r="G53" s="54" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H53" s="53" t="n">
+      <c r="H53" s="55" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I53" s="1" t="s">
@@ -16164,13 +16201,13 @@
       <c r="E54" s="11" t="n">
         <v>20.9090909090909</v>
       </c>
-      <c r="F54" s="54" t="n">
+      <c r="F54" s="56" t="n">
         <v>4.01</v>
       </c>
-      <c r="G54" s="52" t="n">
+      <c r="G54" s="54" t="n">
         <v>-16.8990909090909</v>
       </c>
-      <c r="H54" s="53" t="n">
+      <c r="H54" s="55" t="n">
         <v>-0.808217391304348</v>
       </c>
       <c r="I54" s="1" t="s">
@@ -16193,13 +16230,13 @@
       <c r="E55" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F55" s="54" t="n">
+      <c r="F55" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G55" s="52" t="n">
+      <c r="G55" s="54" t="n">
         <v>-11.31</v>
       </c>
-      <c r="H55" s="53" t="n">
+      <c r="H55" s="55" t="n">
         <v>-0.514090909090909</v>
       </c>
       <c r="I55" s="1" t="s">
@@ -16222,13 +16259,13 @@
       <c r="E56" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F56" s="54" t="n">
+      <c r="F56" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G56" s="52" t="n">
+      <c r="G56" s="54" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H56" s="53" t="n">
+      <c r="H56" s="55" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I56" s="1" t="s">
@@ -16251,13 +16288,13 @@
       <c r="E57" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F57" s="54" t="n">
+      <c r="F57" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G57" s="52" t="n">
+      <c r="G57" s="54" t="n">
         <v>-11.31</v>
       </c>
-      <c r="H57" s="53" t="n">
+      <c r="H57" s="55" t="n">
         <v>-0.514090909090909</v>
       </c>
       <c r="I57" s="1" t="s">
@@ -16280,13 +16317,13 @@
       <c r="E58" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="F58" s="54" t="n">
+      <c r="F58" s="56" t="n">
         <v>2.89</v>
       </c>
-      <c r="G58" s="52" t="n">
+      <c r="G58" s="54" t="n">
         <v>-17.11</v>
       </c>
-      <c r="H58" s="53" t="n">
+      <c r="H58" s="55" t="n">
         <v>-0.8555</v>
       </c>
       <c r="I58" s="1" t="s">
@@ -16309,13 +16346,13 @@
       <c r="E59" s="11" t="n">
         <v>37.6363636363636</v>
       </c>
-      <c r="F59" s="54" t="n">
+      <c r="F59" s="56" t="n">
         <v>1.94</v>
       </c>
-      <c r="G59" s="52" t="n">
+      <c r="G59" s="54" t="n">
         <v>-35.6963636363636</v>
       </c>
-      <c r="H59" s="53" t="n">
+      <c r="H59" s="55" t="n">
         <v>-0.948454106280193</v>
       </c>
       <c r="I59" s="1" t="s">
@@ -16338,13 +16375,13 @@
       <c r="E60" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F60" s="54" t="n">
+      <c r="F60" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G60" s="52" t="n">
+      <c r="G60" s="54" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H60" s="53" t="n">
+      <c r="H60" s="55" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I60" s="1" t="s">
@@ -16367,13 +16404,13 @@
       <c r="E61" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F61" s="54" t="n">
+      <c r="F61" s="56" t="n">
         <v>3.201</v>
       </c>
-      <c r="G61" s="52" t="n">
+      <c r="G61" s="54" t="n">
         <v>-17.2535454545455</v>
       </c>
-      <c r="H61" s="53" t="n">
+      <c r="H61" s="55" t="n">
         <v>-0.843506666666667</v>
       </c>
       <c r="I61" s="1" t="s">
@@ -16396,13 +16433,13 @@
       <c r="E62" s="11" t="n">
         <v>20.55</v>
       </c>
-      <c r="F62" s="54" t="n">
+      <c r="F62" s="56" t="n">
         <v>5.35</v>
       </c>
-      <c r="G62" s="52" t="n">
+      <c r="G62" s="54" t="n">
         <v>-15.2</v>
       </c>
-      <c r="H62" s="53" t="n">
+      <c r="H62" s="55" t="n">
         <v>-0.739659367396594</v>
       </c>
       <c r="I62" s="1" t="s">
@@ -16425,13 +16462,13 @@
       <c r="E63" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F63" s="54" t="n">
+      <c r="F63" s="56" t="n">
         <v>2.67</v>
       </c>
-      <c r="G63" s="52" t="n">
+      <c r="G63" s="54" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H63" s="53" t="n">
+      <c r="H63" s="55" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I63" s="1" t="s">
@@ -16454,13 +16491,13 @@
       <c r="E64" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F64" s="54" t="n">
+      <c r="F64" s="56" t="n">
         <v>10.69</v>
       </c>
-      <c r="G64" s="52" t="n">
+      <c r="G64" s="54" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H64" s="53" t="n">
+      <c r="H64" s="55" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I64" s="1" t="s">
@@ -16468,200 +16505,200 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="62" t="s">
+      <c r="A66" s="64" t="s">
         <v>350</v>
       </c>
-      <c r="B66" s="62"/>
-      <c r="C66" s="62"/>
-      <c r="D66" s="62"/>
-      <c r="E66" s="62"/>
-      <c r="F66" s="62"/>
-      <c r="G66" s="62"/>
-      <c r="H66" s="62"/>
-      <c r="I66" s="62"/>
-      <c r="J66" s="62"/>
+      <c r="B66" s="64"/>
+      <c r="C66" s="64"/>
+      <c r="D66" s="64"/>
+      <c r="E66" s="64"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="64"/>
+      <c r="H66" s="64"/>
+      <c r="I66" s="64"/>
+      <c r="J66" s="64"/>
     </row>
     <row r="67" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="50" t="s">
+      <c r="A67" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B67" s="50" t="s">
+      <c r="B67" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C67" s="50" t="s">
+      <c r="C67" s="52" t="s">
         <v>351</v>
       </c>
-      <c r="D67" s="50" t="s">
+      <c r="D67" s="52" t="s">
         <v>352</v>
       </c>
-      <c r="E67" s="50" t="s">
+      <c r="E67" s="52" t="s">
         <v>353</v>
       </c>
-      <c r="F67" s="50" t="s">
+      <c r="F67" s="52" t="s">
         <v>354</v>
       </c>
-      <c r="G67" s="50" t="s">
+      <c r="G67" s="52" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="55" t="s">
+      <c r="A68" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="B68" s="56" t="s">
+      <c r="B68" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C68" s="55" t="s">
+      <c r="C68" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="D68" s="57" t="n">
+      <c r="D68" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E68" s="57" t="n">
+      <c r="E68" s="59" t="n">
         <v>16.93275</v>
       </c>
-      <c r="F68" s="59" t="n">
+      <c r="F68" s="61" t="n">
         <v>7.57820454545455</v>
       </c>
-      <c r="G68" s="60" t="n">
+      <c r="G68" s="62" t="n">
         <v>0.447547181967167</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="55" t="s">
+      <c r="A69" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="B69" s="56" t="s">
+      <c r="B69" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="55" t="s">
+      <c r="C69" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="D69" s="57" t="n">
+      <c r="D69" s="59" t="n">
         <v>21.2</v>
       </c>
-      <c r="E69" s="57" t="n">
+      <c r="E69" s="59" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F69" s="59" t="n">
+      <c r="F69" s="61" t="n">
         <v>12.6555</v>
       </c>
-      <c r="G69" s="60" t="n">
+      <c r="G69" s="62" t="n">
         <v>0.373809277665372</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="55" t="s">
+      <c r="A70" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="B70" s="56" t="s">
+      <c r="B70" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="55" t="s">
+      <c r="C70" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="D70" s="57" t="n">
+      <c r="D70" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E70" s="57" t="n">
+      <c r="E70" s="59" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F70" s="59" t="n">
+      <c r="F70" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G70" s="60" t="n">
+      <c r="G70" s="62" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="55" t="s">
+      <c r="A71" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="B71" s="56" t="s">
+      <c r="B71" s="58" t="s">
         <v>172</v>
       </c>
-      <c r="C71" s="55" t="s">
+      <c r="C71" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="D71" s="57" t="n">
+      <c r="D71" s="59" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E71" s="57" t="n">
+      <c r="E71" s="59" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F71" s="59" t="n">
+      <c r="F71" s="61" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G71" s="60" t="n">
+      <c r="G71" s="62" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="55" t="s">
+      <c r="A72" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="B72" s="56" t="s">
+      <c r="B72" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="C72" s="55" t="s">
+      <c r="C72" s="57" t="s">
         <v>347</v>
       </c>
-      <c r="D72" s="57" t="n">
+      <c r="D72" s="59" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E72" s="57" t="n">
+      <c r="E72" s="59" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F72" s="59" t="n">
+      <c r="F72" s="61" t="n">
         <v>5.5009545454545</v>
       </c>
-      <c r="G72" s="60" t="n">
+      <c r="G72" s="62" t="n">
         <v>0.162483334922081</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="55" t="s">
+      <c r="A73" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="B73" s="56" t="s">
+      <c r="B73" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="C73" s="55" t="s">
+      <c r="C73" s="57" t="s">
         <v>347</v>
       </c>
-      <c r="D73" s="57" t="n">
+      <c r="D73" s="59" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E73" s="57" t="n">
+      <c r="E73" s="59" t="n">
         <v>30.1455</v>
       </c>
-      <c r="F73" s="59" t="n">
+      <c r="F73" s="61" t="n">
         <v>1.7909545454545</v>
       </c>
-      <c r="G73" s="60" t="n">
+      <c r="G73" s="62" t="n">
         <v>0.0594103446768007</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="55" t="s">
+      <c r="A74" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="B74" s="56" t="s">
+      <c r="B74" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="C74" s="55" t="s">
+      <c r="C74" s="57" t="s">
         <v>345</v>
       </c>
-      <c r="D74" s="57" t="n">
+      <c r="D74" s="59" t="n">
         <v>32.5</v>
       </c>
-      <c r="E74" s="57" t="n">
+      <c r="E74" s="59" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F74" s="59" t="n">
+      <c r="F74" s="61" t="n">
         <v>1.3555</v>
       </c>
-      <c r="G74" s="60" t="n">
+      <c r="G74" s="62" t="n">
         <v>0.0400378077417258</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Set all non-N/A text in Market Comparison to black
344 cells (mostly low-confidence match flags) were using a grey font
color; now black like the rest of the sheet. N/A stays red.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7vKGHgaJfNAAU7B1UJsH7
</commit_message>
<xml_diff>
--- a/output/RSEA_Comparison_Finished1.xlsx
+++ b/output/RSEA_Comparison_Finished1.xlsx
@@ -1140,16 +1140,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00_);[RED]&quot;($&quot;#,##0.00\)"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1258,6 +1257,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -1447,7 +1454,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1632,11 +1639,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1648,31 +1659,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1688,23 +1699,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1821,9 +1832,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>401040</xdr:colOff>
+      <xdr:colOff>400680</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>257400</xdr:rowOff>
+      <xdr:rowOff>257040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1837,7 +1848,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17428680" y="22115880"/>
-          <a:ext cx="2188800" cy="2334960"/>
+          <a:ext cx="2188440" cy="2334600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7828,8 +7839,8 @@
       <c r="AA7" s="45" t="n">
         <v>128.75</v>
       </c>
-      <c r="AB7" s="45"/>
-      <c r="AC7" s="45"/>
+      <c r="AB7" s="46"/>
+      <c r="AC7" s="46"/>
       <c r="AD7" s="11" t="n">
         <f aca="false">IF(COUNT(I7,J7,M7,O7,Q7,S7,U7,V7,Y7,AA7,AC7)=0,"N/A",MIN(I7,J7,M7,O7,Q7,S7,U7,V7,Y7,AA7,AC7))</f>
         <v>122.718181818182</v>
@@ -7935,8 +7946,8 @@
       <c r="AA8" s="45" t="n">
         <v>128.75</v>
       </c>
-      <c r="AB8" s="45"/>
-      <c r="AC8" s="45"/>
+      <c r="AB8" s="46"/>
+      <c r="AC8" s="46"/>
       <c r="AD8" s="11" t="n">
         <f aca="false">IF(COUNT(I8,J8,M8,O8,Q8,S8,U8,V8,Y8,AA8,AC8)=0,"N/A",MIN(I8,J8,M8,O8,Q8,S8,U8,V8,Y8,AA8,AC8))</f>
         <v>128.75</v>
@@ -8706,23 +8717,23 @@
       <c r="M15" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N15" s="46" t="n">
+      <c r="N15" s="47" t="n">
         <v>35.7</v>
       </c>
-      <c r="O15" s="46" t="n">
+      <c r="O15" s="47" t="n">
         <f aca="false">N15/1.1</f>
         <v>32.4545454545455</v>
       </c>
-      <c r="P15" s="46" t="n">
+      <c r="P15" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q15" s="46" t="n">
+      <c r="Q15" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R15" s="46" t="n">
+      <c r="R15" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="S15" s="46" t="n">
+      <c r="S15" s="47" t="n">
         <f aca="false">R15/1.1</f>
         <v>22.7272727272727</v>
       </c>
@@ -8738,10 +8749,10 @@
       <c r="W15" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X15" s="46" t="n">
+      <c r="X15" s="47" t="n">
         <v>35.07</v>
       </c>
-      <c r="Y15" s="46" t="n">
+      <c r="Y15" s="47" t="n">
         <f aca="false">X15/1.1</f>
         <v>31.8818181818182</v>
       </c>
@@ -8815,29 +8826,29 @@
       <c r="K16" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L16" s="46" t="n">
+      <c r="L16" s="47" t="n">
         <v>48.29</v>
       </c>
-      <c r="M16" s="46" t="n">
+      <c r="M16" s="47" t="n">
         <v>43.9</v>
       </c>
-      <c r="N16" s="46" t="n">
+      <c r="N16" s="47" t="n">
         <v>39.95</v>
       </c>
-      <c r="O16" s="46" t="n">
+      <c r="O16" s="47" t="n">
         <f aca="false">N16/1.1</f>
         <v>36.3181818181818</v>
       </c>
-      <c r="P16" s="46" t="n">
+      <c r="P16" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q16" s="46" t="n">
+      <c r="Q16" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R16" s="46" t="n">
+      <c r="R16" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="S16" s="46" t="n">
+      <c r="S16" s="47" t="n">
         <f aca="false">R16/1.1</f>
         <v>25</v>
       </c>
@@ -8847,17 +8858,17 @@
       <c r="U16" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="V16" s="46" t="n">
+      <c r="V16" s="47" t="n">
         <v>21.9</v>
       </c>
-      <c r="W16" s="46" t="n">
+      <c r="W16" s="47" t="n">
         <f aca="false">V16*1.1</f>
         <v>24.09</v>
       </c>
-      <c r="X16" s="46" t="n">
+      <c r="X16" s="47" t="n">
         <v>42.75</v>
       </c>
-      <c r="Y16" s="46" t="n">
+      <c r="Y16" s="47" t="n">
         <f aca="false">X16/1.1</f>
         <v>38.8636363636364</v>
       </c>
@@ -8931,29 +8942,29 @@
       <c r="K17" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L17" s="46" t="n">
+      <c r="L17" s="47" t="n">
         <v>53.63</v>
       </c>
-      <c r="M17" s="46" t="n">
+      <c r="M17" s="47" t="n">
         <v>48.75</v>
       </c>
-      <c r="N17" s="46" t="n">
+      <c r="N17" s="47" t="n">
         <v>35.7</v>
       </c>
-      <c r="O17" s="46" t="n">
+      <c r="O17" s="47" t="n">
         <f aca="false">N17/1.1</f>
         <v>32.4545454545455</v>
       </c>
-      <c r="P17" s="46" t="n">
+      <c r="P17" s="47" t="n">
         <v>11.55</v>
       </c>
-      <c r="Q17" s="46" t="n">
+      <c r="Q17" s="47" t="n">
         <v>10.5</v>
       </c>
-      <c r="R17" s="46" t="n">
+      <c r="R17" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="S17" s="46" t="n">
+      <c r="S17" s="47" t="n">
         <f aca="false">R17/1.1</f>
         <v>22.7272727272727</v>
       </c>
@@ -8969,10 +8980,10 @@
       <c r="W17" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X17" s="46" t="n">
+      <c r="X17" s="47" t="n">
         <v>35.07</v>
       </c>
-      <c r="Y17" s="46" t="n">
+      <c r="Y17" s="47" t="n">
         <f aca="false">X17/1.1</f>
         <v>31.8818181818182</v>
       </c>
@@ -9052,10 +9063,10 @@
       <c r="M18" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N18" s="46" t="n">
+      <c r="N18" s="47" t="n">
         <v>49.5</v>
       </c>
-      <c r="O18" s="46" t="n">
+      <c r="O18" s="47" t="n">
         <f aca="false">N18/1.1</f>
         <v>45</v>
       </c>
@@ -9163,10 +9174,10 @@
       <c r="K19" s="11" t="n">
         <v>99.23</v>
       </c>
-      <c r="L19" s="46" t="n">
+      <c r="L19" s="47" t="n">
         <v>61.59</v>
       </c>
-      <c r="M19" s="46" t="n">
+      <c r="M19" s="47" t="n">
         <v>55.99</v>
       </c>
       <c r="N19" s="11" t="n">
@@ -9416,10 +9427,10 @@
       <c r="Q21" s="11" t="n">
         <v>40.91</v>
       </c>
-      <c r="R21" s="46" t="n">
+      <c r="R21" s="47" t="n">
         <v>37.07</v>
       </c>
-      <c r="S21" s="46" t="n">
+      <c r="S21" s="47" t="n">
         <f aca="false">R21/1.1</f>
         <v>33.7</v>
       </c>
@@ -9745,36 +9756,36 @@
       <c r="K24" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L24" s="46" t="n">
+      <c r="L24" s="47" t="n">
         <v>43.15</v>
       </c>
-      <c r="M24" s="46" t="n">
+      <c r="M24" s="47" t="n">
         <v>39.23</v>
       </c>
-      <c r="N24" s="46" t="n">
+      <c r="N24" s="47" t="n">
         <v>35.75</v>
       </c>
-      <c r="O24" s="46" t="n">
+      <c r="O24" s="47" t="n">
         <f aca="false">N24/1.1</f>
         <v>32.5</v>
       </c>
-      <c r="P24" s="46" t="n">
+      <c r="P24" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q24" s="46" t="n">
+      <c r="Q24" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R24" s="46" t="n">
+      <c r="R24" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="S24" s="46" t="n">
+      <c r="S24" s="47" t="n">
         <f aca="false">R24/1.1</f>
         <v>22.7272727272727</v>
       </c>
-      <c r="T24" s="46" t="n">
+      <c r="T24" s="47" t="n">
         <v>33.19</v>
       </c>
-      <c r="U24" s="46" t="n">
+      <c r="U24" s="47" t="n">
         <f aca="false">T24/1.1</f>
         <v>30.1727272727273</v>
       </c>
@@ -9784,10 +9795,10 @@
       <c r="W24" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X24" s="46" t="n">
+      <c r="X24" s="47" t="n">
         <v>35.9</v>
       </c>
-      <c r="Y24" s="46" t="n">
+      <c r="Y24" s="47" t="n">
         <f aca="false">X24/1.1</f>
         <v>32.6363636363636</v>
       </c>
@@ -9860,10 +9871,10 @@
       <c r="K25" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L25" s="46" t="n">
+      <c r="L25" s="47" t="n">
         <v>46.29</v>
       </c>
-      <c r="M25" s="46" t="n">
+      <c r="M25" s="47" t="n">
         <v>42.08</v>
       </c>
       <c r="N25" s="11" t="n">
@@ -10092,10 +10103,10 @@
       <c r="K27" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L27" s="46" t="n">
+      <c r="L27" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M27" s="46" t="n">
+      <c r="M27" s="47" t="n">
         <v>35.98</v>
       </c>
       <c r="N27" s="11" t="n">
@@ -10260,10 +10271,10 @@
       <c r="AA28" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB28" s="46" t="n">
+      <c r="AB28" s="47" t="n">
         <v>90.08</v>
       </c>
-      <c r="AC28" s="46" t="n">
+      <c r="AC28" s="47" t="n">
         <f aca="false">AB28/1.1</f>
         <v>81.8909090909091</v>
       </c>
@@ -10492,10 +10503,10 @@
       <c r="AA30" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB30" s="46" t="n">
+      <c r="AB30" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC30" s="46" t="n">
+      <c r="AC30" s="47" t="n">
         <f aca="false">AB30/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10587,10 +10598,10 @@
         <f aca="false">T31/1.1</f>
         <v>42.8545454545455</v>
       </c>
-      <c r="V31" s="46" t="n">
+      <c r="V31" s="47" t="n">
         <v>28</v>
       </c>
-      <c r="W31" s="46" t="n">
+      <c r="W31" s="47" t="n">
         <f aca="false">V31*1.1</f>
         <v>30.8</v>
       </c>
@@ -10607,8 +10618,8 @@
       <c r="AA31" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB31" s="47"/>
-      <c r="AC31" s="47"/>
+      <c r="AB31" s="48"/>
+      <c r="AC31" s="48"/>
       <c r="AD31" s="11" t="n">
         <f aca="false">IF(COUNT(I31,J31,M31,O31,Q31,S31,U31,V31,Y31,AA31,AC31)=0,"N/A",MIN(I31,J31,M31,O31,Q31,S31,U31,V31,Y31,AA31,AC31))</f>
         <v>28</v>
@@ -10717,10 +10728,10 @@
       <c r="AA32" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB32" s="46" t="n">
+      <c r="AB32" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC32" s="46" t="n">
+      <c r="AC32" s="47" t="n">
         <f aca="false">AB32/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10787,10 +10798,10 @@
       <c r="M33" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N33" s="46" t="n">
+      <c r="N33" s="47" t="n">
         <v>51</v>
       </c>
-      <c r="O33" s="46" t="n">
+      <c r="O33" s="47" t="n">
         <f aca="false">N33/1.1</f>
         <v>46.3636363636364</v>
       </c>
@@ -10814,10 +10825,10 @@
         <f aca="false">T33/1.1</f>
         <v>53.4909090909091</v>
       </c>
-      <c r="V33" s="46" t="n">
+      <c r="V33" s="47" t="n">
         <v>51.5</v>
       </c>
-      <c r="W33" s="46" t="n">
+      <c r="W33" s="47" t="n">
         <f aca="false">V33*1.1</f>
         <v>56.65</v>
       </c>
@@ -10834,10 +10845,10 @@
       <c r="AA33" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB33" s="46" t="n">
+      <c r="AB33" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC33" s="46" t="n">
+      <c r="AC33" s="47" t="n">
         <f aca="false">AB33/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -10950,10 +10961,10 @@
       <c r="AA34" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB34" s="46" t="n">
+      <c r="AB34" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC34" s="46" t="n">
+      <c r="AC34" s="47" t="n">
         <f aca="false">AB34/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11066,10 +11077,10 @@
       <c r="AA35" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB35" s="46" t="n">
+      <c r="AB35" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC35" s="46" t="n">
+      <c r="AC35" s="47" t="n">
         <f aca="false">AB35/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11183,10 +11194,10 @@
       <c r="AA36" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB36" s="46" t="n">
+      <c r="AB36" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC36" s="46" t="n">
+      <c r="AC36" s="47" t="n">
         <f aca="false">AB36/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11297,10 +11308,10 @@
       <c r="AA37" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB37" s="46" t="n">
+      <c r="AB37" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC37" s="46" t="n">
+      <c r="AC37" s="47" t="n">
         <f aca="false">AB37/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11412,10 +11423,10 @@
       <c r="AA38" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB38" s="46" t="n">
+      <c r="AB38" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC38" s="46" t="n">
+      <c r="AC38" s="47" t="n">
         <f aca="false">AB38/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11528,10 +11539,10 @@
       <c r="AA39" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB39" s="46" t="n">
+      <c r="AB39" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC39" s="46" t="n">
+      <c r="AC39" s="47" t="n">
         <f aca="false">AB39/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11644,10 +11655,10 @@
       <c r="AA40" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB40" s="46" t="n">
+      <c r="AB40" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC40" s="46" t="n">
+      <c r="AC40" s="47" t="n">
         <f aca="false">AB40/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11760,10 +11771,10 @@
       <c r="AA41" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB41" s="46" t="n">
+      <c r="AB41" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC41" s="46" t="n">
+      <c r="AC41" s="47" t="n">
         <f aca="false">AB41/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11876,10 +11887,10 @@
       <c r="AA42" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB42" s="46" t="n">
+      <c r="AB42" s="47" t="n">
         <v>40.83</v>
       </c>
-      <c r="AC42" s="46" t="n">
+      <c r="AC42" s="47" t="n">
         <f aca="false">AB42/1.1</f>
         <v>37.1181818181818</v>
       </c>
@@ -11951,16 +11962,16 @@
       <c r="O43" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P43" s="46" t="n">
+      <c r="P43" s="47" t="n">
         <v>22.05</v>
       </c>
-      <c r="Q43" s="46" t="n">
+      <c r="Q43" s="47" t="n">
         <v>20.05</v>
       </c>
-      <c r="R43" s="46" t="n">
+      <c r="R43" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="S43" s="46" t="n">
+      <c r="S43" s="47" t="n">
         <f aca="false">R43/1.1</f>
         <v>25</v>
       </c>
@@ -11976,19 +11987,19 @@
       <c r="W43" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X43" s="46" t="n">
+      <c r="X43" s="47" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y43" s="46" t="n">
+      <c r="Y43" s="47" t="n">
         <f aca="false">X43/1.1</f>
         <v>29.0545454545455</v>
       </c>
-      <c r="Z43" s="47"/>
-      <c r="AA43" s="47"/>
-      <c r="AB43" s="46" t="n">
+      <c r="Z43" s="48"/>
+      <c r="AA43" s="48"/>
+      <c r="AB43" s="47" t="n">
         <v>35.9</v>
       </c>
-      <c r="AC43" s="46" t="n">
+      <c r="AC43" s="47" t="n">
         <f aca="false">AB43/1.1</f>
         <v>32.6363636363636</v>
       </c>
@@ -12067,10 +12078,10 @@
       <c r="Q44" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="R44" s="46" t="n">
+      <c r="R44" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S44" s="46" t="n">
+      <c r="S44" s="47" t="n">
         <f aca="false">R44/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -12203,10 +12214,10 @@
       <c r="W45" s="11" t="n">
         <v>26.5</v>
       </c>
-      <c r="X45" s="46" t="n">
+      <c r="X45" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y45" s="46" t="n">
+      <c r="Y45" s="47" t="n">
         <f aca="false">X45/1.1</f>
         <v>41.6</v>
       </c>
@@ -12280,16 +12291,16 @@
       <c r="K46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L46" s="46" t="n">
+      <c r="L46" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M46" s="46" t="n">
+      <c r="M46" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N46" s="46" t="n">
+      <c r="N46" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="O46" s="46" t="n">
+      <c r="O46" s="47" t="n">
         <f aca="false">N46/1.1</f>
         <v>25</v>
       </c>
@@ -12299,10 +12310,10 @@
       <c r="Q46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R46" s="46" t="n">
+      <c r="R46" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S46" s="46" t="n">
+      <c r="S46" s="47" t="n">
         <f aca="false">R46/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -12318,10 +12329,10 @@
       <c r="W46" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X46" s="46" t="n">
+      <c r="X46" s="47" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y46" s="46" t="n">
+      <c r="Y46" s="47" t="n">
         <f aca="false">X46/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -12395,50 +12406,50 @@
       <c r="K47" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L47" s="46" t="n">
+      <c r="L47" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M47" s="46" t="n">
+      <c r="M47" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N47" s="46" t="n">
+      <c r="N47" s="47" t="n">
         <v>42.5</v>
       </c>
-      <c r="O47" s="46" t="n">
+      <c r="O47" s="47" t="n">
         <f aca="false">N47/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P47" s="46" t="n">
+      <c r="P47" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q47" s="46" t="n">
+      <c r="Q47" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R47" s="46" t="n">
+      <c r="R47" s="47" t="n">
         <v>30</v>
       </c>
-      <c r="S47" s="46" t="n">
+      <c r="S47" s="47" t="n">
         <f aca="false">R47/1.1</f>
         <v>27.2727272727273</v>
       </c>
-      <c r="T47" s="46" t="n">
+      <c r="T47" s="47" t="n">
         <v>28.66</v>
       </c>
-      <c r="U47" s="46" t="n">
+      <c r="U47" s="47" t="n">
         <f aca="false">T47/1.1</f>
         <v>26.0545454545455</v>
       </c>
-      <c r="V47" s="46" t="n">
+      <c r="V47" s="47" t="n">
         <v>36.5</v>
       </c>
-      <c r="W47" s="46" t="n">
+      <c r="W47" s="47" t="n">
         <f aca="false">V47*1.1</f>
         <v>40.15</v>
       </c>
-      <c r="X47" s="46" t="n">
+      <c r="X47" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y47" s="46" t="n">
+      <c r="Y47" s="47" t="n">
         <f aca="false">X47/1.1</f>
         <v>41.6</v>
       </c>
@@ -12512,43 +12523,43 @@
       <c r="K48" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L48" s="46" t="n">
+      <c r="L48" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M48" s="46" t="n">
+      <c r="M48" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N48" s="46" t="n">
+      <c r="N48" s="47" t="n">
         <v>42.5</v>
       </c>
-      <c r="O48" s="46" t="n">
+      <c r="O48" s="47" t="n">
         <f aca="false">N48/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P48" s="46" t="n">
+      <c r="P48" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q48" s="46" t="n">
+      <c r="Q48" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R48" s="46" t="n">
+      <c r="R48" s="47" t="n">
         <v>33.5</v>
       </c>
-      <c r="S48" s="46" t="n">
+      <c r="S48" s="47" t="n">
         <f aca="false">R48/1.1</f>
         <v>30.4545454545455</v>
       </c>
-      <c r="T48" s="46" t="n">
+      <c r="T48" s="47" t="n">
         <v>18.41</v>
       </c>
-      <c r="U48" s="46" t="n">
+      <c r="U48" s="47" t="n">
         <f aca="false">T48/1.1</f>
         <v>16.7363636363636</v>
       </c>
-      <c r="V48" s="46" t="n">
+      <c r="V48" s="47" t="n">
         <v>28.5</v>
       </c>
-      <c r="W48" s="46" t="n">
+      <c r="W48" s="47" t="n">
         <f aca="false">V48*1.1</f>
         <v>31.35</v>
       </c>
@@ -12634,17 +12645,17 @@
       <c r="M49" s="11" t="n">
         <v>31.52</v>
       </c>
-      <c r="N49" s="46" t="n">
+      <c r="N49" s="47" t="n">
         <v>35.4</v>
       </c>
-      <c r="O49" s="46" t="n">
+      <c r="O49" s="47" t="n">
         <f aca="false">N49/1.1</f>
         <v>32.1818181818182</v>
       </c>
-      <c r="P49" s="46" t="n">
+      <c r="P49" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q49" s="46" t="n">
+      <c r="Q49" s="47" t="n">
         <v>22</v>
       </c>
       <c r="R49" s="11" t="n">
@@ -12668,10 +12679,10 @@
       <c r="W49" s="11" t="n">
         <v>21.9</v>
       </c>
-      <c r="X49" s="46" t="n">
+      <c r="X49" s="47" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y49" s="46" t="n">
+      <c r="Y49" s="47" t="n">
         <f aca="false">X49/1.1</f>
         <v>29.0545454545455</v>
       </c>
@@ -12862,43 +12873,43 @@
       <c r="K51" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L51" s="46" t="n">
+      <c r="L51" s="47" t="n">
         <v>34.67</v>
       </c>
-      <c r="M51" s="46" t="n">
+      <c r="M51" s="47" t="n">
         <v>31.52</v>
       </c>
-      <c r="N51" s="46" t="n">
+      <c r="N51" s="47" t="n">
         <v>28.3</v>
       </c>
-      <c r="O51" s="46" t="n">
+      <c r="O51" s="47" t="n">
         <f aca="false">N51/1.1</f>
         <v>25.7272727272727</v>
       </c>
-      <c r="P51" s="46" t="n">
+      <c r="P51" s="47" t="n">
         <v>11.55</v>
       </c>
-      <c r="Q51" s="46" t="n">
+      <c r="Q51" s="47" t="n">
         <v>10.5</v>
       </c>
-      <c r="R51" s="46" t="n">
+      <c r="R51" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S51" s="46" t="n">
+      <c r="S51" s="47" t="n">
         <f aca="false">R51/1.1</f>
         <v>20.4545454545455</v>
       </c>
-      <c r="T51" s="46" t="n">
+      <c r="T51" s="47" t="n">
         <v>33.04</v>
       </c>
-      <c r="U51" s="46" t="n">
+      <c r="U51" s="47" t="n">
         <f aca="false">T51/1.1</f>
         <v>30.0363636363636</v>
       </c>
-      <c r="V51" s="46" t="n">
+      <c r="V51" s="47" t="n">
         <v>19.5</v>
       </c>
-      <c r="W51" s="46" t="n">
+      <c r="W51" s="47" t="n">
         <f aca="false">V51*1.1</f>
         <v>21.45</v>
       </c>
@@ -12978,29 +12989,29 @@
       <c r="K52" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L52" s="46" t="n">
+      <c r="L52" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M52" s="46" t="n">
+      <c r="M52" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N52" s="46" t="n">
+      <c r="N52" s="47" t="n">
         <v>42.5</v>
       </c>
-      <c r="O52" s="46" t="n">
+      <c r="O52" s="47" t="n">
         <f aca="false">N52/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P52" s="46" t="n">
+      <c r="P52" s="47" t="n">
         <v>45.15</v>
       </c>
-      <c r="Q52" s="46" t="n">
+      <c r="Q52" s="47" t="n">
         <v>41.05</v>
       </c>
-      <c r="R52" s="46" t="n">
+      <c r="R52" s="47" t="n">
         <v>33.5</v>
       </c>
-      <c r="S52" s="46" t="n">
+      <c r="S52" s="47" t="n">
         <f aca="false">R52/1.1</f>
         <v>30.4545454545455</v>
       </c>
@@ -13010,17 +13021,17 @@
       <c r="U52" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="V52" s="46" t="n">
+      <c r="V52" s="47" t="n">
         <v>26.5</v>
       </c>
-      <c r="W52" s="46" t="n">
+      <c r="W52" s="47" t="n">
         <f aca="false">V52*1.1</f>
         <v>29.15</v>
       </c>
-      <c r="X52" s="46" t="n">
+      <c r="X52" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y52" s="46" t="n">
+      <c r="Y52" s="47" t="n">
         <f aca="false">X52/1.1</f>
         <v>41.6</v>
       </c>
@@ -13031,8 +13042,8 @@
       <c r="AA52" s="45" t="n">
         <v>70.25</v>
       </c>
-      <c r="AB52" s="45"/>
-      <c r="AC52" s="45"/>
+      <c r="AB52" s="46"/>
+      <c r="AC52" s="46"/>
       <c r="AD52" s="11" t="n">
         <f aca="false">IF(COUNT(I52,J52,M52,O52,Q52,S52,U52,V52,Y52,AA52,AC52)=0,"N/A",MIN(I52,J52,M52,O52,Q52,S52,U52,V52,Y52,AA52,AC52))</f>
         <v>26.5</v>
@@ -13200,16 +13211,16 @@
       <c r="K54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L54" s="46" t="n">
+      <c r="L54" s="47" t="n">
         <v>34.67</v>
       </c>
-      <c r="M54" s="46" t="n">
+      <c r="M54" s="47" t="n">
         <v>31.52</v>
       </c>
-      <c r="N54" s="46" t="n">
+      <c r="N54" s="47" t="n">
         <v>28.3</v>
       </c>
-      <c r="O54" s="46" t="n">
+      <c r="O54" s="47" t="n">
         <f aca="false">N54/1.1</f>
         <v>25.7272727272727</v>
       </c>
@@ -13219,10 +13230,10 @@
       <c r="Q54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R54" s="46" t="n">
+      <c r="R54" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S54" s="46" t="n">
+      <c r="S54" s="47" t="n">
         <f aca="false">R54/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -13238,10 +13249,10 @@
       <c r="W54" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X54" s="46" t="n">
+      <c r="X54" s="47" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y54" s="46" t="n">
+      <c r="Y54" s="47" t="n">
         <f aca="false">X54/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -13333,10 +13344,10 @@
       <c r="Q55" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R55" s="46" t="n">
+      <c r="R55" s="47" t="n">
         <v>23</v>
       </c>
-      <c r="S55" s="46" t="n">
+      <c r="S55" s="47" t="n">
         <f aca="false">R55/1.1</f>
         <v>20.9090909090909</v>
       </c>
@@ -13364,8 +13375,8 @@
       <c r="AA55" s="42" t="s">
         <v>309</v>
       </c>
-      <c r="AB55" s="47"/>
-      <c r="AC55" s="47"/>
+      <c r="AB55" s="48"/>
+      <c r="AC55" s="48"/>
       <c r="AD55" s="11" t="n">
         <f aca="false">IF(COUNT(I55,J55,M55,O55,Q55,S55,U55,V55,Y55,AA55,AC55)=0,"N/A",MIN(I55,J55,M55,O55,Q55,S55,U55,V55,Y55,AA55,AC55))</f>
         <v>20.9090909090909</v>
@@ -13434,16 +13445,16 @@
       <c r="O56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P56" s="46" t="n">
+      <c r="P56" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q56" s="46" t="n">
+      <c r="Q56" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R56" s="46" t="n">
+      <c r="R56" s="47" t="n">
         <v>33.5</v>
       </c>
-      <c r="S56" s="46" t="n">
+      <c r="S56" s="47" t="n">
         <f aca="false">R56/1.1</f>
         <v>30.4545454545455</v>
       </c>
@@ -13459,10 +13470,10 @@
       <c r="W56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X56" s="46" t="n">
+      <c r="X56" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y56" s="46" t="n">
+      <c r="Y56" s="47" t="n">
         <f aca="false">X56/1.1</f>
         <v>41.6</v>
       </c>
@@ -13472,8 +13483,8 @@
       <c r="AA56" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="AB56" s="47"/>
-      <c r="AC56" s="47"/>
+      <c r="AB56" s="48"/>
+      <c r="AC56" s="48"/>
       <c r="AD56" s="11" t="n">
         <f aca="false">IF(COUNT(I56,J56,M56,O56,Q56,S56,U56,V56,Y56,AA56,AC56)=0,"N/A",MIN(I56,J56,M56,O56,Q56,S56,U56,V56,Y56,AA56,AC56))</f>
         <v>22</v>
@@ -13530,10 +13541,10 @@
       <c r="K57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L57" s="46" t="n">
+      <c r="L57" s="47" t="n">
         <v>39.47</v>
       </c>
-      <c r="M57" s="46" t="n">
+      <c r="M57" s="47" t="n">
         <v>35.88</v>
       </c>
       <c r="N57" s="42" t="s">
@@ -13548,10 +13559,10 @@
       <c r="Q57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R57" s="46" t="n">
+      <c r="R57" s="47" t="n">
         <v>30</v>
       </c>
-      <c r="S57" s="46" t="n">
+      <c r="S57" s="47" t="n">
         <f aca="false">R57/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -13567,10 +13578,10 @@
       <c r="W57" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X57" s="46" t="n">
+      <c r="X57" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y57" s="46" t="n">
+      <c r="Y57" s="47" t="n">
         <f aca="false">X57/1.1</f>
         <v>41.6</v>
       </c>
@@ -13650,23 +13661,23 @@
       <c r="M58" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N58" s="46" t="n">
+      <c r="N58" s="47" t="n">
         <v>42.5</v>
       </c>
-      <c r="O58" s="46" t="n">
+      <c r="O58" s="47" t="n">
         <f aca="false">N58/1.1</f>
         <v>38.6363636363636</v>
       </c>
-      <c r="P58" s="46" t="n">
+      <c r="P58" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q58" s="46" t="n">
+      <c r="Q58" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R58" s="46" t="n">
+      <c r="R58" s="47" t="n">
         <v>30</v>
       </c>
-      <c r="S58" s="46" t="n">
+      <c r="S58" s="47" t="n">
         <f aca="false">R58/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -13682,10 +13693,10 @@
       <c r="W58" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X58" s="46" t="n">
+      <c r="X58" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y58" s="46" t="n">
+      <c r="Y58" s="47" t="n">
         <f aca="false">X58/1.1</f>
         <v>41.6</v>
       </c>
@@ -13765,10 +13776,10 @@
       <c r="M59" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="N59" s="46" t="n">
+      <c r="N59" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="O59" s="46" t="n">
+      <c r="O59" s="47" t="n">
         <f aca="false">N59/1.1</f>
         <v>25</v>
       </c>
@@ -13778,10 +13789,10 @@
       <c r="Q59" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R59" s="46" t="n">
+      <c r="R59" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="S59" s="46" t="n">
+      <c r="S59" s="47" t="n">
         <f aca="false">R59/1.1</f>
         <v>20</v>
       </c>
@@ -13909,10 +13920,10 @@
       <c r="W60" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X60" s="46" t="n">
+      <c r="X60" s="47" t="n">
         <v>41.4</v>
       </c>
-      <c r="Y60" s="46" t="n">
+      <c r="Y60" s="47" t="n">
         <f aca="false">X60/1.1</f>
         <v>37.6363636363636</v>
       </c>
@@ -13986,16 +13997,16 @@
       <c r="K61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L61" s="46" t="n">
+      <c r="L61" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M61" s="46" t="n">
+      <c r="M61" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N61" s="46" t="n">
+      <c r="N61" s="47" t="n">
         <v>42.5</v>
       </c>
-      <c r="O61" s="46" t="n">
+      <c r="O61" s="47" t="n">
         <f aca="false">N61/1.1</f>
         <v>38.6363636363636</v>
       </c>
@@ -14005,10 +14016,10 @@
       <c r="Q61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="R61" s="46" t="n">
+      <c r="R61" s="47" t="n">
         <v>30</v>
       </c>
-      <c r="S61" s="46" t="n">
+      <c r="S61" s="47" t="n">
         <f aca="false">R61/1.1</f>
         <v>27.2727272727273</v>
       </c>
@@ -14024,10 +14035,10 @@
       <c r="W61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X61" s="46" t="n">
+      <c r="X61" s="47" t="n">
         <v>45.76</v>
       </c>
-      <c r="Y61" s="46" t="n">
+      <c r="Y61" s="47" t="n">
         <f aca="false">X61/1.1</f>
         <v>41.6</v>
       </c>
@@ -14101,29 +14112,29 @@
       <c r="K62" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L62" s="46" t="n">
+      <c r="L62" s="47" t="n">
         <v>39.47</v>
       </c>
-      <c r="M62" s="46" t="n">
+      <c r="M62" s="47" t="n">
         <v>35.88</v>
       </c>
-      <c r="N62" s="46" t="n">
+      <c r="N62" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="O62" s="46" t="n">
+      <c r="O62" s="47" t="n">
         <f aca="false">N62/1.1</f>
         <v>25</v>
       </c>
-      <c r="P62" s="46" t="n">
+      <c r="P62" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q62" s="46" t="n">
+      <c r="Q62" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R62" s="46" t="n">
+      <c r="R62" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S62" s="46" t="n">
+      <c r="S62" s="47" t="n">
         <f aca="false">R62/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -14139,10 +14150,10 @@
       <c r="W62" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X62" s="46" t="n">
+      <c r="X62" s="47" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y62" s="46" t="n">
+      <c r="Y62" s="47" t="n">
         <f aca="false">X62/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -14216,10 +14227,10 @@
       <c r="K63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L63" s="46" t="n">
+      <c r="L63" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M63" s="46" t="n">
+      <c r="M63" s="47" t="n">
         <v>35.98</v>
       </c>
       <c r="N63" s="42" t="s">
@@ -14228,16 +14239,16 @@
       <c r="O63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="P63" s="46" t="n">
+      <c r="P63" s="47" t="n">
         <v>22.6</v>
       </c>
-      <c r="Q63" s="46" t="n">
+      <c r="Q63" s="47" t="n">
         <v>20.55</v>
       </c>
-      <c r="R63" s="46" t="n">
+      <c r="R63" s="47" t="n">
         <v>23</v>
       </c>
-      <c r="S63" s="46" t="n">
+      <c r="S63" s="47" t="n">
         <f aca="false">R63/1.1</f>
         <v>20.9090909090909</v>
       </c>
@@ -14253,10 +14264,10 @@
       <c r="W63" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X63" s="46" t="n">
+      <c r="X63" s="47" t="n">
         <v>31.96</v>
       </c>
-      <c r="Y63" s="46" t="n">
+      <c r="Y63" s="47" t="n">
         <f aca="false">X63/1.1</f>
         <v>29.0545454545455</v>
       </c>
@@ -14330,29 +14341,29 @@
       <c r="K64" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L64" s="46" t="n">
+      <c r="L64" s="47" t="n">
         <v>39.58</v>
       </c>
-      <c r="M64" s="46" t="n">
+      <c r="M64" s="47" t="n">
         <v>35.98</v>
       </c>
-      <c r="N64" s="46" t="n">
+      <c r="N64" s="47" t="n">
         <v>27.5</v>
       </c>
-      <c r="O64" s="46" t="n">
+      <c r="O64" s="47" t="n">
         <f aca="false">N64/1.1</f>
         <v>25</v>
       </c>
-      <c r="P64" s="46" t="n">
+      <c r="P64" s="47" t="n">
         <v>24.2</v>
       </c>
-      <c r="Q64" s="46" t="n">
+      <c r="Q64" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="R64" s="46" t="n">
+      <c r="R64" s="47" t="n">
         <v>22.5</v>
       </c>
-      <c r="S64" s="46" t="n">
+      <c r="S64" s="47" t="n">
         <f aca="false">R64/1.1</f>
         <v>20.4545454545455</v>
       </c>
@@ -14368,10 +14379,10 @@
       <c r="W64" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="X64" s="46" t="n">
+      <c r="X64" s="47" t="n">
         <v>24.96</v>
       </c>
-      <c r="Y64" s="46" t="n">
+      <c r="Y64" s="47" t="n">
         <f aca="false">X64/1.1</f>
         <v>22.6909090909091</v>
       </c>
@@ -14445,10 +14456,10 @@
       <c r="K65" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="L65" s="46" t="n">
+      <c r="L65" s="47" t="n">
         <v>39.47</v>
       </c>
-      <c r="M65" s="46" t="n">
+      <c r="M65" s="47" t="n">
         <v>35.88</v>
       </c>
       <c r="N65" s="11" t="n">
@@ -14533,7 +14544,7 @@
       </c>
       <c r="B68" s="35"/>
       <c r="C68" s="35"/>
-      <c r="D68" s="48" t="n">
+      <c r="D68" s="49" t="n">
         <f aca="false">COUNTA(B6:B65)</f>
         <v>60</v>
       </c>
@@ -14544,7 +14555,7 @@
       </c>
       <c r="B69" s="35"/>
       <c r="C69" s="35"/>
-      <c r="D69" s="48" t="n">
+      <c r="D69" s="49" t="n">
         <f aca="false">COUNTIF(J6:J65,"&gt;0")+COUNTIF(M6:M65,"&gt;0")+COUNTIF(O6:O65,"&gt;0")+COUNTIF(Q6:Q65,"&gt;0")+COUNTIF(S6:S65,"&gt;0")+COUNTIF(U6:U65,"&gt;0")+COUNTIF(V6:V65,"&gt;0")+COUNTIF(Y6:Y65,"&gt;0")+COUNTIF(AA6:AA65,"&gt;0")+COUNTIF(AC6:AC65,"&gt;0")</f>
         <v>407</v>
       </c>
@@ -14555,7 +14566,7 @@
       </c>
       <c r="B70" s="35"/>
       <c r="C70" s="35"/>
-      <c r="D70" s="48" t="n">
+      <c r="D70" s="49" t="n">
         <f aca="false">COUNTIF(AE6:AE65,"&lt;0")</f>
         <v>53</v>
       </c>
@@ -14566,7 +14577,7 @@
       </c>
       <c r="B71" s="35"/>
       <c r="C71" s="35"/>
-      <c r="D71" s="48" t="n">
+      <c r="D71" s="49" t="n">
         <f aca="false">COUNTIF(AE6:AE65,"&gt;0")</f>
         <v>7</v>
       </c>
@@ -14577,7 +14588,7 @@
       </c>
       <c r="B72" s="35"/>
       <c r="C72" s="35"/>
-      <c r="D72" s="49" t="n">
+      <c r="D72" s="50" t="n">
         <f aca="false">AVERAGE(AE6:AE65)</f>
         <v>-0.454866678565887</v>
       </c>
@@ -14588,7 +14599,7 @@
       </c>
       <c r="B73" s="35"/>
       <c r="C73" s="35"/>
-      <c r="D73" s="49" t="n">
+      <c r="D73" s="50" t="n">
         <f aca="false">MEDIAN(AE6:AE65)</f>
         <v>-0.523652597402597</v>
       </c>
@@ -14599,7 +14610,7 @@
       </c>
       <c r="B74" s="35"/>
       <c r="C74" s="35"/>
-      <c r="D74" s="48" t="n">
+      <c r="D74" s="49" t="n">
         <f aca="false">COUNTIF(AF6:AF65,"&lt;0")</f>
         <v>15</v>
       </c>
@@ -14610,7 +14621,7 @@
       </c>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
-      <c r="D75" s="48" t="n">
+      <c r="D75" s="49" t="n">
         <f aca="false">COUNTIF(AF6:AF65,"&gt;0")</f>
         <v>7</v>
       </c>
@@ -14621,7 +14632,7 @@
       </c>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
-      <c r="D76" s="49" t="n">
+      <c r="D76" s="50" t="n">
         <f aca="false">AVERAGE(AF6:AF65)</f>
         <v>-0.137849955170021</v>
       </c>
@@ -14632,7 +14643,7 @@
       </c>
       <c r="B77" s="35"/>
       <c r="C77" s="35"/>
-      <c r="D77" s="49" t="n">
+      <c r="D77" s="50" t="n">
         <f aca="false">MEDIAN(AF6:AF65)</f>
         <v>-0.240924975181021</v>
       </c>
@@ -14699,62 +14710,62 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
     </row>
     <row r="2" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="52" t="s">
         <v>332</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="53" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="53" t="s">
         <v>333</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="53" t="s">
         <v>334</v>
       </c>
-      <c r="F4" s="52" t="s">
+      <c r="F4" s="53" t="s">
         <v>335</v>
       </c>
-      <c r="G4" s="52" t="s">
+      <c r="G4" s="53" t="s">
         <v>336</v>
       </c>
-      <c r="H4" s="52" t="s">
+      <c r="H4" s="53" t="s">
         <v>337</v>
       </c>
-      <c r="I4" s="52" t="s">
+      <c r="I4" s="53" t="s">
         <v>338</v>
       </c>
-      <c r="J4" s="52" t="s">
+      <c r="J4" s="53" t="s">
         <v>221</v>
       </c>
     </row>
@@ -14774,13 +14785,13 @@
       <c r="E5" s="11" t="n">
         <v>20.05</v>
       </c>
-      <c r="F5" s="53" t="n">
+      <c r="F5" s="54" t="n">
         <v>16.93275</v>
       </c>
-      <c r="G5" s="54" t="n">
+      <c r="G5" s="55" t="n">
         <v>-3.11725</v>
       </c>
-      <c r="H5" s="55" t="n">
+      <c r="H5" s="56" t="n">
         <v>-0.155473815461347</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -14803,13 +14814,13 @@
       <c r="E6" s="11" t="n">
         <v>122.718181818182</v>
       </c>
-      <c r="F6" s="56" t="n">
+      <c r="F6" s="57" t="n">
         <v>66.83</v>
       </c>
-      <c r="G6" s="54" t="n">
+      <c r="G6" s="55" t="n">
         <v>-55.888181818182</v>
       </c>
-      <c r="H6" s="55" t="n">
+      <c r="H6" s="56" t="n">
         <v>-0.455418919919995</v>
       </c>
       <c r="I6" s="1" t="s">
@@ -14832,13 +14843,13 @@
       <c r="E7" s="11" t="n">
         <v>128.75</v>
       </c>
-      <c r="F7" s="56" t="n">
+      <c r="F7" s="57" t="n">
         <v>44.55</v>
       </c>
-      <c r="G7" s="54" t="n">
+      <c r="G7" s="55" t="n">
         <v>-84.2</v>
       </c>
-      <c r="H7" s="55" t="n">
+      <c r="H7" s="56" t="n">
         <v>-0.653980582524272</v>
       </c>
       <c r="I7" s="1" t="s">
@@ -14861,13 +14872,13 @@
       <c r="E8" s="11" t="n">
         <v>69.245</v>
       </c>
-      <c r="F8" s="53" t="n">
+      <c r="F8" s="54" t="n">
         <v>45.144</v>
       </c>
-      <c r="G8" s="54" t="n">
+      <c r="G8" s="55" t="n">
         <v>-24.101</v>
       </c>
-      <c r="H8" s="55" t="n">
+      <c r="H8" s="56" t="n">
         <v>-0.348054011119937</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -14890,13 +14901,13 @@
       <c r="E9" s="11" t="n">
         <v>81.4</v>
       </c>
-      <c r="F9" s="53" t="n">
+      <c r="F9" s="54" t="n">
         <v>70.538125</v>
       </c>
-      <c r="G9" s="54" t="n">
+      <c r="G9" s="55" t="n">
         <v>-10.861875</v>
       </c>
-      <c r="H9" s="55" t="n">
+      <c r="H9" s="56" t="n">
         <v>-0.133438267813268</v>
       </c>
       <c r="I9" s="1" t="s">
@@ -14919,13 +14930,13 @@
       <c r="E10" s="11" t="n">
         <v>44.209</v>
       </c>
-      <c r="F10" s="53" t="n">
+      <c r="F10" s="54" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G10" s="54" t="n">
+      <c r="G10" s="55" t="n">
         <v>-10.3535</v>
       </c>
-      <c r="H10" s="55" t="n">
+      <c r="H10" s="56" t="n">
         <v>-0.234194394806487</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -14948,13 +14959,13 @@
       <c r="E11" s="11" t="n">
         <v>70.36</v>
       </c>
-      <c r="F11" s="53" t="n">
+      <c r="F11" s="54" t="n">
         <v>45.144</v>
       </c>
-      <c r="G11" s="54" t="n">
+      <c r="G11" s="55" t="n">
         <v>-25.216</v>
       </c>
-      <c r="H11" s="55" t="n">
+      <c r="H11" s="56" t="n">
         <v>-0.358385446276293</v>
       </c>
       <c r="I11" s="1" t="s">
@@ -14962,34 +14973,34 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="57" t="s">
+      <c r="A12" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="58" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="57" t="s">
+      <c r="D12" s="58" t="s">
         <v>345</v>
       </c>
-      <c r="E12" s="59" t="n">
+      <c r="E12" s="60" t="n">
         <v>33.1818181818182</v>
       </c>
-      <c r="F12" s="60" t="n">
+      <c r="F12" s="61" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="62" t="n">
         <v>0.673681818181798</v>
       </c>
-      <c r="H12" s="62" t="n">
+      <c r="H12" s="63" t="n">
         <v>0.0203027397260268</v>
       </c>
-      <c r="I12" s="63" t="s">
+      <c r="I12" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J12" s="57"/>
+      <c r="J12" s="58"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -15007,13 +15018,13 @@
       <c r="E13" s="11" t="n">
         <v>43.09</v>
       </c>
-      <c r="F13" s="53" t="n">
+      <c r="F13" s="54" t="n">
         <v>25.394125</v>
       </c>
-      <c r="G13" s="54" t="n">
+      <c r="G13" s="55" t="n">
         <v>-17.695875</v>
       </c>
-      <c r="H13" s="55" t="n">
+      <c r="H13" s="56" t="n">
         <v>-0.410672429798097</v>
       </c>
       <c r="I13" s="1" t="s">
@@ -15036,13 +15047,13 @@
       <c r="E14" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F14" s="53" t="n">
+      <c r="F14" s="54" t="n">
         <v>8.461375</v>
       </c>
-      <c r="G14" s="54" t="n">
+      <c r="G14" s="55" t="n">
         <v>-13.538625</v>
       </c>
-      <c r="H14" s="55" t="n">
+      <c r="H14" s="56" t="n">
         <v>-0.615392045454545</v>
       </c>
       <c r="I14" s="1" t="s">
@@ -15065,13 +15076,13 @@
       <c r="E15" s="11" t="n">
         <v>21.9</v>
       </c>
-      <c r="F15" s="53" t="n">
+      <c r="F15" s="54" t="n">
         <v>15.81275</v>
       </c>
-      <c r="G15" s="54" t="n">
+      <c r="G15" s="55" t="n">
         <v>-6.08725</v>
       </c>
-      <c r="H15" s="55" t="n">
+      <c r="H15" s="56" t="n">
         <v>-0.277956621004566</v>
       </c>
       <c r="I15" s="1" t="s">
@@ -15094,13 +15105,13 @@
       <c r="E16" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="F16" s="53" t="n">
+      <c r="F16" s="54" t="n">
         <v>8.461375</v>
       </c>
-      <c r="G16" s="54" t="n">
+      <c r="G16" s="55" t="n">
         <v>-2.038625</v>
       </c>
-      <c r="H16" s="55" t="n">
+      <c r="H16" s="56" t="n">
         <v>-0.194154761904762</v>
       </c>
       <c r="I16" s="1" t="s">
@@ -15123,13 +15134,13 @@
       <c r="E17" s="11" t="n">
         <v>37.3909090909091</v>
       </c>
-      <c r="F17" s="53" t="n">
+      <c r="F17" s="54" t="n">
         <v>30.1455</v>
       </c>
-      <c r="G17" s="54" t="n">
+      <c r="G17" s="55" t="n">
         <v>-7.2454090909091</v>
       </c>
-      <c r="H17" s="55" t="n">
+      <c r="H17" s="56" t="n">
         <v>-0.193774617067834</v>
       </c>
       <c r="I17" s="1" t="s">
@@ -15137,34 +15148,34 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B18" s="57" t="s">
+      <c r="B18" s="58" t="s">
         <v>131</v>
       </c>
-      <c r="C18" s="58" t="s">
+      <c r="C18" s="59" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="57" t="s">
+      <c r="D18" s="58" t="s">
         <v>347</v>
       </c>
-      <c r="E18" s="59" t="n">
+      <c r="E18" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="F18" s="60" t="n">
+      <c r="F18" s="61" t="n">
         <v>30.1455</v>
       </c>
-      <c r="G18" s="61" t="n">
+      <c r="G18" s="62" t="n">
         <v>1.7909545454545</v>
       </c>
-      <c r="H18" s="62" t="n">
+      <c r="H18" s="63" t="n">
         <v>0.0631628727156122</v>
       </c>
-      <c r="I18" s="63" t="s">
+      <c r="I18" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J18" s="57"/>
+      <c r="J18" s="58"/>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -15182,13 +15193,13 @@
       <c r="E19" s="11" t="n">
         <v>23.3090909090909</v>
       </c>
-      <c r="F19" s="53" t="n">
+      <c r="F19" s="54" t="n">
         <v>16.93275</v>
       </c>
-      <c r="G19" s="54" t="n">
+      <c r="G19" s="55" t="n">
         <v>-6.3763409090909</v>
       </c>
-      <c r="H19" s="55" t="n">
+      <c r="H19" s="56" t="n">
         <v>-0.273555967238689</v>
       </c>
       <c r="I19" s="1" t="s">
@@ -15196,34 +15207,34 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="57" t="s">
+      <c r="A20" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B20" s="57" t="s">
+      <c r="B20" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="57" t="s">
+      <c r="D20" s="58" t="s">
         <v>348</v>
       </c>
-      <c r="E20" s="59" t="n">
+      <c r="E20" s="60" t="n">
         <v>33.7</v>
       </c>
-      <c r="F20" s="60" t="n">
+      <c r="F20" s="61" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G20" s="61" t="n">
+      <c r="G20" s="62" t="n">
         <v>0.155499999999996</v>
       </c>
-      <c r="H20" s="62" t="n">
+      <c r="H20" s="63" t="n">
         <v>0.00461424332344203</v>
       </c>
-      <c r="I20" s="63" t="s">
+      <c r="I20" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J20" s="57"/>
+      <c r="J20" s="58"/>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
@@ -15241,13 +15252,13 @@
       <c r="E21" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F21" s="53" t="n">
+      <c r="F21" s="54" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G21" s="54" t="n">
+      <c r="G21" s="55" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H21" s="55" t="n">
+      <c r="H21" s="56" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I21" s="1" t="s">
@@ -15270,13 +15281,13 @@
       <c r="E22" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F22" s="53" t="n">
+      <c r="F22" s="54" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G22" s="54" t="n">
+      <c r="G22" s="55" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H22" s="55" t="n">
+      <c r="H22" s="56" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I22" s="1" t="s">
@@ -15299,13 +15310,13 @@
       <c r="E23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F23" s="53" t="n">
+      <c r="F23" s="54" t="n">
         <v>6.011375</v>
       </c>
-      <c r="G23" s="54" t="n">
+      <c r="G23" s="55" t="n">
         <v>-15.988625</v>
       </c>
-      <c r="H23" s="55" t="n">
+      <c r="H23" s="56" t="n">
         <v>-0.726755681818182</v>
       </c>
       <c r="I23" s="1" t="s">
@@ -15313,64 +15324,64 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B24" s="57" t="s">
+      <c r="B24" s="58" t="s">
         <v>159</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D24" s="57" t="s">
+      <c r="D24" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="E24" s="59" t="n">
+      <c r="E24" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F24" s="60" t="n">
+      <c r="F24" s="61" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G24" s="61" t="n">
+      <c r="G24" s="62" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="H24" s="62" t="n">
+      <c r="H24" s="63" t="n">
         <v>0.286299805636541</v>
       </c>
-      <c r="I24" s="63" t="s">
+      <c r="I24" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J24" s="57"/>
+      <c r="J24" s="58"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="58" t="s">
         <v>171</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="57" t="s">
+      <c r="D25" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="E25" s="59" t="n">
+      <c r="E25" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F25" s="60" t="n">
+      <c r="F25" s="61" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G25" s="61" t="n">
+      <c r="G25" s="62" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="H25" s="62" t="n">
+      <c r="H25" s="63" t="n">
         <v>0.286299805636541</v>
       </c>
-      <c r="I25" s="63" t="s">
+      <c r="I25" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J25" s="57"/>
+      <c r="J25" s="58"/>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
@@ -15388,13 +15399,13 @@
       <c r="E26" s="11" t="n">
         <v>21.2</v>
       </c>
-      <c r="F26" s="53" t="n">
+      <c r="F26" s="54" t="n">
         <v>12.03275</v>
       </c>
-      <c r="G26" s="54" t="n">
+      <c r="G26" s="55" t="n">
         <v>-9.16725</v>
       </c>
-      <c r="H26" s="55" t="n">
+      <c r="H26" s="56" t="n">
         <v>-0.432417452830189</v>
       </c>
       <c r="I26" s="1" t="s">
@@ -15402,34 +15413,34 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="57" t="s">
+      <c r="A27" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B27" s="57" t="s">
+      <c r="B27" s="58" t="s">
         <v>167</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="59" t="s">
         <v>168</v>
       </c>
-      <c r="D27" s="57" t="s">
+      <c r="D27" s="58" t="s">
         <v>345</v>
       </c>
-      <c r="E27" s="59" t="n">
+      <c r="E27" s="60" t="n">
         <v>32.5</v>
       </c>
-      <c r="F27" s="60" t="n">
+      <c r="F27" s="61" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G27" s="61" t="n">
+      <c r="G27" s="62" t="n">
         <v>1.3555</v>
       </c>
-      <c r="H27" s="62" t="n">
+      <c r="H27" s="63" t="n">
         <v>0.0417076923076923</v>
       </c>
-      <c r="I27" s="63" t="s">
+      <c r="I27" s="64" t="s">
         <v>346</v>
       </c>
-      <c r="J27" s="57"/>
+      <c r="J27" s="58"/>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -15447,13 +15458,13 @@
       <c r="E28" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="F28" s="53" t="n">
+      <c r="F28" s="54" t="n">
         <v>33.8555</v>
       </c>
-      <c r="G28" s="54" t="n">
+      <c r="G28" s="55" t="n">
         <v>-11.1445</v>
       </c>
-      <c r="H28" s="55" t="n">
+      <c r="H28" s="56" t="n">
         <v>-0.247655555555556</v>
       </c>
       <c r="I28" s="1" t="s">
@@ -15476,13 +15487,13 @@
       <c r="E29" s="11" t="n">
         <v>30.8</v>
       </c>
-      <c r="F29" s="56" t="n">
+      <c r="F29" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G29" s="54" t="n">
+      <c r="G29" s="55" t="n">
         <v>-17.73</v>
       </c>
-      <c r="H29" s="55" t="n">
+      <c r="H29" s="56" t="n">
         <v>-0.575649350649351</v>
       </c>
       <c r="I29" s="1" t="s">
@@ -15505,13 +15516,13 @@
       <c r="E30" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="F30" s="56" t="n">
+      <c r="F30" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G30" s="54" t="n">
+      <c r="G30" s="55" t="n">
         <v>-14.93</v>
       </c>
-      <c r="H30" s="55" t="n">
+      <c r="H30" s="56" t="n">
         <v>-0.533214285714286</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -15534,13 +15545,13 @@
       <c r="E31" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F31" s="56" t="n">
+      <c r="F31" s="57" t="n">
         <v>16.04</v>
       </c>
-      <c r="G31" s="54" t="n">
+      <c r="G31" s="55" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H31" s="55" t="n">
+      <c r="H31" s="56" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I31" s="1" t="s">
@@ -15563,13 +15574,13 @@
       <c r="E32" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F32" s="56" t="n">
+      <c r="F32" s="57" t="n">
         <v>16.04</v>
       </c>
-      <c r="G32" s="54" t="n">
+      <c r="G32" s="55" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H32" s="55" t="n">
+      <c r="H32" s="56" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I32" s="1" t="s">
@@ -15592,13 +15603,13 @@
       <c r="E33" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F33" s="56" t="n">
+      <c r="F33" s="57" t="n">
         <v>16.04</v>
       </c>
-      <c r="G33" s="54" t="n">
+      <c r="G33" s="55" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H33" s="55" t="n">
+      <c r="H33" s="56" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I33" s="1" t="s">
@@ -15621,13 +15632,13 @@
       <c r="E34" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F34" s="56" t="n">
+      <c r="F34" s="57" t="n">
         <v>16.04</v>
       </c>
-      <c r="G34" s="54" t="n">
+      <c r="G34" s="55" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H34" s="55" t="n">
+      <c r="H34" s="56" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I34" s="1" t="s">
@@ -15650,13 +15661,13 @@
       <c r="E35" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F35" s="56" t="n">
+      <c r="F35" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G35" s="54" t="n">
+      <c r="G35" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H35" s="55" t="n">
+      <c r="H35" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I35" s="1" t="s">
@@ -15679,13 +15690,13 @@
       <c r="E36" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F36" s="56" t="n">
+      <c r="F36" s="57" t="n">
         <v>16.04</v>
       </c>
-      <c r="G36" s="54" t="n">
+      <c r="G36" s="55" t="n">
         <v>-14.96</v>
       </c>
-      <c r="H36" s="55" t="n">
+      <c r="H36" s="56" t="n">
         <v>-0.48258064516129</v>
       </c>
       <c r="I36" s="1" t="s">
@@ -15708,13 +15719,13 @@
       <c r="E37" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F37" s="56" t="n">
+      <c r="F37" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G37" s="54" t="n">
+      <c r="G37" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H37" s="55" t="n">
+      <c r="H37" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I37" s="1" t="s">
@@ -15737,13 +15748,13 @@
       <c r="E38" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F38" s="56" t="n">
+      <c r="F38" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G38" s="54" t="n">
+      <c r="G38" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H38" s="55" t="n">
+      <c r="H38" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I38" s="1" t="s">
@@ -15766,13 +15777,13 @@
       <c r="E39" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F39" s="56" t="n">
+      <c r="F39" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G39" s="54" t="n">
+      <c r="G39" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H39" s="55" t="n">
+      <c r="H39" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I39" s="1" t="s">
@@ -15795,13 +15806,13 @@
       <c r="E40" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F40" s="56" t="n">
+      <c r="F40" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G40" s="54" t="n">
+      <c r="G40" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H40" s="55" t="n">
+      <c r="H40" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I40" s="1" t="s">
@@ -15824,13 +15835,13 @@
       <c r="E41" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="F41" s="56" t="n">
+      <c r="F41" s="57" t="n">
         <v>13.07</v>
       </c>
-      <c r="G41" s="54" t="n">
+      <c r="G41" s="55" t="n">
         <v>-17.93</v>
       </c>
-      <c r="H41" s="55" t="n">
+      <c r="H41" s="56" t="n">
         <v>-0.578387096774194</v>
       </c>
       <c r="I41" s="1" t="s">
@@ -15853,13 +15864,13 @@
       <c r="E42" s="11" t="n">
         <v>20.05</v>
       </c>
-      <c r="F42" s="56" t="n">
+      <c r="F42" s="57" t="n">
         <v>5.35</v>
       </c>
-      <c r="G42" s="54" t="n">
+      <c r="G42" s="55" t="n">
         <v>-14.7</v>
       </c>
-      <c r="H42" s="55" t="n">
+      <c r="H42" s="56" t="n">
         <v>-0.733167082294264</v>
       </c>
       <c r="I42" s="1" t="s">
@@ -15882,13 +15893,13 @@
       <c r="E43" s="11" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F43" s="56" t="n">
+      <c r="F43" s="57" t="n">
         <v>2.67</v>
       </c>
-      <c r="G43" s="54" t="n">
+      <c r="G43" s="55" t="n">
         <v>-6.68454545454545</v>
       </c>
-      <c r="H43" s="55" t="n">
+      <c r="H43" s="56" t="n">
         <v>-0.714577259475219</v>
       </c>
       <c r="I43" s="1" t="s">
@@ -15911,13 +15922,13 @@
       <c r="E44" s="11" t="n">
         <v>23.4090909090909</v>
       </c>
-      <c r="F44" s="56" t="n">
+      <c r="F44" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G44" s="54" t="n">
+      <c r="G44" s="55" t="n">
         <v>-12.7190909090909</v>
       </c>
-      <c r="H44" s="55" t="n">
+      <c r="H44" s="56" t="n">
         <v>-0.543339805825243</v>
       </c>
       <c r="I44" s="1" t="s">
@@ -15940,13 +15951,13 @@
       <c r="E45" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F45" s="56" t="n">
+      <c r="F45" s="57" t="n">
         <v>2.67</v>
       </c>
-      <c r="G45" s="54" t="n">
+      <c r="G45" s="55" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H45" s="55" t="n">
+      <c r="H45" s="56" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I45" s="1" t="s">
@@ -15969,13 +15980,13 @@
       <c r="E46" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F46" s="56" t="n">
+      <c r="F46" s="57" t="n">
         <v>9.5</v>
       </c>
-      <c r="G46" s="54" t="n">
+      <c r="G46" s="55" t="n">
         <v>-12.5</v>
       </c>
-      <c r="H46" s="55" t="n">
+      <c r="H46" s="56" t="n">
         <v>-0.568181818181818</v>
       </c>
       <c r="I46" s="1" t="s">
@@ -15998,13 +16009,13 @@
       <c r="E47" s="11" t="n">
         <v>16.7363636363636</v>
       </c>
-      <c r="F47" s="56" t="n">
+      <c r="F47" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G47" s="54" t="n">
+      <c r="G47" s="55" t="n">
         <v>-6.0463636363636</v>
       </c>
-      <c r="H47" s="55" t="n">
+      <c r="H47" s="56" t="n">
         <v>-0.36127104834329</v>
       </c>
       <c r="I47" s="1" t="s">
@@ -16027,13 +16038,13 @@
       <c r="E48" s="11" t="n">
         <v>20.9090909090909</v>
       </c>
-      <c r="F48" s="56" t="n">
+      <c r="F48" s="57" t="n">
         <v>5.35</v>
       </c>
-      <c r="G48" s="54" t="n">
+      <c r="G48" s="55" t="n">
         <v>-15.5590909090909</v>
       </c>
-      <c r="H48" s="55" t="n">
+      <c r="H48" s="56" t="n">
         <v>-0.744130434782609</v>
       </c>
       <c r="I48" s="1" t="s">
@@ -16056,13 +16067,13 @@
       <c r="E49" s="11" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="F49" s="56" t="n">
+      <c r="F49" s="57" t="n">
         <v>5.35</v>
       </c>
-      <c r="G49" s="54" t="n">
+      <c r="G49" s="55" t="n">
         <v>-4.00454545454545</v>
       </c>
-      <c r="H49" s="55" t="n">
+      <c r="H49" s="56" t="n">
         <v>-0.428085519922254</v>
       </c>
       <c r="I49" s="1" t="s">
@@ -16085,13 +16096,13 @@
       <c r="E50" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="F50" s="56" t="n">
+      <c r="F50" s="57" t="n">
         <v>2.67</v>
       </c>
-      <c r="G50" s="54" t="n">
+      <c r="G50" s="55" t="n">
         <v>-7.83</v>
       </c>
-      <c r="H50" s="55" t="n">
+      <c r="H50" s="56" t="n">
         <v>-0.745714285714286</v>
       </c>
       <c r="I50" s="1" t="s">
@@ -16114,13 +16125,13 @@
       <c r="E51" s="11" t="n">
         <v>26.5</v>
       </c>
-      <c r="F51" s="56" t="n">
+      <c r="F51" s="57" t="n">
         <v>9.5</v>
       </c>
-      <c r="G51" s="54" t="n">
+      <c r="G51" s="55" t="n">
         <v>-17</v>
       </c>
-      <c r="H51" s="55" t="n">
+      <c r="H51" s="56" t="n">
         <v>-0.641509433962264</v>
       </c>
       <c r="I51" s="1" t="s">
@@ -16143,13 +16154,13 @@
       <c r="E52" s="11" t="n">
         <v>7.81818181818182</v>
       </c>
-      <c r="F52" s="56" t="n">
+      <c r="F52" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="G52" s="54" t="n">
+      <c r="G52" s="55" t="n">
         <v>-5.81818181818182</v>
       </c>
-      <c r="H52" s="55" t="n">
+      <c r="H52" s="56" t="n">
         <v>-0.744186046511628</v>
       </c>
       <c r="I52" s="1" t="s">
@@ -16172,13 +16183,13 @@
       <c r="E53" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F53" s="56" t="n">
+      <c r="F53" s="57" t="n">
         <v>2.67</v>
       </c>
-      <c r="G53" s="54" t="n">
+      <c r="G53" s="55" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H53" s="55" t="n">
+      <c r="H53" s="56" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I53" s="1" t="s">
@@ -16201,13 +16212,13 @@
       <c r="E54" s="11" t="n">
         <v>20.9090909090909</v>
       </c>
-      <c r="F54" s="56" t="n">
+      <c r="F54" s="57" t="n">
         <v>4.01</v>
       </c>
-      <c r="G54" s="54" t="n">
+      <c r="G54" s="55" t="n">
         <v>-16.8990909090909</v>
       </c>
-      <c r="H54" s="55" t="n">
+      <c r="H54" s="56" t="n">
         <v>-0.808217391304348</v>
       </c>
       <c r="I54" s="1" t="s">
@@ -16230,13 +16241,13 @@
       <c r="E55" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F55" s="56" t="n">
+      <c r="F55" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G55" s="54" t="n">
+      <c r="G55" s="55" t="n">
         <v>-11.31</v>
       </c>
-      <c r="H55" s="55" t="n">
+      <c r="H55" s="56" t="n">
         <v>-0.514090909090909</v>
       </c>
       <c r="I55" s="1" t="s">
@@ -16259,13 +16270,13 @@
       <c r="E56" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F56" s="56" t="n">
+      <c r="F56" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G56" s="54" t="n">
+      <c r="G56" s="55" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H56" s="55" t="n">
+      <c r="H56" s="56" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I56" s="1" t="s">
@@ -16288,13 +16299,13 @@
       <c r="E57" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="F57" s="56" t="n">
+      <c r="F57" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G57" s="54" t="n">
+      <c r="G57" s="55" t="n">
         <v>-11.31</v>
       </c>
-      <c r="H57" s="55" t="n">
+      <c r="H57" s="56" t="n">
         <v>-0.514090909090909</v>
       </c>
       <c r="I57" s="1" t="s">
@@ -16317,13 +16328,13 @@
       <c r="E58" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="F58" s="56" t="n">
+      <c r="F58" s="57" t="n">
         <v>2.89</v>
       </c>
-      <c r="G58" s="54" t="n">
+      <c r="G58" s="55" t="n">
         <v>-17.11</v>
       </c>
-      <c r="H58" s="55" t="n">
+      <c r="H58" s="56" t="n">
         <v>-0.8555</v>
       </c>
       <c r="I58" s="1" t="s">
@@ -16346,13 +16357,13 @@
       <c r="E59" s="11" t="n">
         <v>37.6363636363636</v>
       </c>
-      <c r="F59" s="56" t="n">
+      <c r="F59" s="57" t="n">
         <v>1.94</v>
       </c>
-      <c r="G59" s="54" t="n">
+      <c r="G59" s="55" t="n">
         <v>-35.6963636363636</v>
       </c>
-      <c r="H59" s="55" t="n">
+      <c r="H59" s="56" t="n">
         <v>-0.948454106280193</v>
       </c>
       <c r="I59" s="1" t="s">
@@ -16375,13 +16386,13 @@
       <c r="E60" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F60" s="56" t="n">
+      <c r="F60" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G60" s="54" t="n">
+      <c r="G60" s="55" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H60" s="55" t="n">
+      <c r="H60" s="56" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I60" s="1" t="s">
@@ -16404,13 +16415,13 @@
       <c r="E61" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F61" s="56" t="n">
+      <c r="F61" s="57" t="n">
         <v>3.201</v>
       </c>
-      <c r="G61" s="54" t="n">
+      <c r="G61" s="55" t="n">
         <v>-17.2535454545455</v>
       </c>
-      <c r="H61" s="55" t="n">
+      <c r="H61" s="56" t="n">
         <v>-0.843506666666667</v>
       </c>
       <c r="I61" s="1" t="s">
@@ -16433,13 +16444,13 @@
       <c r="E62" s="11" t="n">
         <v>20.55</v>
       </c>
-      <c r="F62" s="56" t="n">
+      <c r="F62" s="57" t="n">
         <v>5.35</v>
       </c>
-      <c r="G62" s="54" t="n">
+      <c r="G62" s="55" t="n">
         <v>-15.2</v>
       </c>
-      <c r="H62" s="55" t="n">
+      <c r="H62" s="56" t="n">
         <v>-0.739659367396594</v>
       </c>
       <c r="I62" s="1" t="s">
@@ -16462,13 +16473,13 @@
       <c r="E63" s="11" t="n">
         <v>20.4545454545455</v>
       </c>
-      <c r="F63" s="56" t="n">
+      <c r="F63" s="57" t="n">
         <v>2.67</v>
       </c>
-      <c r="G63" s="54" t="n">
+      <c r="G63" s="55" t="n">
         <v>-17.7845454545455</v>
       </c>
-      <c r="H63" s="55" t="n">
+      <c r="H63" s="56" t="n">
         <v>-0.869466666666667</v>
       </c>
       <c r="I63" s="1" t="s">
@@ -16491,13 +16502,13 @@
       <c r="E64" s="11" t="n">
         <v>27.2727272727273</v>
       </c>
-      <c r="F64" s="56" t="n">
+      <c r="F64" s="57" t="n">
         <v>10.69</v>
       </c>
-      <c r="G64" s="54" t="n">
+      <c r="G64" s="55" t="n">
         <v>-16.5827272727273</v>
       </c>
-      <c r="H64" s="55" t="n">
+      <c r="H64" s="56" t="n">
         <v>-0.608033333333334</v>
       </c>
       <c r="I64" s="1" t="s">
@@ -16505,200 +16516,200 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="64" t="s">
+      <c r="A66" s="65" t="s">
         <v>350</v>
       </c>
-      <c r="B66" s="64"/>
-      <c r="C66" s="64"/>
-      <c r="D66" s="64"/>
-      <c r="E66" s="64"/>
-      <c r="F66" s="64"/>
-      <c r="G66" s="64"/>
-      <c r="H66" s="64"/>
-      <c r="I66" s="64"/>
-      <c r="J66" s="64"/>
+      <c r="B66" s="65"/>
+      <c r="C66" s="65"/>
+      <c r="D66" s="65"/>
+      <c r="E66" s="65"/>
+      <c r="F66" s="65"/>
+      <c r="G66" s="65"/>
+      <c r="H66" s="65"/>
+      <c r="I66" s="65"/>
+      <c r="J66" s="65"/>
     </row>
     <row r="67" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="52" t="s">
+      <c r="A67" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B67" s="52" t="s">
+      <c r="B67" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C67" s="52" t="s">
+      <c r="C67" s="53" t="s">
         <v>351</v>
       </c>
-      <c r="D67" s="52" t="s">
+      <c r="D67" s="53" t="s">
         <v>352</v>
       </c>
-      <c r="E67" s="52" t="s">
+      <c r="E67" s="53" t="s">
         <v>353</v>
       </c>
-      <c r="F67" s="52" t="s">
+      <c r="F67" s="53" t="s">
         <v>354</v>
       </c>
-      <c r="G67" s="52" t="s">
+      <c r="G67" s="53" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="57" t="s">
+      <c r="A68" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="B68" s="58" t="s">
+      <c r="B68" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C68" s="57" t="s">
+      <c r="C68" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="D68" s="59" t="n">
+      <c r="D68" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E68" s="59" t="n">
+      <c r="E68" s="60" t="n">
         <v>16.93275</v>
       </c>
-      <c r="F68" s="61" t="n">
+      <c r="F68" s="62" t="n">
         <v>7.57820454545455</v>
       </c>
-      <c r="G68" s="62" t="n">
+      <c r="G68" s="63" t="n">
         <v>0.447547181967167</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="57" t="s">
+      <c r="A69" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="B69" s="58" t="s">
+      <c r="B69" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="57" t="s">
+      <c r="C69" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="D69" s="59" t="n">
+      <c r="D69" s="60" t="n">
         <v>21.2</v>
       </c>
-      <c r="E69" s="59" t="n">
+      <c r="E69" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F69" s="61" t="n">
+      <c r="F69" s="62" t="n">
         <v>12.6555</v>
       </c>
-      <c r="G69" s="62" t="n">
+      <c r="G69" s="63" t="n">
         <v>0.373809277665372</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="57" t="s">
+      <c r="A70" s="58" t="s">
         <v>159</v>
       </c>
-      <c r="B70" s="58" t="s">
+      <c r="B70" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="57" t="s">
+      <c r="C70" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="D70" s="59" t="n">
+      <c r="D70" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E70" s="59" t="n">
+      <c r="E70" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F70" s="61" t="n">
+      <c r="F70" s="62" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G70" s="62" t="n">
+      <c r="G70" s="63" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="57" t="s">
+      <c r="A71" s="58" t="s">
         <v>171</v>
       </c>
-      <c r="B71" s="58" t="s">
+      <c r="B71" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="C71" s="57" t="s">
+      <c r="C71" s="58" t="s">
         <v>349</v>
       </c>
-      <c r="D71" s="59" t="n">
+      <c r="D71" s="60" t="n">
         <v>9.35454545454545</v>
       </c>
-      <c r="E71" s="59" t="n">
+      <c r="E71" s="60" t="n">
         <v>12.03275</v>
       </c>
-      <c r="F71" s="61" t="n">
+      <c r="F71" s="62" t="n">
         <v>2.67820454545455</v>
       </c>
-      <c r="G71" s="62" t="n">
+      <c r="G71" s="63" t="n">
         <v>0.222576264399622</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="57" t="s">
+      <c r="A72" s="58" t="s">
         <v>79</v>
       </c>
-      <c r="B72" s="58" t="s">
+      <c r="B72" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="C72" s="57" t="s">
+      <c r="C72" s="58" t="s">
         <v>347</v>
       </c>
-      <c r="D72" s="59" t="n">
+      <c r="D72" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E72" s="59" t="n">
+      <c r="E72" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F72" s="61" t="n">
+      <c r="F72" s="62" t="n">
         <v>5.5009545454545</v>
       </c>
-      <c r="G72" s="62" t="n">
+      <c r="G72" s="63" t="n">
         <v>0.162483334922081</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="57" t="s">
+      <c r="A73" s="58" t="s">
         <v>131</v>
       </c>
-      <c r="B73" s="58" t="s">
+      <c r="B73" s="59" t="s">
         <v>132</v>
       </c>
-      <c r="C73" s="57" t="s">
+      <c r="C73" s="58" t="s">
         <v>347</v>
       </c>
-      <c r="D73" s="59" t="n">
+      <c r="D73" s="60" t="n">
         <v>28.3545454545455</v>
       </c>
-      <c r="E73" s="59" t="n">
+      <c r="E73" s="60" t="n">
         <v>30.1455</v>
       </c>
-      <c r="F73" s="61" t="n">
+      <c r="F73" s="62" t="n">
         <v>1.7909545454545</v>
       </c>
-      <c r="G73" s="62" t="n">
+      <c r="G73" s="63" t="n">
         <v>0.0594103446768007</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="57" t="s">
+      <c r="A74" s="58" t="s">
         <v>167</v>
       </c>
-      <c r="B74" s="58" t="s">
+      <c r="B74" s="59" t="s">
         <v>168</v>
       </c>
-      <c r="C74" s="57" t="s">
+      <c r="C74" s="58" t="s">
         <v>345</v>
       </c>
-      <c r="D74" s="59" t="n">
+      <c r="D74" s="60" t="n">
         <v>32.5</v>
       </c>
-      <c r="E74" s="59" t="n">
+      <c r="E74" s="60" t="n">
         <v>33.8555</v>
       </c>
-      <c r="F74" s="61" t="n">
+      <c r="F74" s="62" t="n">
         <v>1.3555</v>
       </c>
-      <c r="G74" s="62" t="n">
+      <c r="G74" s="63" t="n">
         <v>0.0400378077417258</v>
       </c>
     </row>

</xml_diff>